<commit_message>
Update data 5 September 2026 (25 bal), sinkronisasi Supabase Cloud, dan rekap grade induk
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F514"/>
+  <dimension ref="A1:F539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TANGGAL: 21-8 s/d 4-9          HARI: ......................          TAHUN: 2026</t>
+          <t>TANGGAL: 21-8 s/d 5-9          HARI: ......................          TAHUN: 2026</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -10276,27 +10276,27 @@
     </row>
     <row r="490" ht="20.25" customHeight="1">
       <c r="A490" s="5" t="n">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B490" s="5" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C490" s="5" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D490" s="6" t="inlineStr">
         <is>
-          <t>39608</t>
+          <t>940845</t>
         </is>
       </c>
       <c r="E490" s="5" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F490" s="5" t="n"/>
     </row>
     <row r="491" ht="20.25" customHeight="1">
       <c r="A491" s="5" t="n">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B491" s="5" t="n">
         <v>72</v>
@@ -10306,17 +10306,17 @@
       </c>
       <c r="D491" s="6" t="inlineStr">
         <is>
-          <t>39610</t>
+          <t>39608</t>
         </is>
       </c>
       <c r="E491" s="5" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F491" s="5" t="n"/>
     </row>
     <row r="492" ht="20.25" customHeight="1">
       <c r="A492" s="5" t="n">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B492" s="5" t="n">
         <v>72</v>
@@ -10326,207 +10326,207 @@
       </c>
       <c r="D492" s="6" t="inlineStr">
         <is>
-          <t>39607</t>
+          <t>39610</t>
         </is>
       </c>
       <c r="E492" s="5" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F492" s="5" t="n"/>
     </row>
     <row r="493" ht="20.25" customHeight="1">
       <c r="A493" s="5" t="n">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B493" s="5" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C493" s="5" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D493" s="6" t="inlineStr">
         <is>
-          <t>39557</t>
+          <t>39607</t>
         </is>
       </c>
       <c r="E493" s="5" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="F493" s="5" t="n"/>
     </row>
     <row r="494" ht="20.25" customHeight="1">
       <c r="A494" s="5" t="n">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B494" s="5" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C494" s="5" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D494" s="6" t="inlineStr">
         <is>
-          <t>39606</t>
+          <t>39557</t>
         </is>
       </c>
       <c r="E494" s="5" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F494" s="5" t="n"/>
     </row>
     <row r="495" ht="20.25" customHeight="1">
       <c r="A495" s="5" t="n">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B495" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C495" s="5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D495" s="6" t="inlineStr">
         <is>
-          <t>39609</t>
+          <t>39606</t>
         </is>
       </c>
       <c r="E495" s="5" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F495" s="5" t="n"/>
     </row>
     <row r="496" ht="20.25" customHeight="1">
       <c r="A496" s="5" t="n">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B496" s="5" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C496" s="5" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D496" s="6" t="inlineStr">
         <is>
-          <t>39559</t>
+          <t>39609</t>
         </is>
       </c>
       <c r="E496" s="5" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F496" s="5" t="n"/>
     </row>
     <row r="497" ht="20.25" customHeight="1">
       <c r="A497" s="5" t="n">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B497" s="5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C497" s="5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D497" s="6" t="inlineStr">
         <is>
-          <t>39554</t>
+          <t>39559</t>
         </is>
       </c>
       <c r="E497" s="5" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F497" s="5" t="n"/>
     </row>
     <row r="498" ht="20.25" customHeight="1">
       <c r="A498" s="5" t="n">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B498" s="5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C498" s="5" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D498" s="6" t="inlineStr">
         <is>
-          <t>39558</t>
+          <t>39554</t>
         </is>
       </c>
       <c r="E498" s="5" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F498" s="5" t="n"/>
     </row>
     <row r="499" ht="20.25" customHeight="1">
       <c r="A499" s="5" t="n">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B499" s="5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C499" s="5" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D499" s="6" t="inlineStr">
         <is>
-          <t>39555</t>
+          <t>39558</t>
         </is>
       </c>
       <c r="E499" s="5" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F499" s="5" t="n"/>
     </row>
     <row r="500" ht="20.25" customHeight="1">
       <c r="A500" s="5" t="n">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B500" s="5" t="n">
         <v>67</v>
       </c>
       <c r="C500" s="5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D500" s="6" t="inlineStr">
         <is>
-          <t>39556</t>
+          <t>39555</t>
         </is>
       </c>
       <c r="E500" s="5" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F500" s="5" t="n"/>
     </row>
     <row r="501" ht="20.25" customHeight="1">
       <c r="A501" s="5" t="n">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B501" s="5" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C501" s="5" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D501" s="6" t="inlineStr">
         <is>
-          <t>39440</t>
+          <t>39556</t>
         </is>
       </c>
       <c r="E501" s="5" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F501" s="5" t="n"/>
     </row>
     <row r="502" ht="20.25" customHeight="1">
       <c r="A502" s="5" t="n">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B502" s="5" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C502" s="5" t="n">
         <v>65</v>
       </c>
       <c r="D502" s="6" t="inlineStr">
         <is>
-          <t>39439</t>
+          <t>39440</t>
         </is>
       </c>
       <c r="E502" s="5" t="n">
@@ -10536,17 +10536,17 @@
     </row>
     <row r="503" ht="20.25" customHeight="1">
       <c r="A503" s="5" t="n">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B503" s="5" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C503" s="5" t="n">
         <v>65</v>
       </c>
       <c r="D503" s="6" t="inlineStr">
         <is>
-          <t>39441</t>
+          <t>39439</t>
         </is>
       </c>
       <c r="E503" s="5" t="n">
@@ -10556,17 +10556,17 @@
     </row>
     <row r="504" ht="20.25" customHeight="1">
       <c r="A504" s="5" t="n">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B504" s="5" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C504" s="5" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D504" s="6" t="inlineStr">
         <is>
-          <t>39553</t>
+          <t>39441</t>
         </is>
       </c>
       <c r="E504" s="5" t="n">
@@ -10576,7 +10576,7 @@
     </row>
     <row r="505" ht="20.25" customHeight="1">
       <c r="A505" s="5" t="n">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B505" s="5" t="n">
         <v>66</v>
@@ -10586,17 +10586,17 @@
       </c>
       <c r="D505" s="6" t="inlineStr">
         <is>
-          <t>39550</t>
+          <t>39553</t>
         </is>
       </c>
       <c r="E505" s="5" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F505" s="5" t="n"/>
     </row>
     <row r="506" ht="20.25" customHeight="1">
       <c r="A506" s="5" t="n">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B506" s="5" t="n">
         <v>66</v>
@@ -10606,17 +10606,17 @@
       </c>
       <c r="D506" s="6" t="inlineStr">
         <is>
-          <t>39552</t>
+          <t>39550</t>
         </is>
       </c>
       <c r="E506" s="5" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F506" s="5" t="n"/>
     </row>
     <row r="507" ht="20.25" customHeight="1">
       <c r="A507" s="5" t="n">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B507" s="5" t="n">
         <v>66</v>
@@ -10626,17 +10626,17 @@
       </c>
       <c r="D507" s="6" t="inlineStr">
         <is>
-          <t>39551</t>
+          <t>39552</t>
         </is>
       </c>
       <c r="E507" s="5" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F507" s="5" t="n"/>
     </row>
     <row r="508" ht="20.25" customHeight="1">
       <c r="A508" s="5" t="n">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B508" s="5" t="n">
         <v>66</v>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="D508" s="6" t="inlineStr">
         <is>
-          <t>39549</t>
+          <t>39551</t>
         </is>
       </c>
       <c r="E508" s="5" t="n">
@@ -10656,17 +10656,17 @@
     </row>
     <row r="509" ht="20.25" customHeight="1">
       <c r="A509" s="5" t="n">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="B509" s="5" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C509" s="5" t="n">
         <v>66</v>
       </c>
       <c r="D509" s="6" t="inlineStr">
         <is>
-          <t>39167</t>
+          <t>39549</t>
         </is>
       </c>
       <c r="E509" s="5" t="n">
@@ -10676,98 +10676,598 @@
     </row>
     <row r="510" ht="20.25" customHeight="1">
       <c r="A510" s="5" t="n">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B510" s="5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C510" s="5" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D510" s="6" t="inlineStr">
         <is>
-          <t>39166</t>
+          <t>39167</t>
         </is>
       </c>
       <c r="E510" s="5" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F510" s="5" t="n"/>
     </row>
     <row r="511" ht="20.25" customHeight="1">
       <c r="A511" s="5" t="n">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B511" s="5" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C511" s="5" t="n">
         <v>67</v>
       </c>
       <c r="D511" s="6" t="inlineStr">
         <is>
-          <t>39165</t>
+          <t>39166</t>
         </is>
       </c>
       <c r="E511" s="5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F511" s="5" t="n"/>
     </row>
     <row r="512" ht="20.25" customHeight="1">
       <c r="A512" s="5" t="n">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B512" s="5" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C512" s="5" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D512" s="6" t="inlineStr">
         <is>
-          <t>39560</t>
+          <t>39165</t>
         </is>
       </c>
       <c r="E512" s="5" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F512" s="5" t="n"/>
     </row>
     <row r="513" ht="20.25" customHeight="1">
       <c r="A513" s="5" t="n">
+        <v>741</v>
+      </c>
+      <c r="B513" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C513" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D513" s="6" t="inlineStr">
+        <is>
+          <t>39560</t>
+        </is>
+      </c>
+      <c r="E513" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F513" s="5" t="n"/>
+    </row>
+    <row r="514" ht="20.25" customHeight="1">
+      <c r="A514" s="5" t="n">
         <v>743</v>
       </c>
-      <c r="B513" s="5" t="n">
+      <c r="B514" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="C513" s="5" t="n">
+      <c r="C514" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="D513" s="6" t="inlineStr">
+      <c r="D514" s="6" t="inlineStr">
         <is>
           <t>39164</t>
         </is>
       </c>
-      <c r="E513" s="5" t="n">
+      <c r="E514" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="F513" s="5" t="n"/>
-    </row>
-    <row r="514" ht="22" customHeight="1">
-      <c r="A514" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (509 BAL)</t>
-        </is>
-      </c>
-      <c r="B514" s="4" t="n"/>
-      <c r="C514" s="4" t="n"/>
-      <c r="D514" s="4" t="n"/>
-      <c r="E514" s="4">
-        <f>SUM(E5:E513)</f>
+      <c r="F514" s="5" t="n"/>
+    </row>
+    <row r="515" ht="20.25" customHeight="1">
+      <c r="A515" s="5" t="n">
+        <v>747</v>
+      </c>
+      <c r="B515" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C515" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D515" s="6" t="inlineStr">
+        <is>
+          <t>123139</t>
+        </is>
+      </c>
+      <c r="E515" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F515" s="5" t="n"/>
+    </row>
+    <row r="516" ht="20.25" customHeight="1">
+      <c r="A516" s="5" t="n">
+        <v>748</v>
+      </c>
+      <c r="B516" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C516" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D516" s="6" t="inlineStr">
+        <is>
+          <t>123140</t>
+        </is>
+      </c>
+      <c r="E516" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F516" s="5" t="n"/>
+    </row>
+    <row r="517" ht="20.25" customHeight="1">
+      <c r="A517" s="5" t="n">
+        <v>749</v>
+      </c>
+      <c r="B517" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C517" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D517" s="6" t="inlineStr">
+        <is>
+          <t>123301</t>
+        </is>
+      </c>
+      <c r="E517" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F517" s="5" t="n"/>
+    </row>
+    <row r="518" ht="20.25" customHeight="1">
+      <c r="A518" s="5" t="n">
+        <v>751</v>
+      </c>
+      <c r="B518" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C518" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D518" s="6" t="inlineStr">
+        <is>
+          <t>39200</t>
+        </is>
+      </c>
+      <c r="E518" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F518" s="5" t="n"/>
+    </row>
+    <row r="519" ht="20.25" customHeight="1">
+      <c r="A519" s="5" t="n">
+        <v>752</v>
+      </c>
+      <c r="B519" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C519" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D519" s="6" t="inlineStr">
+        <is>
+          <t>39325</t>
+        </is>
+      </c>
+      <c r="E519" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F519" s="5" t="n"/>
+    </row>
+    <row r="520" ht="20.25" customHeight="1">
+      <c r="A520" s="5" t="n">
+        <v>753</v>
+      </c>
+      <c r="B520" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C520" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D520" s="6" t="inlineStr">
+        <is>
+          <t>123302</t>
+        </is>
+      </c>
+      <c r="E520" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F520" s="5" t="n"/>
+    </row>
+    <row r="521" ht="20.25" customHeight="1">
+      <c r="A521" s="5" t="n">
+        <v>755</v>
+      </c>
+      <c r="B521" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C521" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D521" s="6" t="inlineStr">
+        <is>
+          <t>123303</t>
+        </is>
+      </c>
+      <c r="E521" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F521" s="5" t="n"/>
+    </row>
+    <row r="522" ht="20.25" customHeight="1">
+      <c r="A522" s="5" t="n">
+        <v>761</v>
+      </c>
+      <c r="B522" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C522" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D522" s="6" t="inlineStr">
+        <is>
+          <t>123141</t>
+        </is>
+      </c>
+      <c r="E522" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F522" s="5" t="n"/>
+    </row>
+    <row r="523" ht="20.25" customHeight="1">
+      <c r="A523" s="5" t="n">
+        <v>762</v>
+      </c>
+      <c r="B523" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C523" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D523" s="6" t="inlineStr">
+        <is>
+          <t>123143</t>
+        </is>
+      </c>
+      <c r="E523" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F523" s="5" t="n"/>
+    </row>
+    <row r="524" ht="20.25" customHeight="1">
+      <c r="A524" s="5" t="n">
+        <v>763</v>
+      </c>
+      <c r="B524" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C524" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D524" s="6" t="inlineStr">
+        <is>
+          <t>123142</t>
+        </is>
+      </c>
+      <c r="E524" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F524" s="5" t="n"/>
+    </row>
+    <row r="525" ht="20.25" customHeight="1">
+      <c r="A525" s="5" t="n">
+        <v>764</v>
+      </c>
+      <c r="B525" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C525" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D525" s="6" t="inlineStr">
+        <is>
+          <t>123304</t>
+        </is>
+      </c>
+      <c r="E525" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F525" s="5" t="n"/>
+    </row>
+    <row r="526" ht="20.25" customHeight="1">
+      <c r="A526" s="5" t="n">
+        <v>765</v>
+      </c>
+      <c r="B526" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C526" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D526" s="6" t="inlineStr">
+        <is>
+          <t>940842</t>
+        </is>
+      </c>
+      <c r="E526" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F526" s="5" t="n"/>
+    </row>
+    <row r="527" ht="20.25" customHeight="1">
+      <c r="A527" s="5" t="n">
+        <v>766</v>
+      </c>
+      <c r="B527" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C527" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D527" s="6" t="inlineStr">
+        <is>
+          <t>940847</t>
+        </is>
+      </c>
+      <c r="E527" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F527" s="5" t="n"/>
+    </row>
+    <row r="528" ht="20.25" customHeight="1">
+      <c r="A528" s="5" t="n">
+        <v>767</v>
+      </c>
+      <c r="B528" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C528" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D528" s="6" t="inlineStr">
+        <is>
+          <t>940843</t>
+        </is>
+      </c>
+      <c r="E528" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F528" s="5" t="n"/>
+    </row>
+    <row r="529" ht="20.25" customHeight="1">
+      <c r="A529" s="5" t="n">
+        <v>768</v>
+      </c>
+      <c r="B529" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C529" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D529" s="6" t="inlineStr">
+        <is>
+          <t>123144</t>
+        </is>
+      </c>
+      <c r="E529" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F529" s="5" t="n"/>
+    </row>
+    <row r="530" ht="20.25" customHeight="1">
+      <c r="A530" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="B530" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C530" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D530" s="6" t="inlineStr">
+        <is>
+          <t>123305</t>
+        </is>
+      </c>
+      <c r="E530" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F530" s="5" t="n"/>
+    </row>
+    <row r="531" ht="20.25" customHeight="1">
+      <c r="A531" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="B531" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C531" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D531" s="6" t="inlineStr">
+        <is>
+          <t>940844</t>
+        </is>
+      </c>
+      <c r="E531" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F531" s="5" t="n"/>
+    </row>
+    <row r="532" ht="20.25" customHeight="1">
+      <c r="A532" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="B532" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C532" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D532" s="6" t="inlineStr">
+        <is>
+          <t>940848</t>
+        </is>
+      </c>
+      <c r="E532" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F532" s="5" t="n"/>
+    </row>
+    <row r="533" ht="20.25" customHeight="1">
+      <c r="A533" s="5" t="n">
+        <v>772</v>
+      </c>
+      <c r="B533" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C533" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D533" s="6" t="inlineStr">
+        <is>
+          <t>940840</t>
+        </is>
+      </c>
+      <c r="E533" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F533" s="5" t="n"/>
+    </row>
+    <row r="534" ht="20.25" customHeight="1">
+      <c r="A534" s="5" t="n">
+        <v>773</v>
+      </c>
+      <c r="B534" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C534" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D534" s="6" t="inlineStr">
+        <is>
+          <t>940841</t>
+        </is>
+      </c>
+      <c r="E534" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F534" s="5" t="n"/>
+    </row>
+    <row r="535" ht="20.25" customHeight="1">
+      <c r="A535" s="5" t="n">
+        <v>786</v>
+      </c>
+      <c r="B535" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C535" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D535" s="6" t="inlineStr">
+        <is>
+          <t>123307</t>
+        </is>
+      </c>
+      <c r="E535" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F535" s="5" t="n"/>
+    </row>
+    <row r="536" ht="20.25" customHeight="1">
+      <c r="A536" s="5" t="n">
+        <v>787</v>
+      </c>
+      <c r="B536" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C536" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D536" s="6" t="inlineStr">
+        <is>
+          <t>940846</t>
+        </is>
+      </c>
+      <c r="E536" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F536" s="5" t="n"/>
+    </row>
+    <row r="537" ht="20.25" customHeight="1">
+      <c r="A537" s="5" t="n">
+        <v>788</v>
+      </c>
+      <c r="B537" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C537" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D537" s="6" t="inlineStr">
+        <is>
+          <t>123306</t>
+        </is>
+      </c>
+      <c r="E537" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F537" s="5" t="n"/>
+    </row>
+    <row r="538" ht="20.25" customHeight="1">
+      <c r="A538" s="5" t="n">
+        <v>789</v>
+      </c>
+      <c r="B538" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C538" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D538" s="6" t="inlineStr">
+        <is>
+          <t>123145</t>
+        </is>
+      </c>
+      <c r="E538" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F538" s="5" t="n"/>
+    </row>
+    <row r="539" ht="22" customHeight="1">
+      <c r="A539" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (534 BAL)</t>
+        </is>
+      </c>
+      <c r="B539" s="4" t="n"/>
+      <c r="C539" s="4" t="n"/>
+      <c r="D539" s="4" t="n"/>
+      <c r="E539" s="4">
+        <f>SUM(E5:E538)</f>
         <v/>
       </c>
-      <c r="F514" s="4" t="inlineStr">
+      <c r="F539" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -10776,12 +11276,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A514:D514"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A539:D539"/>
     <mergeCell ref="B3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10794,7 +11294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I514"/>
+  <dimension ref="A1:I539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10811,14 +11311,14 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 4 SEPTEMBER 2026)</t>
+          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 5 SEPTEMBER 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 509 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 534 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -28820,34 +29320,34 @@
       </c>
       <c r="B490" s="9" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C490" s="9" t="inlineStr">
         <is>
-          <t>JUMAT</t>
+          <t>SABTU</t>
         </is>
       </c>
       <c r="D490" s="9" t="n">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="E490" s="9" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F490" s="9" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G490" s="10" t="inlineStr">
         <is>
-          <t>39608</t>
+          <t>940845</t>
         </is>
       </c>
       <c r="H490" s="9" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I490" s="11" t="inlineStr">
         <is>
-          <t>grade 4 sep.xlsx</t>
+          <t>grade 5 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -28866,7 +29366,7 @@
         </is>
       </c>
       <c r="D491" s="9" t="n">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E491" s="9" t="n">
         <v>72</v>
@@ -28876,11 +29376,11 @@
       </c>
       <c r="G491" s="10" t="inlineStr">
         <is>
-          <t>39610</t>
+          <t>39608</t>
         </is>
       </c>
       <c r="H491" s="9" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I491" s="11" t="inlineStr">
         <is>
@@ -28903,7 +29403,7 @@
         </is>
       </c>
       <c r="D492" s="9" t="n">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="E492" s="9" t="n">
         <v>72</v>
@@ -28913,11 +29413,11 @@
       </c>
       <c r="G492" s="10" t="inlineStr">
         <is>
-          <t>39607</t>
+          <t>39610</t>
         </is>
       </c>
       <c r="H492" s="9" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="I492" s="11" t="inlineStr">
         <is>
@@ -28940,21 +29440,21 @@
         </is>
       </c>
       <c r="D493" s="9" t="n">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="E493" s="9" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F493" s="9" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G493" s="10" t="inlineStr">
         <is>
-          <t>39557</t>
+          <t>39607</t>
         </is>
       </c>
       <c r="H493" s="9" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="I493" s="11" t="inlineStr">
         <is>
@@ -28977,21 +29477,21 @@
         </is>
       </c>
       <c r="D494" s="9" t="n">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="E494" s="9" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F494" s="9" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G494" s="10" t="inlineStr">
         <is>
-          <t>39606</t>
+          <t>39557</t>
         </is>
       </c>
       <c r="H494" s="9" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I494" s="11" t="inlineStr">
         <is>
@@ -29014,21 +29514,21 @@
         </is>
       </c>
       <c r="D495" s="9" t="n">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="E495" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F495" s="9" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G495" s="10" t="inlineStr">
         <is>
-          <t>39609</t>
+          <t>39606</t>
         </is>
       </c>
       <c r="H495" s="9" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I495" s="11" t="inlineStr">
         <is>
@@ -29051,21 +29551,21 @@
         </is>
       </c>
       <c r="D496" s="9" t="n">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="E496" s="9" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F496" s="9" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G496" s="10" t="inlineStr">
         <is>
-          <t>39559</t>
+          <t>39609</t>
         </is>
       </c>
       <c r="H496" s="9" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I496" s="11" t="inlineStr">
         <is>
@@ -29088,21 +29588,21 @@
         </is>
       </c>
       <c r="D497" s="9" t="n">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="E497" s="9" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F497" s="9" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G497" s="10" t="inlineStr">
         <is>
-          <t>39554</t>
+          <t>39559</t>
         </is>
       </c>
       <c r="H497" s="9" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I497" s="11" t="inlineStr">
         <is>
@@ -29125,21 +29625,21 @@
         </is>
       </c>
       <c r="D498" s="9" t="n">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E498" s="9" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F498" s="9" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G498" s="10" t="inlineStr">
         <is>
-          <t>39558</t>
+          <t>39554</t>
         </is>
       </c>
       <c r="H498" s="9" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="I498" s="11" t="inlineStr">
         <is>
@@ -29162,21 +29662,21 @@
         </is>
       </c>
       <c r="D499" s="9" t="n">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E499" s="9" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F499" s="9" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="G499" s="10" t="inlineStr">
         <is>
-          <t>39555</t>
+          <t>39558</t>
         </is>
       </c>
       <c r="H499" s="9" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I499" s="11" t="inlineStr">
         <is>
@@ -29199,21 +29699,21 @@
         </is>
       </c>
       <c r="D500" s="9" t="n">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E500" s="9" t="n">
         <v>67</v>
       </c>
       <c r="F500" s="9" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G500" s="10" t="inlineStr">
         <is>
-          <t>39556</t>
+          <t>39555</t>
         </is>
       </c>
       <c r="H500" s="9" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I500" s="11" t="inlineStr">
         <is>
@@ -29236,21 +29736,21 @@
         </is>
       </c>
       <c r="D501" s="9" t="n">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="E501" s="9" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F501" s="9" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G501" s="10" t="inlineStr">
         <is>
-          <t>39440</t>
+          <t>39556</t>
         </is>
       </c>
       <c r="H501" s="9" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I501" s="11" t="inlineStr">
         <is>
@@ -29273,17 +29773,17 @@
         </is>
       </c>
       <c r="D502" s="9" t="n">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E502" s="9" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F502" s="9" t="n">
         <v>65</v>
       </c>
       <c r="G502" s="10" t="inlineStr">
         <is>
-          <t>39439</t>
+          <t>39440</t>
         </is>
       </c>
       <c r="H502" s="9" t="n">
@@ -29310,17 +29810,17 @@
         </is>
       </c>
       <c r="D503" s="9" t="n">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="E503" s="9" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F503" s="9" t="n">
         <v>65</v>
       </c>
       <c r="G503" s="10" t="inlineStr">
         <is>
-          <t>39441</t>
+          <t>39439</t>
         </is>
       </c>
       <c r="H503" s="9" t="n">
@@ -29347,17 +29847,17 @@
         </is>
       </c>
       <c r="D504" s="9" t="n">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E504" s="9" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F504" s="9" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G504" s="10" t="inlineStr">
         <is>
-          <t>39553</t>
+          <t>39441</t>
         </is>
       </c>
       <c r="H504" s="9" t="n">
@@ -29384,7 +29884,7 @@
         </is>
       </c>
       <c r="D505" s="9" t="n">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E505" s="9" t="n">
         <v>66</v>
@@ -29394,11 +29894,11 @@
       </c>
       <c r="G505" s="10" t="inlineStr">
         <is>
-          <t>39550</t>
+          <t>39553</t>
         </is>
       </c>
       <c r="H505" s="9" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I505" s="11" t="inlineStr">
         <is>
@@ -29421,7 +29921,7 @@
         </is>
       </c>
       <c r="D506" s="9" t="n">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E506" s="9" t="n">
         <v>66</v>
@@ -29431,11 +29931,11 @@
       </c>
       <c r="G506" s="10" t="inlineStr">
         <is>
-          <t>39552</t>
+          <t>39550</t>
         </is>
       </c>
       <c r="H506" s="9" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I506" s="11" t="inlineStr">
         <is>
@@ -29458,7 +29958,7 @@
         </is>
       </c>
       <c r="D507" s="9" t="n">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E507" s="9" t="n">
         <v>66</v>
@@ -29468,11 +29968,11 @@
       </c>
       <c r="G507" s="10" t="inlineStr">
         <is>
-          <t>39551</t>
+          <t>39552</t>
         </is>
       </c>
       <c r="H507" s="9" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I507" s="11" t="inlineStr">
         <is>
@@ -29495,7 +29995,7 @@
         </is>
       </c>
       <c r="D508" s="9" t="n">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="E508" s="9" t="n">
         <v>66</v>
@@ -29505,7 +30005,7 @@
       </c>
       <c r="G508" s="10" t="inlineStr">
         <is>
-          <t>39549</t>
+          <t>39551</t>
         </is>
       </c>
       <c r="H508" s="9" t="n">
@@ -29532,17 +30032,17 @@
         </is>
       </c>
       <c r="D509" s="9" t="n">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="E509" s="9" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F509" s="9" t="n">
         <v>66</v>
       </c>
       <c r="G509" s="10" t="inlineStr">
         <is>
-          <t>39167</t>
+          <t>39549</t>
         </is>
       </c>
       <c r="H509" s="9" t="n">
@@ -29569,21 +30069,21 @@
         </is>
       </c>
       <c r="D510" s="9" t="n">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="E510" s="9" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F510" s="9" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G510" s="10" t="inlineStr">
         <is>
-          <t>39166</t>
+          <t>39167</t>
         </is>
       </c>
       <c r="H510" s="9" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I510" s="11" t="inlineStr">
         <is>
@@ -29606,21 +30106,21 @@
         </is>
       </c>
       <c r="D511" s="9" t="n">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="E511" s="9" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F511" s="9" t="n">
         <v>67</v>
       </c>
       <c r="G511" s="10" t="inlineStr">
         <is>
-          <t>39165</t>
+          <t>39166</t>
         </is>
       </c>
       <c r="H511" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I511" s="11" t="inlineStr">
         <is>
@@ -29643,21 +30143,21 @@
         </is>
       </c>
       <c r="D512" s="9" t="n">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="E512" s="9" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F512" s="9" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G512" s="10" t="inlineStr">
         <is>
-          <t>39560</t>
+          <t>39165</t>
         </is>
       </c>
       <c r="H512" s="9" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I512" s="11" t="inlineStr">
         <is>
@@ -29680,45 +30180,970 @@
         </is>
       </c>
       <c r="D513" s="9" t="n">
+        <v>741</v>
+      </c>
+      <c r="E513" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="F513" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G513" s="10" t="inlineStr">
+        <is>
+          <t>39560</t>
+        </is>
+      </c>
+      <c r="H513" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I513" s="11" t="inlineStr">
+        <is>
+          <t>grade 4 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="514" ht="20" customHeight="1">
+      <c r="A514" s="9" t="n">
+        <v>510</v>
+      </c>
+      <c r="B514" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C514" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D514" s="9" t="n">
         <v>743</v>
       </c>
-      <c r="E513" s="9" t="n">
+      <c r="E514" s="9" t="n">
         <v>67</v>
       </c>
-      <c r="F513" s="9" t="n">
+      <c r="F514" s="9" t="n">
         <v>66</v>
       </c>
-      <c r="G513" s="10" t="inlineStr">
+      <c r="G514" s="10" t="inlineStr">
         <is>
           <t>39164</t>
         </is>
       </c>
-      <c r="H513" s="9" t="n">
+      <c r="H514" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="I513" s="11" t="inlineStr">
+      <c r="I514" s="11" t="inlineStr">
         <is>
           <t>grade 4 sep.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="514">
-      <c r="A514" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (509 BAL)</t>
-        </is>
-      </c>
-      <c r="B514" s="4" t="n"/>
-      <c r="C514" s="4" t="n"/>
-      <c r="D514" s="4" t="n"/>
-      <c r="E514" s="4" t="n"/>
-      <c r="F514" s="4" t="n"/>
-      <c r="G514" s="4" t="n"/>
-      <c r="H514" s="4">
-        <f>SUM(H5:H513)</f>
+    <row r="515" ht="20" customHeight="1">
+      <c r="A515" s="9" t="n">
+        <v>511</v>
+      </c>
+      <c r="B515" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C515" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D515" s="9" t="n">
+        <v>747</v>
+      </c>
+      <c r="E515" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F515" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G515" s="10" t="inlineStr">
+        <is>
+          <t>123139</t>
+        </is>
+      </c>
+      <c r="H515" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I515" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="516" ht="20" customHeight="1">
+      <c r="A516" s="9" t="n">
+        <v>512</v>
+      </c>
+      <c r="B516" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C516" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D516" s="9" t="n">
+        <v>748</v>
+      </c>
+      <c r="E516" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F516" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G516" s="10" t="inlineStr">
+        <is>
+          <t>123140</t>
+        </is>
+      </c>
+      <c r="H516" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I516" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="517" ht="20" customHeight="1">
+      <c r="A517" s="9" t="n">
+        <v>513</v>
+      </c>
+      <c r="B517" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C517" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D517" s="9" t="n">
+        <v>749</v>
+      </c>
+      <c r="E517" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F517" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G517" s="10" t="inlineStr">
+        <is>
+          <t>123301</t>
+        </is>
+      </c>
+      <c r="H517" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I517" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="518" ht="20" customHeight="1">
+      <c r="A518" s="9" t="n">
+        <v>514</v>
+      </c>
+      <c r="B518" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C518" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D518" s="9" t="n">
+        <v>751</v>
+      </c>
+      <c r="E518" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F518" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G518" s="10" t="inlineStr">
+        <is>
+          <t>39200</t>
+        </is>
+      </c>
+      <c r="H518" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I518" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="519" ht="20" customHeight="1">
+      <c r="A519" s="9" t="n">
+        <v>515</v>
+      </c>
+      <c r="B519" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C519" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D519" s="9" t="n">
+        <v>752</v>
+      </c>
+      <c r="E519" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F519" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G519" s="10" t="inlineStr">
+        <is>
+          <t>39325</t>
+        </is>
+      </c>
+      <c r="H519" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I519" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="520" ht="20" customHeight="1">
+      <c r="A520" s="9" t="n">
+        <v>516</v>
+      </c>
+      <c r="B520" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C520" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D520" s="9" t="n">
+        <v>753</v>
+      </c>
+      <c r="E520" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F520" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G520" s="10" t="inlineStr">
+        <is>
+          <t>123302</t>
+        </is>
+      </c>
+      <c r="H520" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I520" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="521" ht="20" customHeight="1">
+      <c r="A521" s="9" t="n">
+        <v>517</v>
+      </c>
+      <c r="B521" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C521" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D521" s="9" t="n">
+        <v>755</v>
+      </c>
+      <c r="E521" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F521" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G521" s="10" t="inlineStr">
+        <is>
+          <t>123303</t>
+        </is>
+      </c>
+      <c r="H521" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I521" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="522" ht="20" customHeight="1">
+      <c r="A522" s="9" t="n">
+        <v>518</v>
+      </c>
+      <c r="B522" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C522" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D522" s="9" t="n">
+        <v>761</v>
+      </c>
+      <c r="E522" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F522" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G522" s="10" t="inlineStr">
+        <is>
+          <t>123141</t>
+        </is>
+      </c>
+      <c r="H522" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I522" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="523" ht="20" customHeight="1">
+      <c r="A523" s="9" t="n">
+        <v>519</v>
+      </c>
+      <c r="B523" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C523" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D523" s="9" t="n">
+        <v>762</v>
+      </c>
+      <c r="E523" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F523" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G523" s="10" t="inlineStr">
+        <is>
+          <t>123143</t>
+        </is>
+      </c>
+      <c r="H523" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I523" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="524" ht="20" customHeight="1">
+      <c r="A524" s="9" t="n">
+        <v>520</v>
+      </c>
+      <c r="B524" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C524" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D524" s="9" t="n">
+        <v>763</v>
+      </c>
+      <c r="E524" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F524" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G524" s="10" t="inlineStr">
+        <is>
+          <t>123142</t>
+        </is>
+      </c>
+      <c r="H524" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I524" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="525" ht="20" customHeight="1">
+      <c r="A525" s="9" t="n">
+        <v>521</v>
+      </c>
+      <c r="B525" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C525" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D525" s="9" t="n">
+        <v>764</v>
+      </c>
+      <c r="E525" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F525" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G525" s="10" t="inlineStr">
+        <is>
+          <t>123304</t>
+        </is>
+      </c>
+      <c r="H525" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I525" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="526" ht="20" customHeight="1">
+      <c r="A526" s="9" t="n">
+        <v>522</v>
+      </c>
+      <c r="B526" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C526" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D526" s="9" t="n">
+        <v>765</v>
+      </c>
+      <c r="E526" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F526" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G526" s="10" t="inlineStr">
+        <is>
+          <t>940842</t>
+        </is>
+      </c>
+      <c r="H526" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I526" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="527" ht="20" customHeight="1">
+      <c r="A527" s="9" t="n">
+        <v>523</v>
+      </c>
+      <c r="B527" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C527" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D527" s="9" t="n">
+        <v>766</v>
+      </c>
+      <c r="E527" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F527" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G527" s="10" t="inlineStr">
+        <is>
+          <t>940847</t>
+        </is>
+      </c>
+      <c r="H527" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I527" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="528" ht="20" customHeight="1">
+      <c r="A528" s="9" t="n">
+        <v>524</v>
+      </c>
+      <c r="B528" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C528" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D528" s="9" t="n">
+        <v>767</v>
+      </c>
+      <c r="E528" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F528" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G528" s="10" t="inlineStr">
+        <is>
+          <t>940843</t>
+        </is>
+      </c>
+      <c r="H528" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I528" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="529" ht="20" customHeight="1">
+      <c r="A529" s="9" t="n">
+        <v>525</v>
+      </c>
+      <c r="B529" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C529" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D529" s="9" t="n">
+        <v>768</v>
+      </c>
+      <c r="E529" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F529" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G529" s="10" t="inlineStr">
+        <is>
+          <t>123144</t>
+        </is>
+      </c>
+      <c r="H529" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I529" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="530" ht="20" customHeight="1">
+      <c r="A530" s="9" t="n">
+        <v>526</v>
+      </c>
+      <c r="B530" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C530" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D530" s="9" t="n">
+        <v>769</v>
+      </c>
+      <c r="E530" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F530" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G530" s="10" t="inlineStr">
+        <is>
+          <t>123305</t>
+        </is>
+      </c>
+      <c r="H530" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I530" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="531" ht="20" customHeight="1">
+      <c r="A531" s="9" t="n">
+        <v>527</v>
+      </c>
+      <c r="B531" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C531" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D531" s="9" t="n">
+        <v>770</v>
+      </c>
+      <c r="E531" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F531" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G531" s="10" t="inlineStr">
+        <is>
+          <t>940844</t>
+        </is>
+      </c>
+      <c r="H531" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I531" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="532" ht="20" customHeight="1">
+      <c r="A532" s="9" t="n">
+        <v>528</v>
+      </c>
+      <c r="B532" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C532" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D532" s="9" t="n">
+        <v>771</v>
+      </c>
+      <c r="E532" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F532" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G532" s="10" t="inlineStr">
+        <is>
+          <t>940848</t>
+        </is>
+      </c>
+      <c r="H532" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I532" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="533" ht="20" customHeight="1">
+      <c r="A533" s="9" t="n">
+        <v>529</v>
+      </c>
+      <c r="B533" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C533" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D533" s="9" t="n">
+        <v>772</v>
+      </c>
+      <c r="E533" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F533" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G533" s="10" t="inlineStr">
+        <is>
+          <t>940840</t>
+        </is>
+      </c>
+      <c r="H533" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I533" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="534" ht="20" customHeight="1">
+      <c r="A534" s="9" t="n">
+        <v>530</v>
+      </c>
+      <c r="B534" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C534" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D534" s="9" t="n">
+        <v>773</v>
+      </c>
+      <c r="E534" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F534" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G534" s="10" t="inlineStr">
+        <is>
+          <t>940841</t>
+        </is>
+      </c>
+      <c r="H534" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I534" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="535" ht="20" customHeight="1">
+      <c r="A535" s="9" t="n">
+        <v>531</v>
+      </c>
+      <c r="B535" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C535" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D535" s="9" t="n">
+        <v>786</v>
+      </c>
+      <c r="E535" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F535" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G535" s="10" t="inlineStr">
+        <is>
+          <t>123307</t>
+        </is>
+      </c>
+      <c r="H535" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I535" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="536" ht="20" customHeight="1">
+      <c r="A536" s="9" t="n">
+        <v>532</v>
+      </c>
+      <c r="B536" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C536" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D536" s="9" t="n">
+        <v>787</v>
+      </c>
+      <c r="E536" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F536" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G536" s="10" t="inlineStr">
+        <is>
+          <t>940846</t>
+        </is>
+      </c>
+      <c r="H536" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I536" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="537" ht="20" customHeight="1">
+      <c r="A537" s="9" t="n">
+        <v>533</v>
+      </c>
+      <c r="B537" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C537" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D537" s="9" t="n">
+        <v>788</v>
+      </c>
+      <c r="E537" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F537" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G537" s="10" t="inlineStr">
+        <is>
+          <t>123306</t>
+        </is>
+      </c>
+      <c r="H537" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I537" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="538" ht="20" customHeight="1">
+      <c r="A538" s="9" t="n">
+        <v>534</v>
+      </c>
+      <c r="B538" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C538" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D538" s="9" t="n">
+        <v>789</v>
+      </c>
+      <c r="E538" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F538" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G538" s="10" t="inlineStr">
+        <is>
+          <t>123145</t>
+        </is>
+      </c>
+      <c r="H538" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I538" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (534 BAL)</t>
+        </is>
+      </c>
+      <c r="B539" s="4" t="n"/>
+      <c r="C539" s="4" t="n"/>
+      <c r="D539" s="4" t="n"/>
+      <c r="E539" s="4" t="n"/>
+      <c r="F539" s="4" t="n"/>
+      <c r="G539" s="4" t="n"/>
+      <c r="H539" s="4">
+        <f>SUM(H5:H538)</f>
         <v/>
       </c>
-      <c r="I514" s="4" t="inlineStr">
+      <c r="I539" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -29727,7 +31152,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A514:G514"/>
+    <mergeCell ref="A539:G539"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -29740,7 +31165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -29762,7 +31187,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Periode: 21 Agustus 2026 s/d 4 September 2026</t>
+          <t>Periode: 21 Agustus 2026 s/d 5 September 2026</t>
         </is>
       </c>
     </row>
@@ -30209,36 +31634,65 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>981</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>39.24</v>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>715 - 789</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4">
-        <f>SUM(D5:D18)</f>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4">
+        <f>SUM(D5:D19)</f>
         <v/>
       </c>
-      <c r="E19" s="4">
-        <f>SUM(E5:E18)</f>
+      <c r="E20" s="4">
+        <f>SUM(E5:E19)</f>
         <v/>
       </c>
-      <c r="F19" s="4">
-        <f>AVERAGE(F5:F18)</f>
+      <c r="F20" s="4">
+        <f>AVERAGE(F5:F19)</f>
         <v/>
       </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>3 - 743</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>3 - 789</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A20:C20"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update data 6 September 2026 (23 bal), sinkronisasi Supabase Cloud, dan rekap grade induk
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F539"/>
+  <dimension ref="A1:F562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TANGGAL: 21-8 s/d 5-9          HARI: ......................          TAHUN: 2026</t>
+          <t>TANGGAL: 21-8 s/d 6-9          HARI: ......................          TAHUN: 2026</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -10916,187 +10916,187 @@
     </row>
     <row r="522" ht="20.25" customHeight="1">
       <c r="A522" s="5" t="n">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="B522" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C522" s="5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D522" s="6" t="inlineStr">
         <is>
-          <t>123141</t>
+          <t>123592</t>
         </is>
       </c>
       <c r="E522" s="5" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F522" s="5" t="n"/>
     </row>
     <row r="523" ht="20.25" customHeight="1">
       <c r="A523" s="5" t="n">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="B523" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C523" s="5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D523" s="6" t="inlineStr">
         <is>
-          <t>123143</t>
+          <t>123596</t>
         </is>
       </c>
       <c r="E523" s="5" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F523" s="5" t="n"/>
     </row>
     <row r="524" ht="20.25" customHeight="1">
       <c r="A524" s="5" t="n">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="B524" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C524" s="5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D524" s="6" t="inlineStr">
         <is>
-          <t>123142</t>
+          <t>123595</t>
         </is>
       </c>
       <c r="E524" s="5" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F524" s="5" t="n"/>
     </row>
     <row r="525" ht="20.25" customHeight="1">
       <c r="A525" s="5" t="n">
-        <v>764</v>
+        <v>759</v>
       </c>
       <c r="B525" s="5" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C525" s="5" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D525" s="6" t="inlineStr">
         <is>
-          <t>123304</t>
+          <t>123593</t>
         </is>
       </c>
       <c r="E525" s="5" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F525" s="5" t="n"/>
     </row>
     <row r="526" ht="20.25" customHeight="1">
       <c r="A526" s="5" t="n">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="B526" s="5" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C526" s="5" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D526" s="6" t="inlineStr">
         <is>
-          <t>940842</t>
+          <t>123594</t>
         </is>
       </c>
       <c r="E526" s="5" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="F526" s="5" t="n"/>
     </row>
     <row r="527" ht="20.25" customHeight="1">
       <c r="A527" s="5" t="n">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="B527" s="5" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C527" s="5" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="D527" s="6" t="inlineStr">
         <is>
-          <t>940847</t>
+          <t>123141</t>
         </is>
       </c>
       <c r="E527" s="5" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F527" s="5" t="n"/>
     </row>
     <row r="528" ht="20.25" customHeight="1">
       <c r="A528" s="5" t="n">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="B528" s="5" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="C528" s="5" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="D528" s="6" t="inlineStr">
         <is>
-          <t>940843</t>
+          <t>123143</t>
         </is>
       </c>
       <c r="E528" s="5" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="F528" s="5" t="n"/>
     </row>
     <row r="529" ht="20.25" customHeight="1">
       <c r="A529" s="5" t="n">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="B529" s="5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C529" s="5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D529" s="6" t="inlineStr">
         <is>
-          <t>123144</t>
+          <t>123142</t>
         </is>
       </c>
       <c r="E529" s="5" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F529" s="5" t="n"/>
     </row>
     <row r="530" ht="20.25" customHeight="1">
       <c r="A530" s="5" t="n">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="B530" s="5" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C530" s="5" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D530" s="6" t="inlineStr">
         <is>
-          <t>123305</t>
+          <t>123304</t>
         </is>
       </c>
       <c r="E530" s="5" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="F530" s="5" t="n"/>
     </row>
     <row r="531" ht="20.25" customHeight="1">
       <c r="A531" s="5" t="n">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="B531" s="5" t="n">
         <v>66</v>
@@ -11106,17 +11106,17 @@
       </c>
       <c r="D531" s="6" t="inlineStr">
         <is>
-          <t>940844</t>
+          <t>940842</t>
         </is>
       </c>
       <c r="E531" s="5" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F531" s="5" t="n"/>
     </row>
     <row r="532" ht="20.25" customHeight="1">
       <c r="A532" s="5" t="n">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="B532" s="5" t="n">
         <v>62</v>
@@ -11126,27 +11126,27 @@
       </c>
       <c r="D532" s="6" t="inlineStr">
         <is>
-          <t>940848</t>
+          <t>940847</t>
         </is>
       </c>
       <c r="E532" s="5" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F532" s="5" t="n"/>
     </row>
     <row r="533" ht="20.25" customHeight="1">
       <c r="A533" s="5" t="n">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="B533" s="5" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C533" s="5" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D533" s="6" t="inlineStr">
         <is>
-          <t>940840</t>
+          <t>940843</t>
         </is>
       </c>
       <c r="E533" s="5" t="n">
@@ -11156,118 +11156,578 @@
     </row>
     <row r="534" ht="20.25" customHeight="1">
       <c r="A534" s="5" t="n">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="B534" s="5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C534" s="5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D534" s="6" t="inlineStr">
         <is>
-          <t>940841</t>
+          <t>123144</t>
         </is>
       </c>
       <c r="E534" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F534" s="5" t="n"/>
     </row>
     <row r="535" ht="20.25" customHeight="1">
       <c r="A535" s="5" t="n">
-        <v>786</v>
+        <v>769</v>
       </c>
       <c r="B535" s="5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C535" s="5" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D535" s="6" t="inlineStr">
         <is>
-          <t>123307</t>
+          <t>123305</t>
         </is>
       </c>
       <c r="E535" s="5" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F535" s="5" t="n"/>
     </row>
     <row r="536" ht="20.25" customHeight="1">
       <c r="A536" s="5" t="n">
-        <v>787</v>
+        <v>770</v>
       </c>
       <c r="B536" s="5" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C536" s="5" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D536" s="6" t="inlineStr">
         <is>
-          <t>940846</t>
+          <t>940844</t>
         </is>
       </c>
       <c r="E536" s="5" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="F536" s="5" t="n"/>
     </row>
     <row r="537" ht="20.25" customHeight="1">
       <c r="A537" s="5" t="n">
-        <v>788</v>
+        <v>771</v>
       </c>
       <c r="B537" s="5" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C537" s="5" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D537" s="6" t="inlineStr">
         <is>
-          <t>123306</t>
+          <t>940848</t>
         </is>
       </c>
       <c r="E537" s="5" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F537" s="5" t="n"/>
     </row>
     <row r="538" ht="20.25" customHeight="1">
       <c r="A538" s="5" t="n">
+        <v>772</v>
+      </c>
+      <c r="B538" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C538" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D538" s="6" t="inlineStr">
+        <is>
+          <t>940840</t>
+        </is>
+      </c>
+      <c r="E538" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F538" s="5" t="n"/>
+    </row>
+    <row r="539" ht="20.25" customHeight="1">
+      <c r="A539" s="5" t="n">
+        <v>773</v>
+      </c>
+      <c r="B539" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C539" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D539" s="6" t="inlineStr">
+        <is>
+          <t>940841</t>
+        </is>
+      </c>
+      <c r="E539" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F539" s="5" t="n"/>
+    </row>
+    <row r="540" ht="20.25" customHeight="1">
+      <c r="A540" s="5" t="n">
+        <v>786</v>
+      </c>
+      <c r="B540" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C540" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D540" s="6" t="inlineStr">
+        <is>
+          <t>123307</t>
+        </is>
+      </c>
+      <c r="E540" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F540" s="5" t="n"/>
+    </row>
+    <row r="541" ht="20.25" customHeight="1">
+      <c r="A541" s="5" t="n">
+        <v>787</v>
+      </c>
+      <c r="B541" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C541" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D541" s="6" t="inlineStr">
+        <is>
+          <t>940846</t>
+        </is>
+      </c>
+      <c r="E541" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F541" s="5" t="n"/>
+    </row>
+    <row r="542" ht="20.25" customHeight="1">
+      <c r="A542" s="5" t="n">
+        <v>788</v>
+      </c>
+      <c r="B542" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C542" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D542" s="6" t="inlineStr">
+        <is>
+          <t>123306</t>
+        </is>
+      </c>
+      <c r="E542" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F542" s="5" t="n"/>
+    </row>
+    <row r="543" ht="20.25" customHeight="1">
+      <c r="A543" s="5" t="n">
         <v>789</v>
       </c>
-      <c r="B538" s="5" t="n">
+      <c r="B543" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="C538" s="5" t="n">
+      <c r="C543" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="D538" s="6" t="inlineStr">
+      <c r="D543" s="6" t="inlineStr">
         <is>
           <t>123145</t>
         </is>
       </c>
-      <c r="E538" s="5" t="n">
+      <c r="E543" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="F538" s="5" t="n"/>
-    </row>
-    <row r="539" ht="22" customHeight="1">
-      <c r="A539" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (534 BAL)</t>
-        </is>
-      </c>
-      <c r="B539" s="4" t="n"/>
-      <c r="C539" s="4" t="n"/>
-      <c r="D539" s="4" t="n"/>
-      <c r="E539" s="4">
-        <f>SUM(E5:E538)</f>
+      <c r="F543" s="5" t="n"/>
+    </row>
+    <row r="544" ht="20.25" customHeight="1">
+      <c r="A544" s="5" t="n">
+        <v>790</v>
+      </c>
+      <c r="B544" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C544" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D544" s="6" t="inlineStr">
+        <is>
+          <t>123420</t>
+        </is>
+      </c>
+      <c r="E544" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F544" s="5" t="n"/>
+    </row>
+    <row r="545" ht="20.25" customHeight="1">
+      <c r="A545" s="5" t="n">
+        <v>791</v>
+      </c>
+      <c r="B545" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C545" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D545" s="6" t="inlineStr">
+        <is>
+          <t>123423</t>
+        </is>
+      </c>
+      <c r="E545" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F545" s="5" t="n"/>
+    </row>
+    <row r="546" ht="20.25" customHeight="1">
+      <c r="A546" s="5" t="n">
+        <v>792</v>
+      </c>
+      <c r="B546" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C546" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D546" s="6" t="inlineStr">
+        <is>
+          <t>123422</t>
+        </is>
+      </c>
+      <c r="E546" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F546" s="5" t="n"/>
+    </row>
+    <row r="547" ht="20.25" customHeight="1">
+      <c r="A547" s="5" t="n">
+        <v>793</v>
+      </c>
+      <c r="B547" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C547" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D547" s="6" t="inlineStr">
+        <is>
+          <t>123421</t>
+        </is>
+      </c>
+      <c r="E547" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F547" s="5" t="n"/>
+    </row>
+    <row r="548" ht="20.25" customHeight="1">
+      <c r="A548" s="5" t="n">
+        <v>794</v>
+      </c>
+      <c r="B548" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C548" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D548" s="6" t="inlineStr">
+        <is>
+          <t>39352</t>
+        </is>
+      </c>
+      <c r="E548" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F548" s="5" t="n"/>
+    </row>
+    <row r="549" ht="20.25" customHeight="1">
+      <c r="A549" s="5" t="n">
+        <v>795</v>
+      </c>
+      <c r="B549" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C549" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D549" s="6" t="inlineStr">
+        <is>
+          <t>39351</t>
+        </is>
+      </c>
+      <c r="E549" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F549" s="5" t="n"/>
+    </row>
+    <row r="550" ht="20.25" customHeight="1">
+      <c r="A550" s="5" t="n">
+        <v>796</v>
+      </c>
+      <c r="B550" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C550" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D550" s="6" t="inlineStr">
+        <is>
+          <t>123367</t>
+        </is>
+      </c>
+      <c r="E550" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F550" s="5" t="n"/>
+    </row>
+    <row r="551" ht="20.25" customHeight="1">
+      <c r="A551" s="5" t="n">
+        <v>797</v>
+      </c>
+      <c r="B551" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C551" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D551" s="6" t="inlineStr">
+        <is>
+          <t>123368</t>
+        </is>
+      </c>
+      <c r="E551" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F551" s="5" t="n"/>
+    </row>
+    <row r="552" ht="20.25" customHeight="1">
+      <c r="A552" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="B552" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C552" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D552" s="6" t="inlineStr">
+        <is>
+          <t>123591</t>
+        </is>
+      </c>
+      <c r="E552" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F552" s="5" t="n"/>
+    </row>
+    <row r="553" ht="20.25" customHeight="1">
+      <c r="A553" s="5" t="n">
+        <v>799</v>
+      </c>
+      <c r="B553" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C553" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D553" s="6" t="inlineStr">
+        <is>
+          <t>123605</t>
+        </is>
+      </c>
+      <c r="E553" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F553" s="5" t="n"/>
+    </row>
+    <row r="554" ht="20.25" customHeight="1">
+      <c r="A554" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="B554" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C554" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D554" s="6" t="inlineStr">
+        <is>
+          <t>39350</t>
+        </is>
+      </c>
+      <c r="E554" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F554" s="5" t="n"/>
+    </row>
+    <row r="555" ht="20.25" customHeight="1">
+      <c r="A555" s="5" t="n">
+        <v>801</v>
+      </c>
+      <c r="B555" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C555" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D555" s="6" t="inlineStr">
+        <is>
+          <t>123366</t>
+        </is>
+      </c>
+      <c r="E555" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F555" s="5" t="n"/>
+    </row>
+    <row r="556" ht="20.25" customHeight="1">
+      <c r="A556" s="5" t="n">
+        <v>802</v>
+      </c>
+      <c r="B556" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C556" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D556" s="6" t="inlineStr">
+        <is>
+          <t>123365</t>
+        </is>
+      </c>
+      <c r="E556" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F556" s="5" t="n"/>
+    </row>
+    <row r="557" ht="20.25" customHeight="1">
+      <c r="A557" s="5" t="n">
+        <v>803</v>
+      </c>
+      <c r="B557" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C557" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D557" s="6" t="inlineStr">
+        <is>
+          <t>123601</t>
+        </is>
+      </c>
+      <c r="E557" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F557" s="5" t="n"/>
+    </row>
+    <row r="558" ht="20.25" customHeight="1">
+      <c r="A558" s="5" t="n">
+        <v>804</v>
+      </c>
+      <c r="B558" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C558" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D558" s="6" t="inlineStr">
+        <is>
+          <t>123602</t>
+        </is>
+      </c>
+      <c r="E558" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F558" s="5" t="n"/>
+    </row>
+    <row r="559" ht="20.25" customHeight="1">
+      <c r="A559" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="B559" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C559" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D559" s="6" t="inlineStr">
+        <is>
+          <t>123603</t>
+        </is>
+      </c>
+      <c r="E559" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F559" s="5" t="n"/>
+    </row>
+    <row r="560" ht="20.25" customHeight="1">
+      <c r="A560" s="5" t="n">
+        <v>806</v>
+      </c>
+      <c r="B560" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C560" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D560" s="6" t="inlineStr">
+        <is>
+          <t>123604</t>
+        </is>
+      </c>
+      <c r="E560" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F560" s="5" t="n"/>
+    </row>
+    <row r="561" ht="20.25" customHeight="1">
+      <c r="A561" s="5" t="n">
+        <v>807</v>
+      </c>
+      <c r="B561" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C561" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D561" s="6" t="inlineStr">
+        <is>
+          <t>123364</t>
+        </is>
+      </c>
+      <c r="E561" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F561" s="5" t="n"/>
+    </row>
+    <row r="562" ht="22" customHeight="1">
+      <c r="A562" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (557 BAL)</t>
+        </is>
+      </c>
+      <c r="B562" s="4" t="n"/>
+      <c r="C562" s="4" t="n"/>
+      <c r="D562" s="4" t="n"/>
+      <c r="E562" s="4">
+        <f>SUM(E5:E561)</f>
         <v/>
       </c>
-      <c r="F539" s="4" t="inlineStr">
+      <c r="F562" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -11281,7 +11741,7 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A539:D539"/>
+    <mergeCell ref="A562:D562"/>
     <mergeCell ref="B3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11294,7 +11754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I539"/>
+  <dimension ref="A1:I562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11311,14 +11771,14 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 5 SEPTEMBER 2026)</t>
+          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 6 SEPTEMBER 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 534 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 557 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -30504,34 +30964,34 @@
       </c>
       <c r="B522" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C522" s="9" t="inlineStr">
         <is>
-          <t>SABTU</t>
+          <t>MINGGU</t>
         </is>
       </c>
       <c r="D522" s="9" t="n">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="E522" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F522" s="9" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G522" s="10" t="inlineStr">
         <is>
-          <t>123141</t>
+          <t>123592</t>
         </is>
       </c>
       <c r="H522" s="9" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I522" s="11" t="inlineStr">
         <is>
-          <t>grade 5 sep.xlsx</t>
+          <t>grade 6 september.xlsx</t>
         </is>
       </c>
     </row>
@@ -30541,34 +31001,34 @@
       </c>
       <c r="B523" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C523" s="9" t="inlineStr">
         <is>
-          <t>SABTU</t>
+          <t>MINGGU</t>
         </is>
       </c>
       <c r="D523" s="9" t="n">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="E523" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F523" s="9" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G523" s="10" t="inlineStr">
         <is>
-          <t>123143</t>
+          <t>123596</t>
         </is>
       </c>
       <c r="H523" s="9" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I523" s="11" t="inlineStr">
         <is>
-          <t>grade 5 sep.xlsx</t>
+          <t>grade 6 september.xlsx</t>
         </is>
       </c>
     </row>
@@ -30578,34 +31038,34 @@
       </c>
       <c r="B524" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C524" s="9" t="inlineStr">
         <is>
-          <t>SABTU</t>
+          <t>MINGGU</t>
         </is>
       </c>
       <c r="D524" s="9" t="n">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="E524" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F524" s="9" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G524" s="10" t="inlineStr">
         <is>
-          <t>123142</t>
+          <t>123595</t>
         </is>
       </c>
       <c r="H524" s="9" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I524" s="11" t="inlineStr">
         <is>
-          <t>grade 5 sep.xlsx</t>
+          <t>grade 6 september.xlsx</t>
         </is>
       </c>
     </row>
@@ -30615,34 +31075,34 @@
       </c>
       <c r="B525" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C525" s="9" t="inlineStr">
         <is>
-          <t>SABTU</t>
+          <t>MINGGU</t>
         </is>
       </c>
       <c r="D525" s="9" t="n">
-        <v>764</v>
+        <v>759</v>
       </c>
       <c r="E525" s="9" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F525" s="9" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G525" s="10" t="inlineStr">
         <is>
-          <t>123304</t>
+          <t>123593</t>
         </is>
       </c>
       <c r="H525" s="9" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I525" s="11" t="inlineStr">
         <is>
-          <t>grade 5 sep.xlsx</t>
+          <t>grade 6 september.xlsx</t>
         </is>
       </c>
     </row>
@@ -30652,34 +31112,34 @@
       </c>
       <c r="B526" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C526" s="9" t="inlineStr">
         <is>
-          <t>SABTU</t>
+          <t>MINGGU</t>
         </is>
       </c>
       <c r="D526" s="9" t="n">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="E526" s="9" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F526" s="9" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G526" s="10" t="inlineStr">
         <is>
-          <t>940842</t>
+          <t>123594</t>
         </is>
       </c>
       <c r="H526" s="9" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I526" s="11" t="inlineStr">
         <is>
-          <t>grade 5 sep.xlsx</t>
+          <t>grade 6 september.xlsx</t>
         </is>
       </c>
     </row>
@@ -30698,21 +31158,21 @@
         </is>
       </c>
       <c r="D527" s="9" t="n">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="E527" s="9" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="F527" s="9" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G527" s="10" t="inlineStr">
         <is>
-          <t>940847</t>
+          <t>123141</t>
         </is>
       </c>
       <c r="H527" s="9" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="I527" s="11" t="inlineStr">
         <is>
@@ -30735,21 +31195,21 @@
         </is>
       </c>
       <c r="D528" s="9" t="n">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="E528" s="9" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F528" s="9" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G528" s="10" t="inlineStr">
         <is>
-          <t>940843</t>
+          <t>123143</t>
         </is>
       </c>
       <c r="H528" s="9" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="I528" s="11" t="inlineStr">
         <is>
@@ -30772,21 +31232,21 @@
         </is>
       </c>
       <c r="D529" s="9" t="n">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="E529" s="9" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F529" s="9" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G529" s="10" t="inlineStr">
         <is>
-          <t>123144</t>
+          <t>123142</t>
         </is>
       </c>
       <c r="H529" s="9" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I529" s="11" t="inlineStr">
         <is>
@@ -30809,21 +31269,21 @@
         </is>
       </c>
       <c r="D530" s="9" t="n">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="E530" s="9" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F530" s="9" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G530" s="10" t="inlineStr">
         <is>
-          <t>123305</t>
+          <t>123304</t>
         </is>
       </c>
       <c r="H530" s="9" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="I530" s="11" t="inlineStr">
         <is>
@@ -30846,7 +31306,7 @@
         </is>
       </c>
       <c r="D531" s="9" t="n">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="E531" s="9" t="n">
         <v>66</v>
@@ -30856,11 +31316,11 @@
       </c>
       <c r="G531" s="10" t="inlineStr">
         <is>
-          <t>940844</t>
+          <t>940842</t>
         </is>
       </c>
       <c r="H531" s="9" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I531" s="11" t="inlineStr">
         <is>
@@ -30883,7 +31343,7 @@
         </is>
       </c>
       <c r="D532" s="9" t="n">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="E532" s="9" t="n">
         <v>62</v>
@@ -30893,11 +31353,11 @@
       </c>
       <c r="G532" s="10" t="inlineStr">
         <is>
-          <t>940848</t>
+          <t>940847</t>
         </is>
       </c>
       <c r="H532" s="9" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I532" s="11" t="inlineStr">
         <is>
@@ -30920,17 +31380,17 @@
         </is>
       </c>
       <c r="D533" s="9" t="n">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="E533" s="9" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F533" s="9" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G533" s="10" t="inlineStr">
         <is>
-          <t>940840</t>
+          <t>940843</t>
         </is>
       </c>
       <c r="H533" s="9" t="n">
@@ -30957,21 +31417,21 @@
         </is>
       </c>
       <c r="D534" s="9" t="n">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="E534" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F534" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G534" s="10" t="inlineStr">
         <is>
-          <t>940841</t>
+          <t>123144</t>
         </is>
       </c>
       <c r="H534" s="9" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I534" s="11" t="inlineStr">
         <is>
@@ -30994,21 +31454,21 @@
         </is>
       </c>
       <c r="D535" s="9" t="n">
-        <v>786</v>
+        <v>769</v>
       </c>
       <c r="E535" s="9" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F535" s="9" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G535" s="10" t="inlineStr">
         <is>
-          <t>123307</t>
+          <t>123305</t>
         </is>
       </c>
       <c r="H535" s="9" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I535" s="11" t="inlineStr">
         <is>
@@ -31031,21 +31491,21 @@
         </is>
       </c>
       <c r="D536" s="9" t="n">
-        <v>787</v>
+        <v>770</v>
       </c>
       <c r="E536" s="9" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F536" s="9" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G536" s="10" t="inlineStr">
         <is>
-          <t>940846</t>
+          <t>940844</t>
         </is>
       </c>
       <c r="H536" s="9" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I536" s="11" t="inlineStr">
         <is>
@@ -31068,21 +31528,21 @@
         </is>
       </c>
       <c r="D537" s="9" t="n">
-        <v>788</v>
+        <v>771</v>
       </c>
       <c r="E537" s="9" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F537" s="9" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="G537" s="10" t="inlineStr">
         <is>
-          <t>123306</t>
+          <t>940848</t>
         </is>
       </c>
       <c r="H537" s="9" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I537" s="11" t="inlineStr">
         <is>
@@ -31105,45 +31565,896 @@
         </is>
       </c>
       <c r="D538" s="9" t="n">
+        <v>772</v>
+      </c>
+      <c r="E538" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F538" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G538" s="10" t="inlineStr">
+        <is>
+          <t>940840</t>
+        </is>
+      </c>
+      <c r="H538" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I538" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="539" ht="20" customHeight="1">
+      <c r="A539" s="9" t="n">
+        <v>535</v>
+      </c>
+      <c r="B539" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C539" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D539" s="9" t="n">
+        <v>773</v>
+      </c>
+      <c r="E539" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F539" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G539" s="10" t="inlineStr">
+        <is>
+          <t>940841</t>
+        </is>
+      </c>
+      <c r="H539" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I539" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="540" ht="20" customHeight="1">
+      <c r="A540" s="9" t="n">
+        <v>536</v>
+      </c>
+      <c r="B540" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C540" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D540" s="9" t="n">
+        <v>786</v>
+      </c>
+      <c r="E540" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F540" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G540" s="10" t="inlineStr">
+        <is>
+          <t>123307</t>
+        </is>
+      </c>
+      <c r="H540" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I540" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="541" ht="20" customHeight="1">
+      <c r="A541" s="9" t="n">
+        <v>537</v>
+      </c>
+      <c r="B541" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C541" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D541" s="9" t="n">
+        <v>787</v>
+      </c>
+      <c r="E541" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F541" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G541" s="10" t="inlineStr">
+        <is>
+          <t>940846</t>
+        </is>
+      </c>
+      <c r="H541" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I541" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="542" ht="20" customHeight="1">
+      <c r="A542" s="9" t="n">
+        <v>538</v>
+      </c>
+      <c r="B542" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C542" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D542" s="9" t="n">
+        <v>788</v>
+      </c>
+      <c r="E542" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F542" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G542" s="10" t="inlineStr">
+        <is>
+          <t>123306</t>
+        </is>
+      </c>
+      <c r="H542" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I542" s="11" t="inlineStr">
+        <is>
+          <t>grade 5 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="543" ht="20" customHeight="1">
+      <c r="A543" s="9" t="n">
+        <v>539</v>
+      </c>
+      <c r="B543" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="C543" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D543" s="9" t="n">
         <v>789</v>
       </c>
-      <c r="E538" s="9" t="n">
+      <c r="E543" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="F538" s="9" t="n">
+      <c r="F543" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="G538" s="10" t="inlineStr">
+      <c r="G543" s="10" t="inlineStr">
         <is>
           <t>123145</t>
         </is>
       </c>
-      <c r="H538" s="9" t="n">
+      <c r="H543" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="I538" s="11" t="inlineStr">
+      <c r="I543" s="11" t="inlineStr">
         <is>
           <t>grade 5 sep.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="539">
-      <c r="A539" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (534 BAL)</t>
-        </is>
-      </c>
-      <c r="B539" s="4" t="n"/>
-      <c r="C539" s="4" t="n"/>
-      <c r="D539" s="4" t="n"/>
-      <c r="E539" s="4" t="n"/>
-      <c r="F539" s="4" t="n"/>
-      <c r="G539" s="4" t="n"/>
-      <c r="H539" s="4">
-        <f>SUM(H5:H538)</f>
+    <row r="544" ht="20" customHeight="1">
+      <c r="A544" s="9" t="n">
+        <v>540</v>
+      </c>
+      <c r="B544" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C544" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D544" s="9" t="n">
+        <v>790</v>
+      </c>
+      <c r="E544" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F544" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G544" s="10" t="inlineStr">
+        <is>
+          <t>123420</t>
+        </is>
+      </c>
+      <c r="H544" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I544" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="545" ht="20" customHeight="1">
+      <c r="A545" s="9" t="n">
+        <v>541</v>
+      </c>
+      <c r="B545" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C545" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D545" s="9" t="n">
+        <v>791</v>
+      </c>
+      <c r="E545" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F545" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G545" s="10" t="inlineStr">
+        <is>
+          <t>123423</t>
+        </is>
+      </c>
+      <c r="H545" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I545" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="546" ht="20" customHeight="1">
+      <c r="A546" s="9" t="n">
+        <v>542</v>
+      </c>
+      <c r="B546" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C546" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D546" s="9" t="n">
+        <v>792</v>
+      </c>
+      <c r="E546" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F546" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G546" s="10" t="inlineStr">
+        <is>
+          <t>123422</t>
+        </is>
+      </c>
+      <c r="H546" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I546" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="547" ht="20" customHeight="1">
+      <c r="A547" s="9" t="n">
+        <v>543</v>
+      </c>
+      <c r="B547" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C547" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D547" s="9" t="n">
+        <v>793</v>
+      </c>
+      <c r="E547" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F547" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G547" s="10" t="inlineStr">
+        <is>
+          <t>123421</t>
+        </is>
+      </c>
+      <c r="H547" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I547" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="548" ht="20" customHeight="1">
+      <c r="A548" s="9" t="n">
+        <v>544</v>
+      </c>
+      <c r="B548" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C548" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D548" s="9" t="n">
+        <v>794</v>
+      </c>
+      <c r="E548" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F548" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G548" s="10" t="inlineStr">
+        <is>
+          <t>39352</t>
+        </is>
+      </c>
+      <c r="H548" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I548" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="549" ht="20" customHeight="1">
+      <c r="A549" s="9" t="n">
+        <v>545</v>
+      </c>
+      <c r="B549" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C549" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D549" s="9" t="n">
+        <v>795</v>
+      </c>
+      <c r="E549" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F549" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G549" s="10" t="inlineStr">
+        <is>
+          <t>39351</t>
+        </is>
+      </c>
+      <c r="H549" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I549" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="550" ht="20" customHeight="1">
+      <c r="A550" s="9" t="n">
+        <v>546</v>
+      </c>
+      <c r="B550" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C550" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D550" s="9" t="n">
+        <v>796</v>
+      </c>
+      <c r="E550" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F550" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G550" s="10" t="inlineStr">
+        <is>
+          <t>123367</t>
+        </is>
+      </c>
+      <c r="H550" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I550" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="551" ht="20" customHeight="1">
+      <c r="A551" s="9" t="n">
+        <v>547</v>
+      </c>
+      <c r="B551" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C551" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D551" s="9" t="n">
+        <v>797</v>
+      </c>
+      <c r="E551" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F551" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G551" s="10" t="inlineStr">
+        <is>
+          <t>123368</t>
+        </is>
+      </c>
+      <c r="H551" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I551" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="552" ht="20" customHeight="1">
+      <c r="A552" s="9" t="n">
+        <v>548</v>
+      </c>
+      <c r="B552" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C552" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D552" s="9" t="n">
+        <v>798</v>
+      </c>
+      <c r="E552" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F552" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G552" s="10" t="inlineStr">
+        <is>
+          <t>123591</t>
+        </is>
+      </c>
+      <c r="H552" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I552" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="553" ht="20" customHeight="1">
+      <c r="A553" s="9" t="n">
+        <v>549</v>
+      </c>
+      <c r="B553" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C553" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D553" s="9" t="n">
+        <v>799</v>
+      </c>
+      <c r="E553" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F553" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G553" s="10" t="inlineStr">
+        <is>
+          <t>123605</t>
+        </is>
+      </c>
+      <c r="H553" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I553" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="554" ht="20" customHeight="1">
+      <c r="A554" s="9" t="n">
+        <v>550</v>
+      </c>
+      <c r="B554" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C554" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D554" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="E554" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F554" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G554" s="10" t="inlineStr">
+        <is>
+          <t>39350</t>
+        </is>
+      </c>
+      <c r="H554" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I554" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="555" ht="20" customHeight="1">
+      <c r="A555" s="9" t="n">
+        <v>551</v>
+      </c>
+      <c r="B555" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C555" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D555" s="9" t="n">
+        <v>801</v>
+      </c>
+      <c r="E555" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F555" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G555" s="10" t="inlineStr">
+        <is>
+          <t>123366</t>
+        </is>
+      </c>
+      <c r="H555" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I555" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="556" ht="20" customHeight="1">
+      <c r="A556" s="9" t="n">
+        <v>552</v>
+      </c>
+      <c r="B556" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C556" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D556" s="9" t="n">
+        <v>802</v>
+      </c>
+      <c r="E556" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F556" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G556" s="10" t="inlineStr">
+        <is>
+          <t>123365</t>
+        </is>
+      </c>
+      <c r="H556" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I556" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="20" customHeight="1">
+      <c r="A557" s="9" t="n">
+        <v>553</v>
+      </c>
+      <c r="B557" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C557" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D557" s="9" t="n">
+        <v>803</v>
+      </c>
+      <c r="E557" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F557" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G557" s="10" t="inlineStr">
+        <is>
+          <t>123601</t>
+        </is>
+      </c>
+      <c r="H557" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I557" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="558" ht="20" customHeight="1">
+      <c r="A558" s="9" t="n">
+        <v>554</v>
+      </c>
+      <c r="B558" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C558" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D558" s="9" t="n">
+        <v>804</v>
+      </c>
+      <c r="E558" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F558" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G558" s="10" t="inlineStr">
+        <is>
+          <t>123602</t>
+        </is>
+      </c>
+      <c r="H558" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I558" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="559" ht="20" customHeight="1">
+      <c r="A559" s="9" t="n">
+        <v>555</v>
+      </c>
+      <c r="B559" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C559" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D559" s="9" t="n">
+        <v>805</v>
+      </c>
+      <c r="E559" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F559" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G559" s="10" t="inlineStr">
+        <is>
+          <t>123603</t>
+        </is>
+      </c>
+      <c r="H559" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I559" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="560" ht="20" customHeight="1">
+      <c r="A560" s="9" t="n">
+        <v>556</v>
+      </c>
+      <c r="B560" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C560" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D560" s="9" t="n">
+        <v>806</v>
+      </c>
+      <c r="E560" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F560" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G560" s="10" t="inlineStr">
+        <is>
+          <t>123604</t>
+        </is>
+      </c>
+      <c r="H560" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I560" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="561" ht="20" customHeight="1">
+      <c r="A561" s="9" t="n">
+        <v>557</v>
+      </c>
+      <c r="B561" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C561" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D561" s="9" t="n">
+        <v>807</v>
+      </c>
+      <c r="E561" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="F561" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G561" s="10" t="inlineStr">
+        <is>
+          <t>123364</t>
+        </is>
+      </c>
+      <c r="H561" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I561" s="11" t="inlineStr">
+        <is>
+          <t>grade 6 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (557 BAL)</t>
+        </is>
+      </c>
+      <c r="B562" s="4" t="n"/>
+      <c r="C562" s="4" t="n"/>
+      <c r="D562" s="4" t="n"/>
+      <c r="E562" s="4" t="n"/>
+      <c r="F562" s="4" t="n"/>
+      <c r="G562" s="4" t="n"/>
+      <c r="H562" s="4">
+        <f>SUM(H5:H561)</f>
         <v/>
       </c>
-      <c r="I539" s="4" t="inlineStr">
+      <c r="I562" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -31152,7 +32463,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A539:G539"/>
+    <mergeCell ref="A562:G562"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31165,7 +32476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -31187,7 +32498,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Periode: 21 Agustus 2026 s/d 5 September 2026</t>
+          <t>Periode: 21 Agustus 2026 s/d 6 September 2026</t>
         </is>
       </c>
     </row>
@@ -31663,35 +32974,64 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>MINGGU</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>881</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>756 - 807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4">
-        <f>SUM(D5:D19)</f>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4">
+        <f>SUM(D5:D20)</f>
         <v/>
       </c>
-      <c r="E20" s="4">
-        <f>SUM(E5:E19)</f>
+      <c r="E21" s="4">
+        <f>SUM(E5:E20)</f>
         <v/>
       </c>
-      <c r="F20" s="4">
-        <f>AVERAGE(F5:F19)</f>
+      <c r="F21" s="4">
+        <f>AVERAGE(F5:F20)</f>
         <v/>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>3 - 789</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>3 - 807</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update data tanggal 7 September 2026 (49 bal: No Gud 808-857), sync Supabase, and update master rekap
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F562"/>
+  <dimension ref="A1:F611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11714,20 +11714,1000 @@
       </c>
       <c r="F561" s="5" t="n"/>
     </row>
-    <row r="562" ht="22" customHeight="1">
-      <c r="A562" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (557 BAL)</t>
-        </is>
-      </c>
-      <c r="B562" s="4" t="n"/>
-      <c r="C562" s="4" t="n"/>
-      <c r="D562" s="4" t="n"/>
-      <c r="E562" s="4">
-        <f>SUM(E5:E561)</f>
+    <row r="562" ht="20.25" customHeight="1">
+      <c r="A562" s="5" t="n">
+        <v>808</v>
+      </c>
+      <c r="B562" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C562" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D562" s="6" t="inlineStr">
+        <is>
+          <t>123997</t>
+        </is>
+      </c>
+      <c r="E562" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F562" s="5" t="n"/>
+    </row>
+    <row r="563" ht="20.25" customHeight="1">
+      <c r="A563" s="5" t="n">
+        <v>809</v>
+      </c>
+      <c r="B563" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C563" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D563" s="6" t="inlineStr">
+        <is>
+          <t>39860</t>
+        </is>
+      </c>
+      <c r="E563" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F563" s="5" t="n"/>
+    </row>
+    <row r="564" ht="20.25" customHeight="1">
+      <c r="A564" s="5" t="n">
+        <v>810</v>
+      </c>
+      <c r="B564" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C564" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D564" s="6" t="inlineStr">
+        <is>
+          <t>124000</t>
+        </is>
+      </c>
+      <c r="E564" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F564" s="5" t="n"/>
+    </row>
+    <row r="565" ht="20.25" customHeight="1">
+      <c r="A565" s="5" t="n">
+        <v>811</v>
+      </c>
+      <c r="B565" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C565" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D565" s="6" t="inlineStr">
+        <is>
+          <t>123998</t>
+        </is>
+      </c>
+      <c r="E565" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F565" s="5" t="n"/>
+    </row>
+    <row r="566" ht="20.25" customHeight="1">
+      <c r="A566" s="5" t="n">
+        <v>812</v>
+      </c>
+      <c r="B566" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C566" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D566" s="6" t="inlineStr">
+        <is>
+          <t>123999</t>
+        </is>
+      </c>
+      <c r="E566" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F566" s="5" t="n"/>
+    </row>
+    <row r="567" ht="20.25" customHeight="1">
+      <c r="A567" s="5" t="n">
+        <v>813</v>
+      </c>
+      <c r="B567" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C567" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D567" s="6" t="inlineStr">
+        <is>
+          <t>123287</t>
+        </is>
+      </c>
+      <c r="E567" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F567" s="5" t="n"/>
+    </row>
+    <row r="568" ht="20.25" customHeight="1">
+      <c r="A568" s="5" t="n">
+        <v>814</v>
+      </c>
+      <c r="B568" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C568" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D568" s="6" t="inlineStr">
+        <is>
+          <t>123284</t>
+        </is>
+      </c>
+      <c r="E568" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F568" s="5" t="n"/>
+    </row>
+    <row r="569" ht="20.25" customHeight="1">
+      <c r="A569" s="5" t="n">
+        <v>815</v>
+      </c>
+      <c r="B569" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C569" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D569" s="6" t="inlineStr">
+        <is>
+          <t>123890</t>
+        </is>
+      </c>
+      <c r="E569" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F569" s="5" t="n"/>
+    </row>
+    <row r="570" ht="20.25" customHeight="1">
+      <c r="A570" s="5" t="n">
+        <v>816</v>
+      </c>
+      <c r="B570" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C570" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D570" s="6" t="inlineStr">
+        <is>
+          <t>39862</t>
+        </is>
+      </c>
+      <c r="E570" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F570" s="5" t="n"/>
+    </row>
+    <row r="571" ht="20.25" customHeight="1">
+      <c r="A571" s="5" t="n">
+        <v>817</v>
+      </c>
+      <c r="B571" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C571" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D571" s="6" t="inlineStr">
+        <is>
+          <t>39851</t>
+        </is>
+      </c>
+      <c r="E571" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F571" s="5" t="n"/>
+    </row>
+    <row r="572" ht="20.25" customHeight="1">
+      <c r="A572" s="5" t="n">
+        <v>818</v>
+      </c>
+      <c r="B572" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C572" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D572" s="6" t="inlineStr">
+        <is>
+          <t>123889</t>
+        </is>
+      </c>
+      <c r="E572" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F572" s="5" t="n"/>
+    </row>
+    <row r="573" ht="20.25" customHeight="1">
+      <c r="A573" s="5" t="n">
+        <v>819</v>
+      </c>
+      <c r="B573" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C573" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D573" s="6" t="inlineStr">
+        <is>
+          <t>123911</t>
+        </is>
+      </c>
+      <c r="E573" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F573" s="5" t="n"/>
+    </row>
+    <row r="574" ht="20.25" customHeight="1">
+      <c r="A574" s="5" t="n">
+        <v>820</v>
+      </c>
+      <c r="B574" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C574" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D574" s="6" t="inlineStr">
+        <is>
+          <t>123891</t>
+        </is>
+      </c>
+      <c r="E574" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F574" s="5" t="n"/>
+    </row>
+    <row r="575" ht="20.25" customHeight="1">
+      <c r="A575" s="5" t="n">
+        <v>821</v>
+      </c>
+      <c r="B575" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C575" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D575" s="6" t="inlineStr">
+        <is>
+          <t>123500</t>
+        </is>
+      </c>
+      <c r="E575" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F575" s="5" t="n"/>
+    </row>
+    <row r="576" ht="20.25" customHeight="1">
+      <c r="A576" s="5" t="n">
+        <v>822</v>
+      </c>
+      <c r="B576" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C576" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D576" s="6" t="inlineStr">
+        <is>
+          <t>123286</t>
+        </is>
+      </c>
+      <c r="E576" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F576" s="5" t="n"/>
+    </row>
+    <row r="577" ht="20.25" customHeight="1">
+      <c r="A577" s="5" t="n">
+        <v>823</v>
+      </c>
+      <c r="B577" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C577" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D577" s="6" t="inlineStr">
+        <is>
+          <t>123285</t>
+        </is>
+      </c>
+      <c r="E577" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F577" s="5" t="n"/>
+    </row>
+    <row r="578" ht="20.25" customHeight="1">
+      <c r="A578" s="5" t="n">
+        <v>824</v>
+      </c>
+      <c r="B578" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C578" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D578" s="6" t="inlineStr">
+        <is>
+          <t>39852</t>
+        </is>
+      </c>
+      <c r="E578" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F578" s="5" t="n"/>
+    </row>
+    <row r="579" ht="20.25" customHeight="1">
+      <c r="A579" s="5" t="n">
+        <v>825</v>
+      </c>
+      <c r="B579" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C579" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D579" s="6" t="inlineStr">
+        <is>
+          <t>39863</t>
+        </is>
+      </c>
+      <c r="E579" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F579" s="5" t="n"/>
+    </row>
+    <row r="580" ht="20.25" customHeight="1">
+      <c r="A580" s="5" t="n">
+        <v>826</v>
+      </c>
+      <c r="B580" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C580" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D580" s="6" t="inlineStr">
+        <is>
+          <t>123895</t>
+        </is>
+      </c>
+      <c r="E580" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F580" s="5" t="n"/>
+    </row>
+    <row r="581" ht="20.25" customHeight="1">
+      <c r="A581" s="5" t="n">
+        <v>827</v>
+      </c>
+      <c r="B581" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C581" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D581" s="6" t="inlineStr">
+        <is>
+          <t>39864</t>
+        </is>
+      </c>
+      <c r="E581" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F581" s="5" t="n"/>
+    </row>
+    <row r="582" ht="20.25" customHeight="1">
+      <c r="A582" s="5" t="n">
+        <v>828</v>
+      </c>
+      <c r="B582" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C582" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D582" s="6" t="inlineStr">
+        <is>
+          <t>39861</t>
+        </is>
+      </c>
+      <c r="E582" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F582" s="5" t="n"/>
+    </row>
+    <row r="583" ht="20.25" customHeight="1">
+      <c r="A583" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="B583" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C583" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D583" s="6" t="inlineStr">
+        <is>
+          <t>123896</t>
+        </is>
+      </c>
+      <c r="E583" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F583" s="5" t="n"/>
+    </row>
+    <row r="584" ht="20.25" customHeight="1">
+      <c r="A584" s="5" t="n">
+        <v>830</v>
+      </c>
+      <c r="B584" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C584" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D584" s="6" t="inlineStr">
+        <is>
+          <t>123894</t>
+        </is>
+      </c>
+      <c r="E584" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F584" s="5" t="n"/>
+    </row>
+    <row r="585" ht="20.25" customHeight="1">
+      <c r="A585" s="5" t="n">
+        <v>831</v>
+      </c>
+      <c r="B585" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C585" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D585" s="6" t="inlineStr">
+        <is>
+          <t>123893</t>
+        </is>
+      </c>
+      <c r="E585" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F585" s="5" t="n"/>
+    </row>
+    <row r="586" ht="20.25" customHeight="1">
+      <c r="A586" s="5" t="n">
+        <v>832</v>
+      </c>
+      <c r="B586" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C586" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D586" s="6" t="inlineStr">
+        <is>
+          <t>123892</t>
+        </is>
+      </c>
+      <c r="E586" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F586" s="5" t="n"/>
+    </row>
+    <row r="587" ht="20.25" customHeight="1">
+      <c r="A587" s="5" t="n">
+        <v>834</v>
+      </c>
+      <c r="B587" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="C587" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D587" s="6" t="inlineStr">
+        <is>
+          <t>39853</t>
+        </is>
+      </c>
+      <c r="E587" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F587" s="5" t="n"/>
+    </row>
+    <row r="588" ht="20.25" customHeight="1">
+      <c r="A588" s="5" t="n">
+        <v>835</v>
+      </c>
+      <c r="B588" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C588" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D588" s="6" t="inlineStr">
+        <is>
+          <t>39856</t>
+        </is>
+      </c>
+      <c r="E588" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F588" s="5" t="n"/>
+    </row>
+    <row r="589" ht="20.25" customHeight="1">
+      <c r="A589" s="5" t="n">
+        <v>836</v>
+      </c>
+      <c r="B589" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C589" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D589" s="6" t="inlineStr">
+        <is>
+          <t>39854</t>
+        </is>
+      </c>
+      <c r="E589" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F589" s="5" t="n"/>
+    </row>
+    <row r="590" ht="20.25" customHeight="1">
+      <c r="A590" s="5" t="n">
+        <v>837</v>
+      </c>
+      <c r="B590" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C590" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D590" s="6" t="inlineStr">
+        <is>
+          <t>39855</t>
+        </is>
+      </c>
+      <c r="E590" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F590" s="5" t="n"/>
+    </row>
+    <row r="591" ht="20.25" customHeight="1">
+      <c r="A591" s="5" t="n">
+        <v>838</v>
+      </c>
+      <c r="B591" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C591" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D591" s="6" t="inlineStr">
+        <is>
+          <t>39858</t>
+        </is>
+      </c>
+      <c r="E591" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F591" s="5" t="n"/>
+    </row>
+    <row r="592" ht="20.25" customHeight="1">
+      <c r="A592" s="5" t="n">
+        <v>839</v>
+      </c>
+      <c r="B592" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C592" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D592" s="6" t="inlineStr">
+        <is>
+          <t>39857</t>
+        </is>
+      </c>
+      <c r="E592" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F592" s="5" t="n"/>
+    </row>
+    <row r="593" ht="20.25" customHeight="1">
+      <c r="A593" s="5" t="n">
+        <v>840</v>
+      </c>
+      <c r="B593" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C593" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D593" s="6" t="inlineStr">
+        <is>
+          <t>39859</t>
+        </is>
+      </c>
+      <c r="E593" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F593" s="5" t="n"/>
+    </row>
+    <row r="594" ht="20.25" customHeight="1">
+      <c r="A594" s="5" t="n">
+        <v>841</v>
+      </c>
+      <c r="B594" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C594" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D594" s="6" t="inlineStr">
+        <is>
+          <t>35113</t>
+        </is>
+      </c>
+      <c r="E594" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F594" s="5" t="n"/>
+    </row>
+    <row r="595" ht="20.25" customHeight="1">
+      <c r="A595" s="5" t="n">
+        <v>842</v>
+      </c>
+      <c r="B595" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C595" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D595" s="6" t="inlineStr">
+        <is>
+          <t>35112</t>
+        </is>
+      </c>
+      <c r="E595" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F595" s="5" t="n"/>
+    </row>
+    <row r="596" ht="20.25" customHeight="1">
+      <c r="A596" s="5" t="n">
+        <v>843</v>
+      </c>
+      <c r="B596" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C596" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D596" s="6" t="inlineStr">
+        <is>
+          <t>123912</t>
+        </is>
+      </c>
+      <c r="E596" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F596" s="5" t="n"/>
+    </row>
+    <row r="597" ht="20.25" customHeight="1">
+      <c r="A597" s="5" t="n">
+        <v>844</v>
+      </c>
+      <c r="B597" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C597" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D597" s="6" t="inlineStr">
+        <is>
+          <t>123915</t>
+        </is>
+      </c>
+      <c r="E597" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F597" s="5" t="n"/>
+    </row>
+    <row r="598" ht="20.25" customHeight="1">
+      <c r="A598" s="5" t="n">
+        <v>845</v>
+      </c>
+      <c r="B598" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C598" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D598" s="6" t="inlineStr">
+        <is>
+          <t>123916</t>
+        </is>
+      </c>
+      <c r="E598" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F598" s="5" t="n"/>
+    </row>
+    <row r="599" ht="20.25" customHeight="1">
+      <c r="A599" s="5" t="n">
+        <v>846</v>
+      </c>
+      <c r="B599" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C599" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D599" s="6" t="inlineStr">
+        <is>
+          <t>123914</t>
+        </is>
+      </c>
+      <c r="E599" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F599" s="5" t="n"/>
+    </row>
+    <row r="600" ht="20.25" customHeight="1">
+      <c r="A600" s="5" t="n">
+        <v>847</v>
+      </c>
+      <c r="B600" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C600" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D600" s="6" t="inlineStr">
+        <is>
+          <t>123913</t>
+        </is>
+      </c>
+      <c r="E600" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F600" s="5" t="n"/>
+    </row>
+    <row r="601" ht="20.25" customHeight="1">
+      <c r="A601" s="5" t="n">
+        <v>848</v>
+      </c>
+      <c r="B601" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C601" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D601" s="6" t="inlineStr">
+        <is>
+          <t>123917</t>
+        </is>
+      </c>
+      <c r="E601" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F601" s="5" t="n"/>
+    </row>
+    <row r="602" ht="20.25" customHeight="1">
+      <c r="A602" s="5" t="n">
+        <v>849</v>
+      </c>
+      <c r="B602" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C602" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D602" s="6" t="inlineStr">
+        <is>
+          <t>123919</t>
+        </is>
+      </c>
+      <c r="E602" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F602" s="5" t="n"/>
+    </row>
+    <row r="603" ht="20.25" customHeight="1">
+      <c r="A603" s="5" t="n">
+        <v>850</v>
+      </c>
+      <c r="B603" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C603" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D603" s="6" t="inlineStr">
+        <is>
+          <t>123921</t>
+        </is>
+      </c>
+      <c r="E603" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F603" s="5" t="n"/>
+    </row>
+    <row r="604" ht="20.25" customHeight="1">
+      <c r="A604" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="B604" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C604" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D604" s="6" t="inlineStr">
+        <is>
+          <t>123918</t>
+        </is>
+      </c>
+      <c r="E604" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F604" s="5" t="n"/>
+    </row>
+    <row r="605" ht="20.25" customHeight="1">
+      <c r="A605" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="B605" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C605" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D605" s="6" t="inlineStr">
+        <is>
+          <t>123920</t>
+        </is>
+      </c>
+      <c r="E605" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F605" s="5" t="n"/>
+    </row>
+    <row r="606" ht="20.25" customHeight="1">
+      <c r="A606" s="5" t="n">
+        <v>853</v>
+      </c>
+      <c r="B606" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="C606" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D606" s="6" t="inlineStr">
+        <is>
+          <t>35117</t>
+        </is>
+      </c>
+      <c r="E606" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F606" s="5" t="n"/>
+    </row>
+    <row r="607" ht="20.25" customHeight="1">
+      <c r="A607" s="5" t="n">
+        <v>854</v>
+      </c>
+      <c r="B607" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="C607" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D607" s="6" t="inlineStr">
+        <is>
+          <t>35114</t>
+        </is>
+      </c>
+      <c r="E607" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F607" s="5" t="n"/>
+    </row>
+    <row r="608" ht="20.25" customHeight="1">
+      <c r="A608" s="5" t="n">
+        <v>855</v>
+      </c>
+      <c r="B608" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="C608" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D608" s="6" t="inlineStr">
+        <is>
+          <t>35116</t>
+        </is>
+      </c>
+      <c r="E608" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F608" s="5" t="n"/>
+    </row>
+    <row r="609" ht="20.25" customHeight="1">
+      <c r="A609" s="5" t="n">
+        <v>856</v>
+      </c>
+      <c r="B609" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="C609" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D609" s="6" t="inlineStr">
+        <is>
+          <t>35115</t>
+        </is>
+      </c>
+      <c r="E609" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F609" s="5" t="n"/>
+    </row>
+    <row r="610" ht="20.25" customHeight="1">
+      <c r="A610" s="5" t="n">
+        <v>857</v>
+      </c>
+      <c r="B610" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C610" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D610" s="6" t="inlineStr">
+        <is>
+          <t>123888</t>
+        </is>
+      </c>
+      <c r="E610" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F610" s="5" t="n"/>
+    </row>
+    <row r="611" ht="22" customHeight="1">
+      <c r="A611" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (606 BAL)</t>
+        </is>
+      </c>
+      <c r="B611" s="4" t="n"/>
+      <c r="C611" s="4" t="n"/>
+      <c r="D611" s="4" t="n"/>
+      <c r="E611" s="4">
+        <f>SUM(E5:E610)</f>
         <v/>
       </c>
-      <c r="F562" s="4" t="inlineStr">
+      <c r="F611" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -11736,12 +12716,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A611:D611"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A562:D562"/>
     <mergeCell ref="B3:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11754,7 +12734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I562"/>
+  <dimension ref="A1:I611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11778,7 +12758,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 557 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 606 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -32438,23 +33418,1836 @@
         </is>
       </c>
     </row>
-    <row r="562">
-      <c r="A562" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (557 BAL)</t>
-        </is>
-      </c>
-      <c r="B562" s="4" t="n"/>
-      <c r="C562" s="4" t="n"/>
-      <c r="D562" s="4" t="n"/>
-      <c r="E562" s="4" t="n"/>
-      <c r="F562" s="4" t="n"/>
-      <c r="G562" s="4" t="n"/>
-      <c r="H562" s="4">
-        <f>SUM(H5:H561)</f>
+    <row r="562" ht="20" customHeight="1">
+      <c r="A562" s="9" t="n">
+        <v>558</v>
+      </c>
+      <c r="B562" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C562" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D562" s="9" t="n">
+        <v>808</v>
+      </c>
+      <c r="E562" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F562" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G562" s="10" t="inlineStr">
+        <is>
+          <t>123997</t>
+        </is>
+      </c>
+      <c r="H562" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I562" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="563" ht="20" customHeight="1">
+      <c r="A563" s="9" t="n">
+        <v>559</v>
+      </c>
+      <c r="B563" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C563" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D563" s="9" t="n">
+        <v>809</v>
+      </c>
+      <c r="E563" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F563" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G563" s="10" t="inlineStr">
+        <is>
+          <t>39860</t>
+        </is>
+      </c>
+      <c r="H563" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I563" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="564" ht="20" customHeight="1">
+      <c r="A564" s="9" t="n">
+        <v>560</v>
+      </c>
+      <c r="B564" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C564" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D564" s="9" t="n">
+        <v>810</v>
+      </c>
+      <c r="E564" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F564" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G564" s="10" t="inlineStr">
+        <is>
+          <t>124000</t>
+        </is>
+      </c>
+      <c r="H564" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I564" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="565" ht="20" customHeight="1">
+      <c r="A565" s="9" t="n">
+        <v>561</v>
+      </c>
+      <c r="B565" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C565" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D565" s="9" t="n">
+        <v>811</v>
+      </c>
+      <c r="E565" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F565" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G565" s="10" t="inlineStr">
+        <is>
+          <t>123998</t>
+        </is>
+      </c>
+      <c r="H565" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I565" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="566" ht="20" customHeight="1">
+      <c r="A566" s="9" t="n">
+        <v>562</v>
+      </c>
+      <c r="B566" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C566" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D566" s="9" t="n">
+        <v>812</v>
+      </c>
+      <c r="E566" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F566" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G566" s="10" t="inlineStr">
+        <is>
+          <t>123999</t>
+        </is>
+      </c>
+      <c r="H566" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I566" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="20" customHeight="1">
+      <c r="A567" s="9" t="n">
+        <v>563</v>
+      </c>
+      <c r="B567" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C567" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D567" s="9" t="n">
+        <v>813</v>
+      </c>
+      <c r="E567" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F567" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G567" s="10" t="inlineStr">
+        <is>
+          <t>123287</t>
+        </is>
+      </c>
+      <c r="H567" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I567" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="568" ht="20" customHeight="1">
+      <c r="A568" s="9" t="n">
+        <v>564</v>
+      </c>
+      <c r="B568" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C568" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D568" s="9" t="n">
+        <v>814</v>
+      </c>
+      <c r="E568" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F568" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G568" s="10" t="inlineStr">
+        <is>
+          <t>123284</t>
+        </is>
+      </c>
+      <c r="H568" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I568" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="569" ht="20" customHeight="1">
+      <c r="A569" s="9" t="n">
+        <v>565</v>
+      </c>
+      <c r="B569" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C569" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D569" s="9" t="n">
+        <v>815</v>
+      </c>
+      <c r="E569" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F569" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G569" s="10" t="inlineStr">
+        <is>
+          <t>123890</t>
+        </is>
+      </c>
+      <c r="H569" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I569" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="570" ht="20" customHeight="1">
+      <c r="A570" s="9" t="n">
+        <v>566</v>
+      </c>
+      <c r="B570" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C570" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D570" s="9" t="n">
+        <v>816</v>
+      </c>
+      <c r="E570" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F570" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G570" s="10" t="inlineStr">
+        <is>
+          <t>39862</t>
+        </is>
+      </c>
+      <c r="H570" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I570" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="571" ht="20" customHeight="1">
+      <c r="A571" s="9" t="n">
+        <v>567</v>
+      </c>
+      <c r="B571" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C571" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D571" s="9" t="n">
+        <v>817</v>
+      </c>
+      <c r="E571" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F571" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G571" s="10" t="inlineStr">
+        <is>
+          <t>39851</t>
+        </is>
+      </c>
+      <c r="H571" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I571" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="572" ht="20" customHeight="1">
+      <c r="A572" s="9" t="n">
+        <v>568</v>
+      </c>
+      <c r="B572" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C572" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D572" s="9" t="n">
+        <v>818</v>
+      </c>
+      <c r="E572" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F572" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G572" s="10" t="inlineStr">
+        <is>
+          <t>123889</t>
+        </is>
+      </c>
+      <c r="H572" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I572" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="573" ht="20" customHeight="1">
+      <c r="A573" s="9" t="n">
+        <v>569</v>
+      </c>
+      <c r="B573" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C573" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D573" s="9" t="n">
+        <v>819</v>
+      </c>
+      <c r="E573" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F573" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G573" s="10" t="inlineStr">
+        <is>
+          <t>123911</t>
+        </is>
+      </c>
+      <c r="H573" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I573" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="574" ht="20" customHeight="1">
+      <c r="A574" s="9" t="n">
+        <v>570</v>
+      </c>
+      <c r="B574" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C574" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D574" s="9" t="n">
+        <v>820</v>
+      </c>
+      <c r="E574" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F574" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G574" s="10" t="inlineStr">
+        <is>
+          <t>123891</t>
+        </is>
+      </c>
+      <c r="H574" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I574" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="575" ht="20" customHeight="1">
+      <c r="A575" s="9" t="n">
+        <v>571</v>
+      </c>
+      <c r="B575" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C575" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D575" s="9" t="n">
+        <v>821</v>
+      </c>
+      <c r="E575" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F575" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G575" s="10" t="inlineStr">
+        <is>
+          <t>123500</t>
+        </is>
+      </c>
+      <c r="H575" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I575" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="576" ht="20" customHeight="1">
+      <c r="A576" s="9" t="n">
+        <v>572</v>
+      </c>
+      <c r="B576" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C576" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D576" s="9" t="n">
+        <v>822</v>
+      </c>
+      <c r="E576" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F576" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G576" s="10" t="inlineStr">
+        <is>
+          <t>123286</t>
+        </is>
+      </c>
+      <c r="H576" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I576" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="577" ht="20" customHeight="1">
+      <c r="A577" s="9" t="n">
+        <v>573</v>
+      </c>
+      <c r="B577" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C577" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D577" s="9" t="n">
+        <v>823</v>
+      </c>
+      <c r="E577" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F577" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G577" s="10" t="inlineStr">
+        <is>
+          <t>123285</t>
+        </is>
+      </c>
+      <c r="H577" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I577" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="578" ht="20" customHeight="1">
+      <c r="A578" s="9" t="n">
+        <v>574</v>
+      </c>
+      <c r="B578" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C578" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D578" s="9" t="n">
+        <v>824</v>
+      </c>
+      <c r="E578" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F578" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G578" s="10" t="inlineStr">
+        <is>
+          <t>39852</t>
+        </is>
+      </c>
+      <c r="H578" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I578" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="579" ht="20" customHeight="1">
+      <c r="A579" s="9" t="n">
+        <v>575</v>
+      </c>
+      <c r="B579" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C579" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D579" s="9" t="n">
+        <v>825</v>
+      </c>
+      <c r="E579" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F579" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G579" s="10" t="inlineStr">
+        <is>
+          <t>39863</t>
+        </is>
+      </c>
+      <c r="H579" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I579" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="580" ht="20" customHeight="1">
+      <c r="A580" s="9" t="n">
+        <v>576</v>
+      </c>
+      <c r="B580" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C580" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D580" s="9" t="n">
+        <v>826</v>
+      </c>
+      <c r="E580" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F580" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G580" s="10" t="inlineStr">
+        <is>
+          <t>123895</t>
+        </is>
+      </c>
+      <c r="H580" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I580" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="20" customHeight="1">
+      <c r="A581" s="9" t="n">
+        <v>577</v>
+      </c>
+      <c r="B581" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C581" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D581" s="9" t="n">
+        <v>827</v>
+      </c>
+      <c r="E581" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F581" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G581" s="10" t="inlineStr">
+        <is>
+          <t>39864</t>
+        </is>
+      </c>
+      <c r="H581" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I581" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="582" ht="20" customHeight="1">
+      <c r="A582" s="9" t="n">
+        <v>578</v>
+      </c>
+      <c r="B582" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C582" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D582" s="9" t="n">
+        <v>828</v>
+      </c>
+      <c r="E582" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F582" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G582" s="10" t="inlineStr">
+        <is>
+          <t>39861</t>
+        </is>
+      </c>
+      <c r="H582" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I582" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="583" ht="20" customHeight="1">
+      <c r="A583" s="9" t="n">
+        <v>579</v>
+      </c>
+      <c r="B583" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C583" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>829</v>
+      </c>
+      <c r="E583" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F583" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G583" s="10" t="inlineStr">
+        <is>
+          <t>123896</t>
+        </is>
+      </c>
+      <c r="H583" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I583" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="584" ht="20" customHeight="1">
+      <c r="A584" s="9" t="n">
+        <v>580</v>
+      </c>
+      <c r="B584" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C584" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D584" s="9" t="n">
+        <v>830</v>
+      </c>
+      <c r="E584" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F584" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G584" s="10" t="inlineStr">
+        <is>
+          <t>123894</t>
+        </is>
+      </c>
+      <c r="H584" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I584" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="20" customHeight="1">
+      <c r="A585" s="9" t="n">
+        <v>581</v>
+      </c>
+      <c r="B585" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C585" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D585" s="9" t="n">
+        <v>831</v>
+      </c>
+      <c r="E585" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F585" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G585" s="10" t="inlineStr">
+        <is>
+          <t>123893</t>
+        </is>
+      </c>
+      <c r="H585" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I585" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="20" customHeight="1">
+      <c r="A586" s="9" t="n">
+        <v>582</v>
+      </c>
+      <c r="B586" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C586" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D586" s="9" t="n">
+        <v>832</v>
+      </c>
+      <c r="E586" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F586" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G586" s="10" t="inlineStr">
+        <is>
+          <t>123892</t>
+        </is>
+      </c>
+      <c r="H586" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I586" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="587" ht="20" customHeight="1">
+      <c r="A587" s="9" t="n">
+        <v>583</v>
+      </c>
+      <c r="B587" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C587" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D587" s="9" t="n">
+        <v>834</v>
+      </c>
+      <c r="E587" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F587" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G587" s="10" t="inlineStr">
+        <is>
+          <t>39853</t>
+        </is>
+      </c>
+      <c r="H587" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I587" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="20" customHeight="1">
+      <c r="A588" s="9" t="n">
+        <v>584</v>
+      </c>
+      <c r="B588" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C588" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D588" s="9" t="n">
+        <v>835</v>
+      </c>
+      <c r="E588" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F588" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G588" s="10" t="inlineStr">
+        <is>
+          <t>39856</t>
+        </is>
+      </c>
+      <c r="H588" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I588" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="20" customHeight="1">
+      <c r="A589" s="9" t="n">
+        <v>585</v>
+      </c>
+      <c r="B589" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C589" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D589" s="9" t="n">
+        <v>836</v>
+      </c>
+      <c r="E589" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F589" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G589" s="10" t="inlineStr">
+        <is>
+          <t>39854</t>
+        </is>
+      </c>
+      <c r="H589" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I589" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="590" ht="20" customHeight="1">
+      <c r="A590" s="9" t="n">
+        <v>586</v>
+      </c>
+      <c r="B590" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C590" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D590" s="9" t="n">
+        <v>837</v>
+      </c>
+      <c r="E590" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F590" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G590" s="10" t="inlineStr">
+        <is>
+          <t>39855</t>
+        </is>
+      </c>
+      <c r="H590" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I590" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="591" ht="20" customHeight="1">
+      <c r="A591" s="9" t="n">
+        <v>587</v>
+      </c>
+      <c r="B591" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C591" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D591" s="9" t="n">
+        <v>838</v>
+      </c>
+      <c r="E591" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F591" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G591" s="10" t="inlineStr">
+        <is>
+          <t>39858</t>
+        </is>
+      </c>
+      <c r="H591" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I591" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="592" ht="20" customHeight="1">
+      <c r="A592" s="9" t="n">
+        <v>588</v>
+      </c>
+      <c r="B592" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C592" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D592" s="9" t="n">
+        <v>839</v>
+      </c>
+      <c r="E592" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F592" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G592" s="10" t="inlineStr">
+        <is>
+          <t>39857</t>
+        </is>
+      </c>
+      <c r="H592" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I592" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="593" ht="20" customHeight="1">
+      <c r="A593" s="9" t="n">
+        <v>589</v>
+      </c>
+      <c r="B593" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C593" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D593" s="9" t="n">
+        <v>840</v>
+      </c>
+      <c r="E593" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F593" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G593" s="10" t="inlineStr">
+        <is>
+          <t>39859</t>
+        </is>
+      </c>
+      <c r="H593" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I593" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="20" customHeight="1">
+      <c r="A594" s="9" t="n">
+        <v>590</v>
+      </c>
+      <c r="B594" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C594" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D594" s="9" t="n">
+        <v>841</v>
+      </c>
+      <c r="E594" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F594" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G594" s="10" t="inlineStr">
+        <is>
+          <t>35113</t>
+        </is>
+      </c>
+      <c r="H594" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I594" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="595" ht="20" customHeight="1">
+      <c r="A595" s="9" t="n">
+        <v>591</v>
+      </c>
+      <c r="B595" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C595" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D595" s="9" t="n">
+        <v>842</v>
+      </c>
+      <c r="E595" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F595" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G595" s="10" t="inlineStr">
+        <is>
+          <t>35112</t>
+        </is>
+      </c>
+      <c r="H595" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I595" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="596" ht="20" customHeight="1">
+      <c r="A596" s="9" t="n">
+        <v>592</v>
+      </c>
+      <c r="B596" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C596" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D596" s="9" t="n">
+        <v>843</v>
+      </c>
+      <c r="E596" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F596" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G596" s="10" t="inlineStr">
+        <is>
+          <t>123912</t>
+        </is>
+      </c>
+      <c r="H596" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I596" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="597" ht="20" customHeight="1">
+      <c r="A597" s="9" t="n">
+        <v>593</v>
+      </c>
+      <c r="B597" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C597" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D597" s="9" t="n">
+        <v>844</v>
+      </c>
+      <c r="E597" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F597" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G597" s="10" t="inlineStr">
+        <is>
+          <t>123915</t>
+        </is>
+      </c>
+      <c r="H597" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I597" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="598" ht="20" customHeight="1">
+      <c r="A598" s="9" t="n">
+        <v>594</v>
+      </c>
+      <c r="B598" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C598" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D598" s="9" t="n">
+        <v>845</v>
+      </c>
+      <c r="E598" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F598" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G598" s="10" t="inlineStr">
+        <is>
+          <t>123916</t>
+        </is>
+      </c>
+      <c r="H598" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I598" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="599" ht="20" customHeight="1">
+      <c r="A599" s="9" t="n">
+        <v>595</v>
+      </c>
+      <c r="B599" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C599" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D599" s="9" t="n">
+        <v>846</v>
+      </c>
+      <c r="E599" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F599" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G599" s="10" t="inlineStr">
+        <is>
+          <t>123914</t>
+        </is>
+      </c>
+      <c r="H599" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I599" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="600" ht="20" customHeight="1">
+      <c r="A600" s="9" t="n">
+        <v>596</v>
+      </c>
+      <c r="B600" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C600" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D600" s="9" t="n">
+        <v>847</v>
+      </c>
+      <c r="E600" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F600" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G600" s="10" t="inlineStr">
+        <is>
+          <t>123913</t>
+        </is>
+      </c>
+      <c r="H600" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I600" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="601" ht="20" customHeight="1">
+      <c r="A601" s="9" t="n">
+        <v>597</v>
+      </c>
+      <c r="B601" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C601" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D601" s="9" t="n">
+        <v>848</v>
+      </c>
+      <c r="E601" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F601" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G601" s="10" t="inlineStr">
+        <is>
+          <t>123917</t>
+        </is>
+      </c>
+      <c r="H601" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I601" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="602" ht="20" customHeight="1">
+      <c r="A602" s="9" t="n">
+        <v>598</v>
+      </c>
+      <c r="B602" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C602" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D602" s="9" t="n">
+        <v>849</v>
+      </c>
+      <c r="E602" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F602" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G602" s="10" t="inlineStr">
+        <is>
+          <t>123919</t>
+        </is>
+      </c>
+      <c r="H602" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I602" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="603" ht="20" customHeight="1">
+      <c r="A603" s="9" t="n">
+        <v>599</v>
+      </c>
+      <c r="B603" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C603" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D603" s="9" t="n">
+        <v>850</v>
+      </c>
+      <c r="E603" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F603" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G603" s="10" t="inlineStr">
+        <is>
+          <t>123921</t>
+        </is>
+      </c>
+      <c r="H603" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I603" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="604" ht="20" customHeight="1">
+      <c r="A604" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="B604" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C604" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D604" s="9" t="n">
+        <v>851</v>
+      </c>
+      <c r="E604" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F604" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G604" s="10" t="inlineStr">
+        <is>
+          <t>123918</t>
+        </is>
+      </c>
+      <c r="H604" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I604" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="605" ht="20" customHeight="1">
+      <c r="A605" s="9" t="n">
+        <v>601</v>
+      </c>
+      <c r="B605" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C605" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D605" s="9" t="n">
+        <v>852</v>
+      </c>
+      <c r="E605" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F605" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G605" s="10" t="inlineStr">
+        <is>
+          <t>123920</t>
+        </is>
+      </c>
+      <c r="H605" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I605" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="606" ht="20" customHeight="1">
+      <c r="A606" s="9" t="n">
+        <v>602</v>
+      </c>
+      <c r="B606" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C606" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D606" s="9" t="n">
+        <v>853</v>
+      </c>
+      <c r="E606" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F606" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G606" s="10" t="inlineStr">
+        <is>
+          <t>35117</t>
+        </is>
+      </c>
+      <c r="H606" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I606" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="607" ht="20" customHeight="1">
+      <c r="A607" s="9" t="n">
+        <v>603</v>
+      </c>
+      <c r="B607" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C607" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D607" s="9" t="n">
+        <v>854</v>
+      </c>
+      <c r="E607" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F607" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G607" s="10" t="inlineStr">
+        <is>
+          <t>35114</t>
+        </is>
+      </c>
+      <c r="H607" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I607" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="608" ht="20" customHeight="1">
+      <c r="A608" s="9" t="n">
+        <v>604</v>
+      </c>
+      <c r="B608" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C608" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D608" s="9" t="n">
+        <v>855</v>
+      </c>
+      <c r="E608" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F608" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G608" s="10" t="inlineStr">
+        <is>
+          <t>35116</t>
+        </is>
+      </c>
+      <c r="H608" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I608" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="609" ht="20" customHeight="1">
+      <c r="A609" s="9" t="n">
+        <v>605</v>
+      </c>
+      <c r="B609" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C609" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D609" s="9" t="n">
+        <v>856</v>
+      </c>
+      <c r="E609" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F609" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G609" s="10" t="inlineStr">
+        <is>
+          <t>35115</t>
+        </is>
+      </c>
+      <c r="H609" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I609" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="610" ht="20" customHeight="1">
+      <c r="A610" s="9" t="n">
+        <v>606</v>
+      </c>
+      <c r="B610" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C610" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D610" s="9" t="n">
+        <v>857</v>
+      </c>
+      <c r="E610" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F610" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G610" s="10" t="inlineStr">
+        <is>
+          <t>123888</t>
+        </is>
+      </c>
+      <c r="H610" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I610" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (606 BAL)</t>
+        </is>
+      </c>
+      <c r="B611" s="4" t="n"/>
+      <c r="C611" s="4" t="n"/>
+      <c r="D611" s="4" t="n"/>
+      <c r="E611" s="4" t="n"/>
+      <c r="F611" s="4" t="n"/>
+      <c r="G611" s="4" t="n"/>
+      <c r="H611" s="4">
+        <f>SUM(H5:H610)</f>
         <v/>
       </c>
-      <c r="I562" s="4" t="inlineStr">
+      <c r="I611" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -32463,8 +35256,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A562:G562"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A611:G611"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32476,7 +35269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -33003,37 +35796,66 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>2120</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>43.27</v>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>808 - 857</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4">
-        <f>SUM(D5:D20)</f>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4">
+        <f>SUM(D5:D21)</f>
         <v/>
       </c>
-      <c r="E21" s="4">
-        <f>SUM(E5:E20)</f>
+      <c r="E22" s="4">
+        <f>SUM(E5:E21)</f>
         <v/>
       </c>
-      <c r="F21" s="4">
-        <f>AVERAGE(F5:F20)</f>
+      <c r="F22" s="4">
+        <f>AVERAGE(F5:F21)</f>
         <v/>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>3 - 807</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>3 - 857</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A22:C22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data 8 September 2026 (39 bal): sync Supabase, seed_data, web UI v5.3, dan rekap Excel
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F611"/>
+  <dimension ref="A1:F645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TANGGAL: 21-8 s/d 6-9          HARI: ......................          TAHUN: 2026</t>
+          <t>TANGGAL: 21-8 s/d 8-9          HARI: ......................          TAHUN: 2026</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -12216,47 +12216,47 @@
     </row>
     <row r="587" ht="20.25" customHeight="1">
       <c r="A587" s="5" t="n">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B587" s="5" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C587" s="5" t="n">
         <v>72</v>
       </c>
       <c r="D587" s="6" t="inlineStr">
         <is>
-          <t>39853</t>
+          <t>124372</t>
         </is>
       </c>
       <c r="E587" s="5" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F587" s="5" t="n"/>
     </row>
     <row r="588" ht="20.25" customHeight="1">
       <c r="A588" s="5" t="n">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B588" s="5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C588" s="5" t="n">
         <v>72</v>
       </c>
       <c r="D588" s="6" t="inlineStr">
         <is>
-          <t>39856</t>
+          <t>39853</t>
         </is>
       </c>
       <c r="E588" s="5" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F588" s="5" t="n"/>
     </row>
     <row r="589" ht="20.25" customHeight="1">
       <c r="A589" s="5" t="n">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B589" s="5" t="n">
         <v>72</v>
@@ -12266,7 +12266,7 @@
       </c>
       <c r="D589" s="6" t="inlineStr">
         <is>
-          <t>39854</t>
+          <t>39856</t>
         </is>
       </c>
       <c r="E589" s="5" t="n">
@@ -12276,7 +12276,7 @@
     </row>
     <row r="590" ht="20.25" customHeight="1">
       <c r="A590" s="5" t="n">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B590" s="5" t="n">
         <v>72</v>
@@ -12286,7 +12286,7 @@
       </c>
       <c r="D590" s="6" t="inlineStr">
         <is>
-          <t>39855</t>
+          <t>39854</t>
         </is>
       </c>
       <c r="E590" s="5" t="n">
@@ -12296,47 +12296,47 @@
     </row>
     <row r="591" ht="20.25" customHeight="1">
       <c r="A591" s="5" t="n">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B591" s="5" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C591" s="5" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D591" s="6" t="inlineStr">
         <is>
-          <t>39858</t>
+          <t>39855</t>
         </is>
       </c>
       <c r="E591" s="5" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F591" s="5" t="n"/>
     </row>
     <row r="592" ht="20.25" customHeight="1">
       <c r="A592" s="5" t="n">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B592" s="5" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C592" s="5" t="n">
         <v>68</v>
       </c>
       <c r="D592" s="6" t="inlineStr">
         <is>
-          <t>39857</t>
+          <t>39858</t>
         </is>
       </c>
       <c r="E592" s="5" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F592" s="5" t="n"/>
     </row>
     <row r="593" ht="20.25" customHeight="1">
       <c r="A593" s="5" t="n">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B593" s="5" t="n">
         <v>70</v>
@@ -12346,67 +12346,67 @@
       </c>
       <c r="D593" s="6" t="inlineStr">
         <is>
-          <t>39859</t>
+          <t>39857</t>
         </is>
       </c>
       <c r="E593" s="5" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F593" s="5" t="n"/>
     </row>
     <row r="594" ht="20.25" customHeight="1">
       <c r="A594" s="5" t="n">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B594" s="5" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C594" s="5" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="D594" s="6" t="inlineStr">
         <is>
-          <t>35113</t>
+          <t>39859</t>
         </is>
       </c>
       <c r="E594" s="5" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F594" s="5" t="n"/>
     </row>
     <row r="595" ht="20.25" customHeight="1">
       <c r="A595" s="5" t="n">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B595" s="5" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C595" s="5" t="n">
         <v>55</v>
       </c>
       <c r="D595" s="6" t="inlineStr">
         <is>
-          <t>35112</t>
+          <t>35113</t>
         </is>
       </c>
       <c r="E595" s="5" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="F595" s="5" t="n"/>
     </row>
     <row r="596" ht="20.25" customHeight="1">
       <c r="A596" s="5" t="n">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B596" s="5" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C596" s="5" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D596" s="6" t="inlineStr">
         <is>
-          <t>123912</t>
+          <t>35112</t>
         </is>
       </c>
       <c r="E596" s="5" t="n">
@@ -12416,37 +12416,37 @@
     </row>
     <row r="597" ht="20.25" customHeight="1">
       <c r="A597" s="5" t="n">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B597" s="5" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C597" s="5" t="n">
         <v>58</v>
       </c>
       <c r="D597" s="6" t="inlineStr">
         <is>
-          <t>123915</t>
+          <t>123912</t>
         </is>
       </c>
       <c r="E597" s="5" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F597" s="5" t="n"/>
     </row>
     <row r="598" ht="20.25" customHeight="1">
       <c r="A598" s="5" t="n">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B598" s="5" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C598" s="5" t="n">
         <v>58</v>
       </c>
       <c r="D598" s="6" t="inlineStr">
         <is>
-          <t>123916</t>
+          <t>123915</t>
         </is>
       </c>
       <c r="E598" s="5" t="n">
@@ -12456,7 +12456,7 @@
     </row>
     <row r="599" ht="20.25" customHeight="1">
       <c r="A599" s="5" t="n">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B599" s="5" t="n">
         <v>60</v>
@@ -12466,7 +12466,7 @@
       </c>
       <c r="D599" s="6" t="inlineStr">
         <is>
-          <t>123914</t>
+          <t>123916</t>
         </is>
       </c>
       <c r="E599" s="5" t="n">
@@ -12476,7 +12476,7 @@
     </row>
     <row r="600" ht="20.25" customHeight="1">
       <c r="A600" s="5" t="n">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B600" s="5" t="n">
         <v>60</v>
@@ -12486,17 +12486,17 @@
       </c>
       <c r="D600" s="6" t="inlineStr">
         <is>
-          <t>123913</t>
+          <t>123914</t>
         </is>
       </c>
       <c r="E600" s="5" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F600" s="5" t="n"/>
     </row>
     <row r="601" ht="20.25" customHeight="1">
       <c r="A601" s="5" t="n">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B601" s="5" t="n">
         <v>60</v>
@@ -12506,67 +12506,67 @@
       </c>
       <c r="D601" s="6" t="inlineStr">
         <is>
-          <t>123917</t>
+          <t>123913</t>
         </is>
       </c>
       <c r="E601" s="5" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F601" s="5" t="n"/>
     </row>
     <row r="602" ht="20.25" customHeight="1">
       <c r="A602" s="5" t="n">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B602" s="5" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C602" s="5" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D602" s="6" t="inlineStr">
         <is>
-          <t>123919</t>
+          <t>123917</t>
         </is>
       </c>
       <c r="E602" s="5" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F602" s="5" t="n"/>
     </row>
     <row r="603" ht="20.25" customHeight="1">
       <c r="A603" s="5" t="n">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B603" s="5" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C603" s="5" t="n">
         <v>56</v>
       </c>
       <c r="D603" s="6" t="inlineStr">
         <is>
-          <t>123921</t>
+          <t>123919</t>
         </is>
       </c>
       <c r="E603" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F603" s="5" t="n"/>
     </row>
     <row r="604" ht="20.25" customHeight="1">
       <c r="A604" s="5" t="n">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B604" s="5" t="n">
         <v>57</v>
       </c>
       <c r="C604" s="5" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D604" s="6" t="inlineStr">
         <is>
-          <t>123918</t>
+          <t>123921</t>
         </is>
       </c>
       <c r="E604" s="5" t="n">
@@ -12576,47 +12576,47 @@
     </row>
     <row r="605" ht="20.25" customHeight="1">
       <c r="A605" s="5" t="n">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B605" s="5" t="n">
         <v>57</v>
       </c>
       <c r="C605" s="5" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D605" s="6" t="inlineStr">
         <is>
-          <t>123920</t>
+          <t>123918</t>
         </is>
       </c>
       <c r="E605" s="5" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F605" s="5" t="n"/>
     </row>
     <row r="606" ht="20.25" customHeight="1">
       <c r="A606" s="5" t="n">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B606" s="5" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C606" s="5" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D606" s="6" t="inlineStr">
         <is>
-          <t>35117</t>
+          <t>123920</t>
         </is>
       </c>
       <c r="E606" s="5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F606" s="5" t="n"/>
     </row>
     <row r="607" ht="20.25" customHeight="1">
       <c r="A607" s="5" t="n">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B607" s="5" t="n">
         <v>52</v>
@@ -12626,17 +12626,17 @@
       </c>
       <c r="D607" s="6" t="inlineStr">
         <is>
-          <t>35114</t>
+          <t>35117</t>
         </is>
       </c>
       <c r="E607" s="5" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F607" s="5" t="n"/>
     </row>
     <row r="608" ht="20.25" customHeight="1">
       <c r="A608" s="5" t="n">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B608" s="5" t="n">
         <v>52</v>
@@ -12646,17 +12646,17 @@
       </c>
       <c r="D608" s="6" t="inlineStr">
         <is>
-          <t>35116</t>
+          <t>35114</t>
         </is>
       </c>
       <c r="E608" s="5" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F608" s="5" t="n"/>
     </row>
     <row r="609" ht="20.25" customHeight="1">
       <c r="A609" s="5" t="n">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B609" s="5" t="n">
         <v>52</v>
@@ -12666,7 +12666,7 @@
       </c>
       <c r="D609" s="6" t="inlineStr">
         <is>
-          <t>35115</t>
+          <t>35116</t>
         </is>
       </c>
       <c r="E609" s="5" t="n">
@@ -12676,38 +12676,718 @@
     </row>
     <row r="610" ht="20.25" customHeight="1">
       <c r="A610" s="5" t="n">
+        <v>856</v>
+      </c>
+      <c r="B610" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="C610" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D610" s="6" t="inlineStr">
+        <is>
+          <t>35115</t>
+        </is>
+      </c>
+      <c r="E610" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F610" s="5" t="n"/>
+    </row>
+    <row r="611" ht="20.25" customHeight="1">
+      <c r="A611" s="5" t="n">
         <v>857</v>
       </c>
-      <c r="B610" s="5" t="n">
+      <c r="B611" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="C610" s="5" t="n">
+      <c r="C611" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="D610" s="6" t="inlineStr">
+      <c r="D611" s="6" t="inlineStr">
         <is>
           <t>123888</t>
         </is>
       </c>
-      <c r="E610" s="5" t="n">
+      <c r="E611" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="F610" s="5" t="n"/>
-    </row>
-    <row r="611" ht="22" customHeight="1">
-      <c r="A611" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (606 BAL)</t>
-        </is>
-      </c>
-      <c r="B611" s="4" t="n"/>
-      <c r="C611" s="4" t="n"/>
-      <c r="D611" s="4" t="n"/>
-      <c r="E611" s="4">
-        <f>SUM(E5:E610)</f>
+      <c r="F611" s="5" t="n"/>
+    </row>
+    <row r="612" ht="20.25" customHeight="1">
+      <c r="A612" s="5" t="n">
+        <v>858</v>
+      </c>
+      <c r="B612" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C612" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D612" s="6" t="inlineStr">
+        <is>
+          <t>124373</t>
+        </is>
+      </c>
+      <c r="E612" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F612" s="5" t="n"/>
+    </row>
+    <row r="613" ht="20.25" customHeight="1">
+      <c r="A613" s="5" t="n">
+        <v>860</v>
+      </c>
+      <c r="B613" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C613" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D613" s="6" t="inlineStr">
+        <is>
+          <t>124284</t>
+        </is>
+      </c>
+      <c r="E613" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F613" s="5" t="n"/>
+    </row>
+    <row r="614" ht="20.25" customHeight="1">
+      <c r="A614" s="5" t="n">
+        <v>861</v>
+      </c>
+      <c r="B614" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C614" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D614" s="6" t="inlineStr">
+        <is>
+          <t>124367</t>
+        </is>
+      </c>
+      <c r="E614" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F614" s="5" t="n"/>
+    </row>
+    <row r="615" ht="20.25" customHeight="1">
+      <c r="A615" s="5" t="n">
+        <v>862</v>
+      </c>
+      <c r="B615" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C615" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D615" s="6" t="inlineStr">
+        <is>
+          <t>124368</t>
+        </is>
+      </c>
+      <c r="E615" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F615" s="5" t="n"/>
+    </row>
+    <row r="616" ht="20.25" customHeight="1">
+      <c r="A616" s="5" t="n">
+        <v>863</v>
+      </c>
+      <c r="B616" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C616" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D616" s="6" t="inlineStr">
+        <is>
+          <t>124370</t>
+        </is>
+      </c>
+      <c r="E616" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F616" s="5" t="n"/>
+    </row>
+    <row r="617" ht="20.25" customHeight="1">
+      <c r="A617" s="5" t="n">
+        <v>866</v>
+      </c>
+      <c r="B617" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C617" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D617" s="6" t="inlineStr">
+        <is>
+          <t>124371</t>
+        </is>
+      </c>
+      <c r="E617" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F617" s="5" t="n"/>
+    </row>
+    <row r="618" ht="20.25" customHeight="1">
+      <c r="A618" s="5" t="n">
+        <v>868</v>
+      </c>
+      <c r="B618" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C618" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D618" s="6" t="inlineStr">
+        <is>
+          <t>124369</t>
+        </is>
+      </c>
+      <c r="E618" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F618" s="5" t="n"/>
+    </row>
+    <row r="619" ht="20.25" customHeight="1">
+      <c r="A619" s="5" t="n">
+        <v>869</v>
+      </c>
+      <c r="B619" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C619" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D619" s="6" t="inlineStr">
+        <is>
+          <t>124285</t>
+        </is>
+      </c>
+      <c r="E619" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F619" s="5" t="n"/>
+    </row>
+    <row r="620" ht="20.25" customHeight="1">
+      <c r="A620" s="5" t="n">
+        <v>870</v>
+      </c>
+      <c r="B620" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C620" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D620" s="6" t="inlineStr">
+        <is>
+          <t>39833</t>
+        </is>
+      </c>
+      <c r="E620" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F620" s="5" t="n"/>
+    </row>
+    <row r="621" ht="20.25" customHeight="1">
+      <c r="A621" s="5" t="n">
+        <v>872</v>
+      </c>
+      <c r="B621" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C621" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D621" s="6" t="inlineStr">
+        <is>
+          <t>124366</t>
+        </is>
+      </c>
+      <c r="E621" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F621" s="5" t="n"/>
+    </row>
+    <row r="622" ht="20.25" customHeight="1">
+      <c r="A622" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="B622" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C622" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="D622" s="6" t="inlineStr">
+        <is>
+          <t>33879</t>
+        </is>
+      </c>
+      <c r="E622" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F622" s="5" t="n"/>
+    </row>
+    <row r="623" ht="20.25" customHeight="1">
+      <c r="A623" s="5" t="n">
+        <v>874</v>
+      </c>
+      <c r="B623" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C623" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D623" s="6" t="inlineStr">
+        <is>
+          <t>123934</t>
+        </is>
+      </c>
+      <c r="E623" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F623" s="5" t="n"/>
+    </row>
+    <row r="624" ht="20.25" customHeight="1">
+      <c r="A624" s="5" t="n">
+        <v>875</v>
+      </c>
+      <c r="B624" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C624" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D624" s="6" t="inlineStr">
+        <is>
+          <t>123935</t>
+        </is>
+      </c>
+      <c r="E624" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F624" s="5" t="n"/>
+    </row>
+    <row r="625" ht="20.25" customHeight="1">
+      <c r="A625" s="5" t="n">
+        <v>876</v>
+      </c>
+      <c r="B625" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C625" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D625" s="6" t="inlineStr">
+        <is>
+          <t>123933</t>
+        </is>
+      </c>
+      <c r="E625" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F625" s="5" t="n"/>
+    </row>
+    <row r="626" ht="20.25" customHeight="1">
+      <c r="A626" s="5" t="n">
+        <v>877</v>
+      </c>
+      <c r="B626" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C626" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D626" s="6" t="inlineStr">
+        <is>
+          <t>123944</t>
+        </is>
+      </c>
+      <c r="E626" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F626" s="5" t="n"/>
+    </row>
+    <row r="627" ht="20.25" customHeight="1">
+      <c r="A627" s="5" t="n">
+        <v>878</v>
+      </c>
+      <c r="B627" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C627" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D627" s="6" t="inlineStr">
+        <is>
+          <t>123932</t>
+        </is>
+      </c>
+      <c r="E627" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F627" s="5" t="n"/>
+    </row>
+    <row r="628" ht="20.25" customHeight="1">
+      <c r="A628" s="5" t="n">
+        <v>879</v>
+      </c>
+      <c r="B628" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C628" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D628" s="6" t="inlineStr">
+        <is>
+          <t>123929</t>
+        </is>
+      </c>
+      <c r="E628" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F628" s="5" t="n"/>
+    </row>
+    <row r="629" ht="20.25" customHeight="1">
+      <c r="A629" s="5" t="n">
+        <v>880</v>
+      </c>
+      <c r="B629" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C629" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D629" s="6" t="inlineStr">
+        <is>
+          <t>123931</t>
+        </is>
+      </c>
+      <c r="E629" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F629" s="5" t="n"/>
+    </row>
+    <row r="630" ht="20.25" customHeight="1">
+      <c r="A630" s="5" t="n">
+        <v>881</v>
+      </c>
+      <c r="B630" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C630" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D630" s="6" t="inlineStr">
+        <is>
+          <t>123930</t>
+        </is>
+      </c>
+      <c r="E630" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F630" s="5" t="n"/>
+    </row>
+    <row r="631" ht="20.25" customHeight="1">
+      <c r="A631" s="5" t="n">
+        <v>882</v>
+      </c>
+      <c r="B631" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C631" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D631" s="6" t="inlineStr">
+        <is>
+          <t>123941</t>
+        </is>
+      </c>
+      <c r="E631" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F631" s="5" t="n"/>
+    </row>
+    <row r="632" ht="20.25" customHeight="1">
+      <c r="A632" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="B632" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C632" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D632" s="6" t="inlineStr">
+        <is>
+          <t>124227</t>
+        </is>
+      </c>
+      <c r="E632" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F632" s="5" t="n"/>
+    </row>
+    <row r="633" ht="20.25" customHeight="1">
+      <c r="A633" s="5" t="n">
+        <v>884</v>
+      </c>
+      <c r="B633" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C633" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D633" s="6" t="inlineStr">
+        <is>
+          <t>123940</t>
+        </is>
+      </c>
+      <c r="E633" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F633" s="5" t="n"/>
+    </row>
+    <row r="634" ht="20.25" customHeight="1">
+      <c r="A634" s="5" t="n">
+        <v>885</v>
+      </c>
+      <c r="B634" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C634" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D634" s="6" t="inlineStr">
+        <is>
+          <t>123943</t>
+        </is>
+      </c>
+      <c r="E634" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F634" s="5" t="n"/>
+    </row>
+    <row r="635" ht="20.25" customHeight="1">
+      <c r="A635" s="5" t="n">
+        <v>886</v>
+      </c>
+      <c r="B635" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C635" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D635" s="6" t="inlineStr">
+        <is>
+          <t>123942</t>
+        </is>
+      </c>
+      <c r="E635" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F635" s="5" t="n"/>
+    </row>
+    <row r="636" ht="20.25" customHeight="1">
+      <c r="A636" s="5" t="n">
+        <v>887</v>
+      </c>
+      <c r="B636" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C636" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D636" s="6" t="inlineStr">
+        <is>
+          <t>123937</t>
+        </is>
+      </c>
+      <c r="E636" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F636" s="5" t="n"/>
+    </row>
+    <row r="637" ht="20.25" customHeight="1">
+      <c r="A637" s="5" t="n">
+        <v>888</v>
+      </c>
+      <c r="B637" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C637" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D637" s="6" t="inlineStr">
+        <is>
+          <t>33883</t>
+        </is>
+      </c>
+      <c r="E637" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F637" s="5" t="n"/>
+    </row>
+    <row r="638" ht="20.25" customHeight="1">
+      <c r="A638" s="5" t="n">
+        <v>889</v>
+      </c>
+      <c r="B638" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C638" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D638" s="6" t="inlineStr">
+        <is>
+          <t>123936</t>
+        </is>
+      </c>
+      <c r="E638" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F638" s="5" t="n"/>
+    </row>
+    <row r="639" ht="20.25" customHeight="1">
+      <c r="A639" s="5" t="n">
+        <v>890</v>
+      </c>
+      <c r="B639" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C639" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D639" s="6" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="E639" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F639" s="5" t="n"/>
+    </row>
+    <row r="640" ht="20.25" customHeight="1">
+      <c r="A640" s="5" t="n">
+        <v>891</v>
+      </c>
+      <c r="B640" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C640" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D640" s="6" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="E640" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F640" s="5" t="n"/>
+    </row>
+    <row r="641" ht="20.25" customHeight="1">
+      <c r="A641" s="5" t="n">
+        <v>892</v>
+      </c>
+      <c r="B641" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="C641" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D641" s="6" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="E641" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F641" s="5" t="n"/>
+    </row>
+    <row r="642" ht="20.25" customHeight="1">
+      <c r="A642" s="5" t="n">
+        <v>893</v>
+      </c>
+      <c r="B642" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="C642" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D642" s="6" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="E642" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F642" s="5" t="n"/>
+    </row>
+    <row r="643" ht="20.25" customHeight="1">
+      <c r="A643" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="B643" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="C643" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D643" s="6" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="E643" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F643" s="5" t="n"/>
+    </row>
+    <row r="644" ht="20.25" customHeight="1">
+      <c r="A644" s="5" t="n">
+        <v>895</v>
+      </c>
+      <c r="B644" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="C644" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D644" s="6" t="inlineStr">
+        <is>
+          <t>33882</t>
+        </is>
+      </c>
+      <c r="E644" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F644" s="5" t="n"/>
+    </row>
+    <row r="645" ht="22" customHeight="1">
+      <c r="A645" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (640 BAL)</t>
+        </is>
+      </c>
+      <c r="B645" s="4" t="n"/>
+      <c r="C645" s="4" t="n"/>
+      <c r="D645" s="4" t="n"/>
+      <c r="E645" s="4">
+        <f>SUM(E5:E644)</f>
         <v/>
       </c>
-      <c r="F611" s="4" t="inlineStr">
+      <c r="F645" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -12716,10 +13396,10 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A611:D611"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="A645:D645"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -12734,7 +13414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I611"/>
+  <dimension ref="A1:I645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12751,14 +13431,14 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 6 SEPTEMBER 2026)</t>
+          <t>REKAP DATA BAL DENGAN BARKOT (21 AGUSTUS - 8 SEPTEMBER 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 606 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 640 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -34349,34 +35029,34 @@
       </c>
       <c r="B587" s="9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C587" s="9" t="inlineStr">
         <is>
-          <t>SENIN</t>
+          <t>SELASA</t>
         </is>
       </c>
       <c r="D587" s="9" t="n">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="E587" s="9" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F587" s="9" t="n">
         <v>72</v>
       </c>
       <c r="G587" s="10" t="inlineStr">
         <is>
-          <t>39853</t>
+          <t>124372</t>
         </is>
       </c>
       <c r="H587" s="9" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I587" s="11" t="inlineStr">
         <is>
-          <t>grade 7 september.xlsx</t>
+          <t>grade 8 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -34395,21 +35075,21 @@
         </is>
       </c>
       <c r="D588" s="9" t="n">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E588" s="9" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F588" s="9" t="n">
         <v>72</v>
       </c>
       <c r="G588" s="10" t="inlineStr">
         <is>
-          <t>39856</t>
+          <t>39853</t>
         </is>
       </c>
       <c r="H588" s="9" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I588" s="11" t="inlineStr">
         <is>
@@ -34432,7 +35112,7 @@
         </is>
       </c>
       <c r="D589" s="9" t="n">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E589" s="9" t="n">
         <v>72</v>
@@ -34442,7 +35122,7 @@
       </c>
       <c r="G589" s="10" t="inlineStr">
         <is>
-          <t>39854</t>
+          <t>39856</t>
         </is>
       </c>
       <c r="H589" s="9" t="n">
@@ -34469,7 +35149,7 @@
         </is>
       </c>
       <c r="D590" s="9" t="n">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E590" s="9" t="n">
         <v>72</v>
@@ -34479,7 +35159,7 @@
       </c>
       <c r="G590" s="10" t="inlineStr">
         <is>
-          <t>39855</t>
+          <t>39854</t>
         </is>
       </c>
       <c r="H590" s="9" t="n">
@@ -34506,21 +35186,21 @@
         </is>
       </c>
       <c r="D591" s="9" t="n">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="E591" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F591" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G591" s="10" t="inlineStr">
         <is>
-          <t>39858</t>
+          <t>39855</t>
         </is>
       </c>
       <c r="H591" s="9" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I591" s="11" t="inlineStr">
         <is>
@@ -34543,21 +35223,21 @@
         </is>
       </c>
       <c r="D592" s="9" t="n">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="E592" s="9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F592" s="9" t="n">
         <v>68</v>
       </c>
       <c r="G592" s="10" t="inlineStr">
         <is>
-          <t>39857</t>
+          <t>39858</t>
         </is>
       </c>
       <c r="H592" s="9" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I592" s="11" t="inlineStr">
         <is>
@@ -34580,7 +35260,7 @@
         </is>
       </c>
       <c r="D593" s="9" t="n">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E593" s="9" t="n">
         <v>70</v>
@@ -34590,11 +35270,11 @@
       </c>
       <c r="G593" s="10" t="inlineStr">
         <is>
-          <t>39859</t>
+          <t>39857</t>
         </is>
       </c>
       <c r="H593" s="9" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I593" s="11" t="inlineStr">
         <is>
@@ -34617,21 +35297,21 @@
         </is>
       </c>
       <c r="D594" s="9" t="n">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E594" s="9" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="F594" s="9" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G594" s="10" t="inlineStr">
         <is>
-          <t>35113</t>
+          <t>39859</t>
         </is>
       </c>
       <c r="H594" s="9" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I594" s="11" t="inlineStr">
         <is>
@@ -34654,21 +35334,21 @@
         </is>
       </c>
       <c r="D595" s="9" t="n">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="E595" s="9" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F595" s="9" t="n">
         <v>55</v>
       </c>
       <c r="G595" s="10" t="inlineStr">
         <is>
-          <t>35112</t>
+          <t>35113</t>
         </is>
       </c>
       <c r="H595" s="9" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="I595" s="11" t="inlineStr">
         <is>
@@ -34691,17 +35371,17 @@
         </is>
       </c>
       <c r="D596" s="9" t="n">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="E596" s="9" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F596" s="9" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G596" s="10" t="inlineStr">
         <is>
-          <t>123912</t>
+          <t>35112</t>
         </is>
       </c>
       <c r="H596" s="9" t="n">
@@ -34728,21 +35408,21 @@
         </is>
       </c>
       <c r="D597" s="9" t="n">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E597" s="9" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F597" s="9" t="n">
         <v>58</v>
       </c>
       <c r="G597" s="10" t="inlineStr">
         <is>
-          <t>123915</t>
+          <t>123912</t>
         </is>
       </c>
       <c r="H597" s="9" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I597" s="11" t="inlineStr">
         <is>
@@ -34765,17 +35445,17 @@
         </is>
       </c>
       <c r="D598" s="9" t="n">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="E598" s="9" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F598" s="9" t="n">
         <v>58</v>
       </c>
       <c r="G598" s="10" t="inlineStr">
         <is>
-          <t>123916</t>
+          <t>123915</t>
         </is>
       </c>
       <c r="H598" s="9" t="n">
@@ -34802,7 +35482,7 @@
         </is>
       </c>
       <c r="D599" s="9" t="n">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E599" s="9" t="n">
         <v>60</v>
@@ -34812,7 +35492,7 @@
       </c>
       <c r="G599" s="10" t="inlineStr">
         <is>
-          <t>123914</t>
+          <t>123916</t>
         </is>
       </c>
       <c r="H599" s="9" t="n">
@@ -34839,7 +35519,7 @@
         </is>
       </c>
       <c r="D600" s="9" t="n">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E600" s="9" t="n">
         <v>60</v>
@@ -34849,11 +35529,11 @@
       </c>
       <c r="G600" s="10" t="inlineStr">
         <is>
-          <t>123913</t>
+          <t>123914</t>
         </is>
       </c>
       <c r="H600" s="9" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I600" s="11" t="inlineStr">
         <is>
@@ -34876,7 +35556,7 @@
         </is>
       </c>
       <c r="D601" s="9" t="n">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E601" s="9" t="n">
         <v>60</v>
@@ -34886,11 +35566,11 @@
       </c>
       <c r="G601" s="10" t="inlineStr">
         <is>
-          <t>123917</t>
+          <t>123913</t>
         </is>
       </c>
       <c r="H601" s="9" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I601" s="11" t="inlineStr">
         <is>
@@ -34913,21 +35593,21 @@
         </is>
       </c>
       <c r="D602" s="9" t="n">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="E602" s="9" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F602" s="9" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G602" s="10" t="inlineStr">
         <is>
-          <t>123919</t>
+          <t>123917</t>
         </is>
       </c>
       <c r="H602" s="9" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I602" s="11" t="inlineStr">
         <is>
@@ -34950,21 +35630,21 @@
         </is>
       </c>
       <c r="D603" s="9" t="n">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="E603" s="9" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F603" s="9" t="n">
         <v>56</v>
       </c>
       <c r="G603" s="10" t="inlineStr">
         <is>
-          <t>123921</t>
+          <t>123919</t>
         </is>
       </c>
       <c r="H603" s="9" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I603" s="11" t="inlineStr">
         <is>
@@ -34987,17 +35667,17 @@
         </is>
       </c>
       <c r="D604" s="9" t="n">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="E604" s="9" t="n">
         <v>57</v>
       </c>
       <c r="F604" s="9" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G604" s="10" t="inlineStr">
         <is>
-          <t>123918</t>
+          <t>123921</t>
         </is>
       </c>
       <c r="H604" s="9" t="n">
@@ -35024,21 +35704,21 @@
         </is>
       </c>
       <c r="D605" s="9" t="n">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="E605" s="9" t="n">
         <v>57</v>
       </c>
       <c r="F605" s="9" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G605" s="10" t="inlineStr">
         <is>
-          <t>123920</t>
+          <t>123918</t>
         </is>
       </c>
       <c r="H605" s="9" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I605" s="11" t="inlineStr">
         <is>
@@ -35061,21 +35741,21 @@
         </is>
       </c>
       <c r="D606" s="9" t="n">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E606" s="9" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F606" s="9" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="G606" s="10" t="inlineStr">
         <is>
-          <t>35117</t>
+          <t>123920</t>
         </is>
       </c>
       <c r="H606" s="9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I606" s="11" t="inlineStr">
         <is>
@@ -35098,7 +35778,7 @@
         </is>
       </c>
       <c r="D607" s="9" t="n">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E607" s="9" t="n">
         <v>52</v>
@@ -35108,11 +35788,11 @@
       </c>
       <c r="G607" s="10" t="inlineStr">
         <is>
-          <t>35114</t>
+          <t>35117</t>
         </is>
       </c>
       <c r="H607" s="9" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I607" s="11" t="inlineStr">
         <is>
@@ -35135,7 +35815,7 @@
         </is>
       </c>
       <c r="D608" s="9" t="n">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="E608" s="9" t="n">
         <v>52</v>
@@ -35145,11 +35825,11 @@
       </c>
       <c r="G608" s="10" t="inlineStr">
         <is>
-          <t>35116</t>
+          <t>35114</t>
         </is>
       </c>
       <c r="H608" s="9" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I608" s="11" t="inlineStr">
         <is>
@@ -35172,7 +35852,7 @@
         </is>
       </c>
       <c r="D609" s="9" t="n">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E609" s="9" t="n">
         <v>52</v>
@@ -35182,7 +35862,7 @@
       </c>
       <c r="G609" s="10" t="inlineStr">
         <is>
-          <t>35115</t>
+          <t>35116</t>
         </is>
       </c>
       <c r="H609" s="9" t="n">
@@ -35209,45 +35889,1303 @@
         </is>
       </c>
       <c r="D610" s="9" t="n">
+        <v>856</v>
+      </c>
+      <c r="E610" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F610" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G610" s="10" t="inlineStr">
+        <is>
+          <t>35115</t>
+        </is>
+      </c>
+      <c r="H610" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I610" s="11" t="inlineStr">
+        <is>
+          <t>grade 7 september.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="611" ht="20" customHeight="1">
+      <c r="A611" s="9" t="n">
+        <v>607</v>
+      </c>
+      <c r="B611" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C611" s="9" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D611" s="9" t="n">
         <v>857</v>
       </c>
-      <c r="E610" s="9" t="n">
+      <c r="E611" s="9" t="n">
         <v>68</v>
       </c>
-      <c r="F610" s="9" t="n">
+      <c r="F611" s="9" t="n">
         <v>66</v>
       </c>
-      <c r="G610" s="10" t="inlineStr">
+      <c r="G611" s="10" t="inlineStr">
         <is>
           <t>123888</t>
         </is>
       </c>
-      <c r="H610" s="9" t="n">
+      <c r="H611" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="I610" s="11" t="inlineStr">
+      <c r="I611" s="11" t="inlineStr">
         <is>
           <t>grade 7 september.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="611">
-      <c r="A611" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (606 BAL)</t>
-        </is>
-      </c>
-      <c r="B611" s="4" t="n"/>
-      <c r="C611" s="4" t="n"/>
-      <c r="D611" s="4" t="n"/>
-      <c r="E611" s="4" t="n"/>
-      <c r="F611" s="4" t="n"/>
-      <c r="G611" s="4" t="n"/>
-      <c r="H611" s="4">
-        <f>SUM(H5:H610)</f>
+    <row r="612" ht="20" customHeight="1">
+      <c r="A612" s="9" t="n">
+        <v>608</v>
+      </c>
+      <c r="B612" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C612" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D612" s="9" t="n">
+        <v>858</v>
+      </c>
+      <c r="E612" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F612" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G612" s="10" t="inlineStr">
+        <is>
+          <t>124373</t>
+        </is>
+      </c>
+      <c r="H612" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I612" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="613" ht="20" customHeight="1">
+      <c r="A613" s="9" t="n">
+        <v>609</v>
+      </c>
+      <c r="B613" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C613" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D613" s="9" t="n">
+        <v>860</v>
+      </c>
+      <c r="E613" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F613" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G613" s="10" t="inlineStr">
+        <is>
+          <t>124284</t>
+        </is>
+      </c>
+      <c r="H613" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I613" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="614" ht="20" customHeight="1">
+      <c r="A614" s="9" t="n">
+        <v>610</v>
+      </c>
+      <c r="B614" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C614" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D614" s="9" t="n">
+        <v>861</v>
+      </c>
+      <c r="E614" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F614" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G614" s="10" t="inlineStr">
+        <is>
+          <t>124367</t>
+        </is>
+      </c>
+      <c r="H614" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I614" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="615" ht="20" customHeight="1">
+      <c r="A615" s="9" t="n">
+        <v>611</v>
+      </c>
+      <c r="B615" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C615" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D615" s="9" t="n">
+        <v>862</v>
+      </c>
+      <c r="E615" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F615" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G615" s="10" t="inlineStr">
+        <is>
+          <t>124368</t>
+        </is>
+      </c>
+      <c r="H615" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I615" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="616" ht="20" customHeight="1">
+      <c r="A616" s="9" t="n">
+        <v>612</v>
+      </c>
+      <c r="B616" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C616" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D616" s="9" t="n">
+        <v>863</v>
+      </c>
+      <c r="E616" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F616" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G616" s="10" t="inlineStr">
+        <is>
+          <t>124370</t>
+        </is>
+      </c>
+      <c r="H616" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I616" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="617" ht="20" customHeight="1">
+      <c r="A617" s="9" t="n">
+        <v>613</v>
+      </c>
+      <c r="B617" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C617" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D617" s="9" t="n">
+        <v>866</v>
+      </c>
+      <c r="E617" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F617" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G617" s="10" t="inlineStr">
+        <is>
+          <t>124371</t>
+        </is>
+      </c>
+      <c r="H617" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I617" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="618" ht="20" customHeight="1">
+      <c r="A618" s="9" t="n">
+        <v>614</v>
+      </c>
+      <c r="B618" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C618" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D618" s="9" t="n">
+        <v>868</v>
+      </c>
+      <c r="E618" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F618" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G618" s="10" t="inlineStr">
+        <is>
+          <t>124369</t>
+        </is>
+      </c>
+      <c r="H618" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I618" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="619" ht="20" customHeight="1">
+      <c r="A619" s="9" t="n">
+        <v>615</v>
+      </c>
+      <c r="B619" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C619" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D619" s="9" t="n">
+        <v>869</v>
+      </c>
+      <c r="E619" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F619" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G619" s="10" t="inlineStr">
+        <is>
+          <t>124285</t>
+        </is>
+      </c>
+      <c r="H619" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I619" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="620" ht="20" customHeight="1">
+      <c r="A620" s="9" t="n">
+        <v>616</v>
+      </c>
+      <c r="B620" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C620" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D620" s="9" t="n">
+        <v>870</v>
+      </c>
+      <c r="E620" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F620" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G620" s="10" t="inlineStr">
+        <is>
+          <t>39833</t>
+        </is>
+      </c>
+      <c r="H620" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I620" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="621" ht="20" customHeight="1">
+      <c r="A621" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="B621" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C621" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D621" s="9" t="n">
+        <v>872</v>
+      </c>
+      <c r="E621" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F621" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G621" s="10" t="inlineStr">
+        <is>
+          <t>124366</t>
+        </is>
+      </c>
+      <c r="H621" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I621" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="622" ht="20" customHeight="1">
+      <c r="A622" s="9" t="n">
+        <v>618</v>
+      </c>
+      <c r="B622" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C622" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D622" s="9" t="n">
+        <v>873</v>
+      </c>
+      <c r="E622" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F622" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="G622" s="10" t="inlineStr">
+        <is>
+          <t>33879</t>
+        </is>
+      </c>
+      <c r="H622" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I622" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="623" ht="20" customHeight="1">
+      <c r="A623" s="9" t="n">
+        <v>619</v>
+      </c>
+      <c r="B623" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C623" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D623" s="9" t="n">
+        <v>874</v>
+      </c>
+      <c r="E623" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F623" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G623" s="10" t="inlineStr">
+        <is>
+          <t>123934</t>
+        </is>
+      </c>
+      <c r="H623" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I623" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="624" ht="20" customHeight="1">
+      <c r="A624" s="9" t="n">
+        <v>620</v>
+      </c>
+      <c r="B624" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C624" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D624" s="9" t="n">
+        <v>875</v>
+      </c>
+      <c r="E624" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F624" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G624" s="10" t="inlineStr">
+        <is>
+          <t>123935</t>
+        </is>
+      </c>
+      <c r="H624" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I624" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="625" ht="20" customHeight="1">
+      <c r="A625" s="9" t="n">
+        <v>621</v>
+      </c>
+      <c r="B625" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C625" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D625" s="9" t="n">
+        <v>876</v>
+      </c>
+      <c r="E625" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F625" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G625" s="10" t="inlineStr">
+        <is>
+          <t>123933</t>
+        </is>
+      </c>
+      <c r="H625" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I625" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="626" ht="20" customHeight="1">
+      <c r="A626" s="9" t="n">
+        <v>622</v>
+      </c>
+      <c r="B626" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C626" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D626" s="9" t="n">
+        <v>877</v>
+      </c>
+      <c r="E626" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F626" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G626" s="10" t="inlineStr">
+        <is>
+          <t>123944</t>
+        </is>
+      </c>
+      <c r="H626" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I626" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="627" ht="20" customHeight="1">
+      <c r="A627" s="9" t="n">
+        <v>623</v>
+      </c>
+      <c r="B627" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C627" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D627" s="9" t="n">
+        <v>878</v>
+      </c>
+      <c r="E627" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F627" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G627" s="10" t="inlineStr">
+        <is>
+          <t>123932</t>
+        </is>
+      </c>
+      <c r="H627" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I627" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="628" ht="20" customHeight="1">
+      <c r="A628" s="9" t="n">
+        <v>624</v>
+      </c>
+      <c r="B628" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C628" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D628" s="9" t="n">
+        <v>879</v>
+      </c>
+      <c r="E628" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F628" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G628" s="10" t="inlineStr">
+        <is>
+          <t>123929</t>
+        </is>
+      </c>
+      <c r="H628" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I628" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="629" ht="20" customHeight="1">
+      <c r="A629" s="9" t="n">
+        <v>625</v>
+      </c>
+      <c r="B629" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C629" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D629" s="9" t="n">
+        <v>880</v>
+      </c>
+      <c r="E629" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F629" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G629" s="10" t="inlineStr">
+        <is>
+          <t>123931</t>
+        </is>
+      </c>
+      <c r="H629" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I629" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="630" ht="20" customHeight="1">
+      <c r="A630" s="9" t="n">
+        <v>626</v>
+      </c>
+      <c r="B630" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C630" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D630" s="9" t="n">
+        <v>881</v>
+      </c>
+      <c r="E630" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F630" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G630" s="10" t="inlineStr">
+        <is>
+          <t>123930</t>
+        </is>
+      </c>
+      <c r="H630" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I630" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="631" ht="20" customHeight="1">
+      <c r="A631" s="9" t="n">
+        <v>627</v>
+      </c>
+      <c r="B631" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C631" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D631" s="9" t="n">
+        <v>882</v>
+      </c>
+      <c r="E631" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F631" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G631" s="10" t="inlineStr">
+        <is>
+          <t>123941</t>
+        </is>
+      </c>
+      <c r="H631" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I631" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="632" ht="20" customHeight="1">
+      <c r="A632" s="9" t="n">
+        <v>628</v>
+      </c>
+      <c r="B632" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C632" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D632" s="9" t="n">
+        <v>883</v>
+      </c>
+      <c r="E632" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F632" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G632" s="10" t="inlineStr">
+        <is>
+          <t>124227</t>
+        </is>
+      </c>
+      <c r="H632" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I632" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="633" ht="20" customHeight="1">
+      <c r="A633" s="9" t="n">
+        <v>629</v>
+      </c>
+      <c r="B633" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C633" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D633" s="9" t="n">
+        <v>884</v>
+      </c>
+      <c r="E633" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F633" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G633" s="10" t="inlineStr">
+        <is>
+          <t>123940</t>
+        </is>
+      </c>
+      <c r="H633" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I633" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="634" ht="20" customHeight="1">
+      <c r="A634" s="9" t="n">
+        <v>630</v>
+      </c>
+      <c r="B634" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C634" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D634" s="9" t="n">
+        <v>885</v>
+      </c>
+      <c r="E634" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F634" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G634" s="10" t="inlineStr">
+        <is>
+          <t>123943</t>
+        </is>
+      </c>
+      <c r="H634" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I634" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="635" ht="20" customHeight="1">
+      <c r="A635" s="9" t="n">
+        <v>631</v>
+      </c>
+      <c r="B635" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C635" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D635" s="9" t="n">
+        <v>886</v>
+      </c>
+      <c r="E635" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F635" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G635" s="10" t="inlineStr">
+        <is>
+          <t>123942</t>
+        </is>
+      </c>
+      <c r="H635" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I635" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="636" ht="20" customHeight="1">
+      <c r="A636" s="9" t="n">
+        <v>632</v>
+      </c>
+      <c r="B636" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C636" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D636" s="9" t="n">
+        <v>887</v>
+      </c>
+      <c r="E636" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F636" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G636" s="10" t="inlineStr">
+        <is>
+          <t>123937</t>
+        </is>
+      </c>
+      <c r="H636" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I636" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="637" ht="20" customHeight="1">
+      <c r="A637" s="9" t="n">
+        <v>633</v>
+      </c>
+      <c r="B637" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C637" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D637" s="9" t="n">
+        <v>888</v>
+      </c>
+      <c r="E637" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="F637" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G637" s="10" t="inlineStr">
+        <is>
+          <t>33883</t>
+        </is>
+      </c>
+      <c r="H637" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I637" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="638" ht="20" customHeight="1">
+      <c r="A638" s="9" t="n">
+        <v>634</v>
+      </c>
+      <c r="B638" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C638" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D638" s="9" t="n">
+        <v>889</v>
+      </c>
+      <c r="E638" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F638" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G638" s="10" t="inlineStr">
+        <is>
+          <t>123936</t>
+        </is>
+      </c>
+      <c r="H638" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I638" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="639" ht="20" customHeight="1">
+      <c r="A639" s="9" t="n">
+        <v>635</v>
+      </c>
+      <c r="B639" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C639" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D639" s="9" t="n">
+        <v>890</v>
+      </c>
+      <c r="E639" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F639" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G639" s="10" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="H639" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I639" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="640" ht="20" customHeight="1">
+      <c r="A640" s="9" t="n">
+        <v>636</v>
+      </c>
+      <c r="B640" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C640" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D640" s="9" t="n">
+        <v>891</v>
+      </c>
+      <c r="E640" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F640" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G640" s="10" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="H640" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I640" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="641" ht="20" customHeight="1">
+      <c r="A641" s="9" t="n">
+        <v>637</v>
+      </c>
+      <c r="B641" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C641" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D641" s="9" t="n">
+        <v>892</v>
+      </c>
+      <c r="E641" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F641" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G641" s="10" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="H641" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I641" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="642" ht="20" customHeight="1">
+      <c r="A642" s="9" t="n">
+        <v>638</v>
+      </c>
+      <c r="B642" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C642" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D642" s="9" t="n">
+        <v>893</v>
+      </c>
+      <c r="E642" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F642" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G642" s="10" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="H642" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I642" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="643" ht="20" customHeight="1">
+      <c r="A643" s="9" t="n">
+        <v>639</v>
+      </c>
+      <c r="B643" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C643" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D643" s="9" t="n">
+        <v>894</v>
+      </c>
+      <c r="E643" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="F643" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G643" s="10" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="H643" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I643" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="644" ht="20" customHeight="1">
+      <c r="A644" s="9" t="n">
+        <v>640</v>
+      </c>
+      <c r="B644" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C644" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D644" s="9" t="n">
+        <v>895</v>
+      </c>
+      <c r="E644" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F644" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G644" s="10" t="inlineStr">
+        <is>
+          <t>33882</t>
+        </is>
+      </c>
+      <c r="H644" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I644" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (640 BAL)</t>
+        </is>
+      </c>
+      <c r="B645" s="4" t="n"/>
+      <c r="C645" s="4" t="n"/>
+      <c r="D645" s="4" t="n"/>
+      <c r="E645" s="4" t="n"/>
+      <c r="F645" s="4" t="n"/>
+      <c r="G645" s="4" t="n"/>
+      <c r="H645" s="4">
+        <f>SUM(H5:H644)</f>
         <v/>
       </c>
-      <c r="I611" s="4" t="inlineStr">
+      <c r="I645" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -35256,8 +37194,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A645:G645"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A611:G611"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35269,7 +37207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -35825,37 +37763,66 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>1349</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>39.68</v>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>833 - 895</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4">
-        <f>SUM(D5:D21)</f>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4">
+        <f>SUM(D5:D22)</f>
         <v/>
       </c>
-      <c r="E22" s="4">
-        <f>SUM(E5:E21)</f>
+      <c r="E23" s="4">
+        <f>SUM(E5:E22)</f>
         <v/>
       </c>
-      <c r="F22" s="4">
-        <f>AVERAGE(F5:F21)</f>
+      <c r="F23" s="4">
+        <f>AVERAGE(F5:F22)</f>
         <v/>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>3 - 857</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>3 - 895</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A22:C22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: tambah data bal 10 September 2026 (23 bal), sync Supabase Cloud, update rekap Excel dan cache v5.5
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F645"/>
+  <dimension ref="A1:F685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12736,47 +12736,47 @@
     </row>
     <row r="613" ht="20.25" customHeight="1">
       <c r="A613" s="5" t="n">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B613" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C613" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="C613" s="5" t="n">
-        <v>68</v>
-      </c>
       <c r="D613" s="6" t="inlineStr">
         <is>
-          <t>124284</t>
+          <t>124853</t>
         </is>
       </c>
       <c r="E613" s="5" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F613" s="5" t="n"/>
     </row>
     <row r="614" ht="20.25" customHeight="1">
       <c r="A614" s="5" t="n">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B614" s="5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C614" s="5" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D614" s="6" t="inlineStr">
         <is>
-          <t>124367</t>
+          <t>124284</t>
         </is>
       </c>
       <c r="E614" s="5" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F614" s="5" t="n"/>
     </row>
     <row r="615" ht="20.25" customHeight="1">
       <c r="A615" s="5" t="n">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B615" s="5" t="n">
         <v>72</v>
@@ -12786,317 +12786,317 @@
       </c>
       <c r="D615" s="6" t="inlineStr">
         <is>
-          <t>124368</t>
+          <t>124367</t>
         </is>
       </c>
       <c r="E615" s="5" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F615" s="5" t="n"/>
     </row>
     <row r="616" ht="20.25" customHeight="1">
       <c r="A616" s="5" t="n">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B616" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C616" s="5" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D616" s="6" t="inlineStr">
         <is>
-          <t>124370</t>
+          <t>124368</t>
         </is>
       </c>
       <c r="E616" s="5" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F616" s="5" t="n"/>
     </row>
     <row r="617" ht="20.25" customHeight="1">
       <c r="A617" s="5" t="n">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="B617" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C617" s="5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D617" s="6" t="inlineStr">
         <is>
-          <t>124371</t>
+          <t>124370</t>
         </is>
       </c>
       <c r="E617" s="5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F617" s="5" t="n"/>
     </row>
     <row r="618" ht="20.25" customHeight="1">
       <c r="A618" s="5" t="n">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="B618" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C618" s="5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D618" s="6" t="inlineStr">
         <is>
-          <t>124369</t>
+          <t>124851</t>
         </is>
       </c>
       <c r="E618" s="5" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F618" s="5" t="n"/>
     </row>
     <row r="619" ht="20.25" customHeight="1">
       <c r="A619" s="5" t="n">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="B619" s="5" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C619" s="5" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D619" s="6" t="inlineStr">
         <is>
-          <t>124285</t>
+          <t>124852</t>
         </is>
       </c>
       <c r="E619" s="5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F619" s="5" t="n"/>
     </row>
     <row r="620" ht="20.25" customHeight="1">
       <c r="A620" s="5" t="n">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="B620" s="5" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="C620" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="D620" s="6" t="inlineStr">
         <is>
-          <t>39833</t>
+          <t>124371</t>
         </is>
       </c>
       <c r="E620" s="5" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F620" s="5" t="n"/>
     </row>
     <row r="621" ht="20.25" customHeight="1">
       <c r="A621" s="5" t="n">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="B621" s="5" t="n">
         <v>72</v>
       </c>
       <c r="C621" s="5" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D621" s="6" t="inlineStr">
         <is>
-          <t>124366</t>
+          <t>124586</t>
         </is>
       </c>
       <c r="E621" s="5" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="F621" s="5" t="n"/>
     </row>
     <row r="622" ht="20.25" customHeight="1">
       <c r="A622" s="5" t="n">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="B622" s="5" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="C622" s="5" t="n">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="D622" s="6" t="inlineStr">
         <is>
-          <t>33879</t>
+          <t>124369</t>
         </is>
       </c>
       <c r="E622" s="5" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F622" s="5" t="n"/>
     </row>
     <row r="623" ht="20.25" customHeight="1">
       <c r="A623" s="5" t="n">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="B623" s="5" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C623" s="5" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D623" s="6" t="inlineStr">
         <is>
-          <t>123934</t>
+          <t>124285</t>
         </is>
       </c>
       <c r="E623" s="5" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F623" s="5" t="n"/>
     </row>
     <row r="624" ht="20.25" customHeight="1">
       <c r="A624" s="5" t="n">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="B624" s="5" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C624" s="5" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D624" s="6" t="inlineStr">
         <is>
-          <t>123935</t>
+          <t>39833</t>
         </is>
       </c>
       <c r="E624" s="5" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F624" s="5" t="n"/>
     </row>
     <row r="625" ht="20.25" customHeight="1">
       <c r="A625" s="5" t="n">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="B625" s="5" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C625" s="5" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="D625" s="6" t="inlineStr">
         <is>
-          <t>123933</t>
+          <t>124250</t>
         </is>
       </c>
       <c r="E625" s="5" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F625" s="5" t="n"/>
     </row>
     <row r="626" ht="20.25" customHeight="1">
       <c r="A626" s="5" t="n">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="B626" s="5" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="C626" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="D626" s="6" t="inlineStr">
         <is>
-          <t>123944</t>
+          <t>124366</t>
         </is>
       </c>
       <c r="E626" s="5" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F626" s="5" t="n"/>
     </row>
     <row r="627" ht="20.25" customHeight="1">
       <c r="A627" s="5" t="n">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="B627" s="5" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C627" s="5" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D627" s="6" t="inlineStr">
         <is>
-          <t>123932</t>
+          <t>33879</t>
         </is>
       </c>
       <c r="E627" s="5" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F627" s="5" t="n"/>
     </row>
     <row r="628" ht="20.25" customHeight="1">
       <c r="A628" s="5" t="n">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="B628" s="5" t="n">
         <v>57</v>
       </c>
       <c r="C628" s="5" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D628" s="6" t="inlineStr">
         <is>
-          <t>123929</t>
+          <t>123934</t>
         </is>
       </c>
       <c r="E628" s="5" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="F628" s="5" t="n"/>
     </row>
     <row r="629" ht="20.25" customHeight="1">
       <c r="A629" s="5" t="n">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="B629" s="5" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C629" s="5" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D629" s="6" t="inlineStr">
         <is>
-          <t>123931</t>
+          <t>123935</t>
         </is>
       </c>
       <c r="E629" s="5" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F629" s="5" t="n"/>
     </row>
     <row r="630" ht="20.25" customHeight="1">
       <c r="A630" s="5" t="n">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="B630" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C630" s="5" t="n">
         <v>57</v>
       </c>
-      <c r="C630" s="5" t="n">
-        <v>55</v>
-      </c>
       <c r="D630" s="6" t="inlineStr">
         <is>
-          <t>123930</t>
+          <t>123933</t>
         </is>
       </c>
       <c r="E630" s="5" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F630" s="5" t="n"/>
     </row>
     <row r="631" ht="20.25" customHeight="1">
       <c r="A631" s="5" t="n">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="B631" s="5" t="n">
         <v>57</v>
@@ -13106,67 +13106,67 @@
       </c>
       <c r="D631" s="6" t="inlineStr">
         <is>
-          <t>123941</t>
+          <t>123944</t>
         </is>
       </c>
       <c r="E631" s="5" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F631" s="5" t="n"/>
     </row>
     <row r="632" ht="20.25" customHeight="1">
       <c r="A632" s="5" t="n">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="B632" s="5" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="C632" s="5" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="D632" s="6" t="inlineStr">
         <is>
-          <t>124227</t>
+          <t>123932</t>
         </is>
       </c>
       <c r="E632" s="5" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F632" s="5" t="n"/>
     </row>
     <row r="633" ht="20.25" customHeight="1">
       <c r="A633" s="5" t="n">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="B633" s="5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C633" s="5" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D633" s="6" t="inlineStr">
         <is>
-          <t>123940</t>
+          <t>123929</t>
         </is>
       </c>
       <c r="E633" s="5" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F633" s="5" t="n"/>
     </row>
     <row r="634" ht="20.25" customHeight="1">
       <c r="A634" s="5" t="n">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="B634" s="5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C634" s="5" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D634" s="6" t="inlineStr">
         <is>
-          <t>123943</t>
+          <t>123931</t>
         </is>
       </c>
       <c r="E634" s="5" t="n">
@@ -13176,177 +13176,177 @@
     </row>
     <row r="635" ht="20.25" customHeight="1">
       <c r="A635" s="5" t="n">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="B635" s="5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C635" s="5" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D635" s="6" t="inlineStr">
         <is>
-          <t>123942</t>
+          <t>123930</t>
         </is>
       </c>
       <c r="E635" s="5" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F635" s="5" t="n"/>
     </row>
     <row r="636" ht="20.25" customHeight="1">
       <c r="A636" s="5" t="n">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="B636" s="5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C636" s="5" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D636" s="6" t="inlineStr">
         <is>
-          <t>123937</t>
+          <t>123941</t>
         </is>
       </c>
       <c r="E636" s="5" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F636" s="5" t="n"/>
     </row>
     <row r="637" ht="20.25" customHeight="1">
       <c r="A637" s="5" t="n">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="B637" s="5" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="C637" s="5" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="D637" s="6" t="inlineStr">
         <is>
-          <t>33883</t>
+          <t>124227</t>
         </is>
       </c>
       <c r="E637" s="5" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F637" s="5" t="n"/>
     </row>
     <row r="638" ht="20.25" customHeight="1">
       <c r="A638" s="5" t="n">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="B638" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C638" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="C638" s="5" t="n">
-        <v>55</v>
-      </c>
       <c r="D638" s="6" t="inlineStr">
         <is>
-          <t>123936</t>
+          <t>123940</t>
         </is>
       </c>
       <c r="E638" s="5" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="F638" s="5" t="n"/>
     </row>
     <row r="639" ht="20.25" customHeight="1">
       <c r="A639" s="5" t="n">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="B639" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C639" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="C639" s="5" t="n">
-        <v>55</v>
-      </c>
       <c r="D639" s="6" t="inlineStr">
         <is>
-          <t>123938</t>
+          <t>123943</t>
         </is>
       </c>
       <c r="E639" s="5" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F639" s="5" t="n"/>
     </row>
     <row r="640" ht="20.25" customHeight="1">
       <c r="A640" s="5" t="n">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="B640" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C640" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="C640" s="5" t="n">
-        <v>55</v>
-      </c>
       <c r="D640" s="6" t="inlineStr">
         <is>
-          <t>123939</t>
+          <t>123942</t>
         </is>
       </c>
       <c r="E640" s="5" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F640" s="5" t="n"/>
     </row>
     <row r="641" ht="20.25" customHeight="1">
       <c r="A641" s="5" t="n">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="B641" s="5" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C641" s="5" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D641" s="6" t="inlineStr">
         <is>
-          <t>33881</t>
+          <t>123937</t>
         </is>
       </c>
       <c r="E641" s="5" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F641" s="5" t="n"/>
     </row>
     <row r="642" ht="20.25" customHeight="1">
       <c r="A642" s="5" t="n">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="B642" s="5" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C642" s="5" t="n">
         <v>50</v>
       </c>
       <c r="D642" s="6" t="inlineStr">
         <is>
-          <t>33884</t>
+          <t>33883</t>
         </is>
       </c>
       <c r="E642" s="5" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="F642" s="5" t="n"/>
     </row>
     <row r="643" ht="20.25" customHeight="1">
       <c r="A643" s="5" t="n">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="B643" s="5" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C643" s="5" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D643" s="6" t="inlineStr">
         <is>
-          <t>33880</t>
+          <t>123936</t>
         </is>
       </c>
       <c r="E643" s="5" t="n">
@@ -13356,38 +13356,858 @@
     </row>
     <row r="644" ht="20.25" customHeight="1">
       <c r="A644" s="5" t="n">
+        <v>890</v>
+      </c>
+      <c r="B644" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C644" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D644" s="6" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="E644" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F644" s="5" t="n"/>
+    </row>
+    <row r="645" ht="20.25" customHeight="1">
+      <c r="A645" s="5" t="n">
+        <v>891</v>
+      </c>
+      <c r="B645" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C645" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D645" s="6" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="E645" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F645" s="5" t="n"/>
+    </row>
+    <row r="646" ht="20.25" customHeight="1">
+      <c r="A646" s="5" t="n">
+        <v>892</v>
+      </c>
+      <c r="B646" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="C646" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D646" s="6" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="E646" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F646" s="5" t="n"/>
+    </row>
+    <row r="647" ht="20.25" customHeight="1">
+      <c r="A647" s="5" t="n">
+        <v>893</v>
+      </c>
+      <c r="B647" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="C647" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D647" s="6" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="E647" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F647" s="5" t="n"/>
+    </row>
+    <row r="648" ht="20.25" customHeight="1">
+      <c r="A648" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="B648" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="C648" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D648" s="6" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="E648" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F648" s="5" t="n"/>
+    </row>
+    <row r="649" ht="20.25" customHeight="1">
+      <c r="A649" s="5" t="n">
         <v>895</v>
       </c>
-      <c r="B644" s="5" t="n">
+      <c r="B649" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="C644" s="5" t="n">
+      <c r="C649" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="D644" s="6" t="inlineStr">
+      <c r="D649" s="6" t="inlineStr">
         <is>
           <t>33882</t>
         </is>
       </c>
-      <c r="E644" s="5" t="n">
+      <c r="E649" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="F644" s="5" t="n"/>
-    </row>
-    <row r="645" ht="22" customHeight="1">
-      <c r="A645" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (640 BAL)</t>
-        </is>
-      </c>
-      <c r="B645" s="4" t="n"/>
-      <c r="C645" s="4" t="n"/>
-      <c r="D645" s="4" t="n"/>
-      <c r="E645" s="4">
-        <f>SUM(E5:E644)</f>
+      <c r="F649" s="5" t="n"/>
+    </row>
+    <row r="650" ht="20.25" customHeight="1">
+      <c r="A650" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="B650" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C650" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D650" s="6" t="inlineStr">
+        <is>
+          <t>124854</t>
+        </is>
+      </c>
+      <c r="E650" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F650" s="5" t="n"/>
+    </row>
+    <row r="651" ht="20.25" customHeight="1">
+      <c r="A651" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="B651" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C651" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D651" s="6" t="inlineStr">
+        <is>
+          <t>124855</t>
+        </is>
+      </c>
+      <c r="E651" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F651" s="5" t="n"/>
+    </row>
+    <row r="652" ht="20.25" customHeight="1">
+      <c r="A652" s="5" t="n">
+        <v>901</v>
+      </c>
+      <c r="B652" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C652" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D652" s="6" t="inlineStr">
+        <is>
+          <t>124856</t>
+        </is>
+      </c>
+      <c r="E652" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F652" s="5" t="n"/>
+    </row>
+    <row r="653" ht="20.25" customHeight="1">
+      <c r="A653" s="5" t="n">
+        <v>902</v>
+      </c>
+      <c r="B653" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C653" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D653" s="6" t="inlineStr">
+        <is>
+          <t>124857</t>
+        </is>
+      </c>
+      <c r="E653" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F653" s="5" t="n"/>
+    </row>
+    <row r="654" ht="20.25" customHeight="1">
+      <c r="A654" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="B654" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C654" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D654" s="6" t="inlineStr">
+        <is>
+          <t>124526</t>
+        </is>
+      </c>
+      <c r="E654" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F654" s="5" t="n"/>
+    </row>
+    <row r="655" ht="20.25" customHeight="1">
+      <c r="A655" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="B655" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C655" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D655" s="6" t="inlineStr">
+        <is>
+          <t>124588</t>
+        </is>
+      </c>
+      <c r="E655" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F655" s="5" t="n"/>
+    </row>
+    <row r="656" ht="20.25" customHeight="1">
+      <c r="A656" s="5" t="n">
+        <v>905</v>
+      </c>
+      <c r="B656" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C656" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D656" s="6" t="inlineStr">
+        <is>
+          <t>124587</t>
+        </is>
+      </c>
+      <c r="E656" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F656" s="5" t="n"/>
+    </row>
+    <row r="657" ht="20.25" customHeight="1">
+      <c r="A657" s="5" t="n">
+        <v>907</v>
+      </c>
+      <c r="B657" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C657" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="D657" s="6" t="inlineStr">
+        <is>
+          <t>33889</t>
+        </is>
+      </c>
+      <c r="E657" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F657" s="5" t="n"/>
+    </row>
+    <row r="658" ht="20.25" customHeight="1">
+      <c r="A658" s="5" t="n">
+        <v>911</v>
+      </c>
+      <c r="B658" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C658" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D658" s="6" t="inlineStr">
+        <is>
+          <t>124808</t>
+        </is>
+      </c>
+      <c r="E658" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F658" s="5" t="n"/>
+    </row>
+    <row r="659" ht="20.25" customHeight="1">
+      <c r="A659" s="5" t="n">
+        <v>912</v>
+      </c>
+      <c r="B659" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C659" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D659" s="6" t="inlineStr">
+        <is>
+          <t>124589</t>
+        </is>
+      </c>
+      <c r="E659" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F659" s="5" t="n"/>
+    </row>
+    <row r="660" ht="20.25" customHeight="1">
+      <c r="A660" s="5" t="n">
+        <v>913</v>
+      </c>
+      <c r="B660" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C660" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D660" s="6" t="inlineStr">
+        <is>
+          <t>33890</t>
+        </is>
+      </c>
+      <c r="E660" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F660" s="5" t="n"/>
+    </row>
+    <row r="661" ht="20.25" customHeight="1">
+      <c r="A661" s="5" t="n">
+        <v>914</v>
+      </c>
+      <c r="B661" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C661" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D661" s="6" t="inlineStr">
+        <is>
+          <t>124525</t>
+        </is>
+      </c>
+      <c r="E661" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F661" s="5" t="n"/>
+    </row>
+    <row r="662" ht="20.25" customHeight="1">
+      <c r="A662" s="5" t="n">
+        <v>915</v>
+      </c>
+      <c r="B662" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C662" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D662" s="6" t="inlineStr">
+        <is>
+          <t>124523</t>
+        </is>
+      </c>
+      <c r="E662" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F662" s="5" t="n"/>
+    </row>
+    <row r="663" ht="20.25" customHeight="1">
+      <c r="A663" s="5" t="n">
+        <v>916</v>
+      </c>
+      <c r="B663" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C663" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D663" s="6" t="inlineStr">
+        <is>
+          <t>124524</t>
+        </is>
+      </c>
+      <c r="E663" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F663" s="5" t="n"/>
+    </row>
+    <row r="664" ht="20.25" customHeight="1">
+      <c r="A664" s="5" t="n">
+        <v>917</v>
+      </c>
+      <c r="B664" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C664" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D664" s="6" t="inlineStr">
+        <is>
+          <t>125244</t>
+        </is>
+      </c>
+      <c r="E664" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F664" s="5" t="inlineStr">
+        <is>
+          <t>mateng</t>
+        </is>
+      </c>
+    </row>
+    <row r="665" ht="20.25" customHeight="1">
+      <c r="A665" s="5" t="n">
+        <v>918</v>
+      </c>
+      <c r="B665" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C665" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D665" s="6" t="inlineStr">
+        <is>
+          <t>125245</t>
+        </is>
+      </c>
+      <c r="E665" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F665" s="5" t="inlineStr">
+        <is>
+          <t>mateng</t>
+        </is>
+      </c>
+    </row>
+    <row r="666" ht="20.25" customHeight="1">
+      <c r="A666" s="5" t="n">
+        <v>919</v>
+      </c>
+      <c r="B666" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C666" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D666" s="6" t="inlineStr">
+        <is>
+          <t>125057</t>
+        </is>
+      </c>
+      <c r="E666" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F666" s="5" t="n"/>
+    </row>
+    <row r="667" ht="20.25" customHeight="1">
+      <c r="A667" s="5" t="n">
+        <v>920</v>
+      </c>
+      <c r="B667" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C667" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D667" s="6" t="inlineStr">
+        <is>
+          <t>125055</t>
+        </is>
+      </c>
+      <c r="E667" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F667" s="5" t="n"/>
+    </row>
+    <row r="668" ht="20.25" customHeight="1">
+      <c r="A668" s="5" t="n">
+        <v>921</v>
+      </c>
+      <c r="B668" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C668" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D668" s="6" t="inlineStr">
+        <is>
+          <t>125242</t>
+        </is>
+      </c>
+      <c r="E668" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F668" s="5" t="n"/>
+    </row>
+    <row r="669" ht="20.25" customHeight="1">
+      <c r="A669" s="5" t="n">
+        <v>922</v>
+      </c>
+      <c r="B669" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C669" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D669" s="6" t="inlineStr">
+        <is>
+          <t>125243</t>
+        </is>
+      </c>
+      <c r="E669" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F669" s="5" t="inlineStr">
+        <is>
+          <t>mateng</t>
+        </is>
+      </c>
+    </row>
+    <row r="670" ht="20.25" customHeight="1">
+      <c r="A670" s="5" t="n">
+        <v>923</v>
+      </c>
+      <c r="B670" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C670" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D670" s="6" t="inlineStr">
+        <is>
+          <t>125058</t>
+        </is>
+      </c>
+      <c r="E670" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F670" s="5" t="n"/>
+    </row>
+    <row r="671" ht="20.25" customHeight="1">
+      <c r="A671" s="5" t="n">
+        <v>924</v>
+      </c>
+      <c r="B671" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C671" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D671" s="6" t="inlineStr">
+        <is>
+          <t>125056</t>
+        </is>
+      </c>
+      <c r="E671" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F671" s="5" t="n"/>
+    </row>
+    <row r="672" ht="20.25" customHeight="1">
+      <c r="A672" s="5" t="n">
+        <v>925</v>
+      </c>
+      <c r="B672" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C672" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D672" s="6" t="inlineStr">
+        <is>
+          <t>125059</t>
+        </is>
+      </c>
+      <c r="E672" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F672" s="5" t="n"/>
+    </row>
+    <row r="673" ht="20.25" customHeight="1">
+      <c r="A673" s="5" t="n">
+        <v>926</v>
+      </c>
+      <c r="B673" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C673" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D673" s="6" t="inlineStr">
+        <is>
+          <t>125246</t>
+        </is>
+      </c>
+      <c r="E673" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F673" s="5" t="inlineStr">
+        <is>
+          <t>mateng</t>
+        </is>
+      </c>
+    </row>
+    <row r="674" ht="20.25" customHeight="1">
+      <c r="A674" s="5" t="n">
+        <v>927</v>
+      </c>
+      <c r="B674" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C674" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D674" s="6" t="inlineStr">
+        <is>
+          <t>125061</t>
+        </is>
+      </c>
+      <c r="E674" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F674" s="5" t="n"/>
+    </row>
+    <row r="675" ht="20.25" customHeight="1">
+      <c r="A675" s="5" t="n">
+        <v>928</v>
+      </c>
+      <c r="B675" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C675" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D675" s="6" t="inlineStr">
+        <is>
+          <t>125247</t>
+        </is>
+      </c>
+      <c r="E675" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F675" s="5" t="inlineStr">
+        <is>
+          <t>mateng</t>
+        </is>
+      </c>
+    </row>
+    <row r="676" ht="20.25" customHeight="1">
+      <c r="A676" s="5" t="n">
+        <v>929</v>
+      </c>
+      <c r="B676" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C676" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D676" s="6" t="inlineStr">
+        <is>
+          <t>125248</t>
+        </is>
+      </c>
+      <c r="E676" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F676" s="5" t="n"/>
+    </row>
+    <row r="677" ht="20.25" customHeight="1">
+      <c r="A677" s="5" t="n">
+        <v>932</v>
+      </c>
+      <c r="B677" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C677" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D677" s="6" t="inlineStr">
+        <is>
+          <t>125060</t>
+        </is>
+      </c>
+      <c r="E677" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F677" s="5" t="n"/>
+    </row>
+    <row r="678" ht="20.25" customHeight="1">
+      <c r="A678" s="5" t="n">
+        <v>933</v>
+      </c>
+      <c r="B678" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C678" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D678" s="6" t="inlineStr">
+        <is>
+          <t>125062</t>
+        </is>
+      </c>
+      <c r="E678" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F678" s="5" t="n"/>
+    </row>
+    <row r="679" ht="20.25" customHeight="1">
+      <c r="A679" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="B679" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C679" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D679" s="6" t="inlineStr">
+        <is>
+          <t>124539</t>
+        </is>
+      </c>
+      <c r="E679" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F679" s="5" t="n"/>
+    </row>
+    <row r="680" ht="20.25" customHeight="1">
+      <c r="A680" s="5" t="n">
+        <v>935</v>
+      </c>
+      <c r="B680" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C680" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D680" s="6" t="inlineStr">
+        <is>
+          <t>124538</t>
+        </is>
+      </c>
+      <c r="E680" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F680" s="5" t="n"/>
+    </row>
+    <row r="681" ht="20.25" customHeight="1">
+      <c r="A681" s="5" t="n">
+        <v>936</v>
+      </c>
+      <c r="B681" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C681" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D681" s="6" t="inlineStr">
+        <is>
+          <t>124537</t>
+        </is>
+      </c>
+      <c r="E681" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F681" s="5" t="n"/>
+    </row>
+    <row r="682" ht="20.25" customHeight="1">
+      <c r="A682" s="5" t="n">
+        <v>937</v>
+      </c>
+      <c r="B682" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C682" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D682" s="6" t="inlineStr">
+        <is>
+          <t>124536</t>
+        </is>
+      </c>
+      <c r="E682" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F682" s="5" t="n"/>
+    </row>
+    <row r="683" ht="20.25" customHeight="1">
+      <c r="A683" s="5" t="n">
+        <v>938</v>
+      </c>
+      <c r="B683" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="C683" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D683" s="6" t="inlineStr">
+        <is>
+          <t>125053</t>
+        </is>
+      </c>
+      <c r="E683" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F683" s="5" t="n"/>
+    </row>
+    <row r="684" ht="20.25" customHeight="1">
+      <c r="A684" s="5" t="n">
+        <v>939</v>
+      </c>
+      <c r="B684" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="C684" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D684" s="6" t="inlineStr">
+        <is>
+          <t>125054</t>
+        </is>
+      </c>
+      <c r="E684" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F684" s="5" t="n"/>
+    </row>
+    <row r="685" ht="22" customHeight="1">
+      <c r="A685" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (680 BAL)</t>
+        </is>
+      </c>
+      <c r="B685" s="4" t="n"/>
+      <c r="C685" s="4" t="n"/>
+      <c r="D685" s="4" t="n"/>
+      <c r="E685" s="4">
+        <f>SUM(E5:E684)</f>
         <v/>
       </c>
-      <c r="F645" s="4" t="inlineStr">
+      <c r="F685" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -13399,7 +14219,7 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A645:D645"/>
+    <mergeCell ref="A685:D685"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -13414,7 +14234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I645"/>
+  <dimension ref="A1:I685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13438,7 +14258,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 640 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 680 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -35991,34 +36811,34 @@
       </c>
       <c r="B613" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C613" s="9" t="inlineStr">
         <is>
-          <t>SELASA</t>
+          <t>RABU</t>
         </is>
       </c>
       <c r="D613" s="9" t="n">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E613" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F613" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="F613" s="9" t="n">
-        <v>68</v>
-      </c>
       <c r="G613" s="10" t="inlineStr">
         <is>
-          <t>124284</t>
+          <t>124853</t>
         </is>
       </c>
       <c r="H613" s="9" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="I613" s="11" t="inlineStr">
         <is>
-          <t>grade 8 sep.xlsx</t>
+          <t>grade 9 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -36037,21 +36857,21 @@
         </is>
       </c>
       <c r="D614" s="9" t="n">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E614" s="9" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F614" s="9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G614" s="10" t="inlineStr">
         <is>
-          <t>124367</t>
+          <t>124284</t>
         </is>
       </c>
       <c r="H614" s="9" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="I614" s="11" t="inlineStr">
         <is>
@@ -36074,7 +36894,7 @@
         </is>
       </c>
       <c r="D615" s="9" t="n">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E615" s="9" t="n">
         <v>72</v>
@@ -36084,11 +36904,11 @@
       </c>
       <c r="G615" s="10" t="inlineStr">
         <is>
-          <t>124368</t>
+          <t>124367</t>
         </is>
       </c>
       <c r="H615" s="9" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="I615" s="11" t="inlineStr">
         <is>
@@ -36111,21 +36931,21 @@
         </is>
       </c>
       <c r="D616" s="9" t="n">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="E616" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F616" s="9" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G616" s="10" t="inlineStr">
         <is>
-          <t>124370</t>
+          <t>124368</t>
         </is>
       </c>
       <c r="H616" s="9" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I616" s="11" t="inlineStr">
         <is>
@@ -36148,21 +36968,21 @@
         </is>
       </c>
       <c r="D617" s="9" t="n">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="E617" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F617" s="9" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G617" s="10" t="inlineStr">
         <is>
-          <t>124371</t>
+          <t>124370</t>
         </is>
       </c>
       <c r="H617" s="9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I617" s="11" t="inlineStr">
         <is>
@@ -36176,34 +36996,34 @@
       </c>
       <c r="B618" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C618" s="9" t="inlineStr">
         <is>
-          <t>SELASA</t>
+          <t>RABU</t>
         </is>
       </c>
       <c r="D618" s="9" t="n">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="E618" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F618" s="9" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G618" s="10" t="inlineStr">
         <is>
-          <t>124369</t>
+          <t>124851</t>
         </is>
       </c>
       <c r="H618" s="9" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="I618" s="11" t="inlineStr">
         <is>
-          <t>grade 8 sep.xlsx</t>
+          <t>grade 9 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -36213,34 +37033,34 @@
       </c>
       <c r="B619" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C619" s="9" t="inlineStr">
         <is>
-          <t>SELASA</t>
+          <t>RABU</t>
         </is>
       </c>
       <c r="D619" s="9" t="n">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="E619" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F619" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G619" s="10" t="inlineStr">
         <is>
-          <t>124285</t>
+          <t>124852</t>
         </is>
       </c>
       <c r="H619" s="9" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I619" s="11" t="inlineStr">
         <is>
-          <t>grade 8 sep.xlsx</t>
+          <t>grade 9 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -36259,21 +37079,21 @@
         </is>
       </c>
       <c r="D620" s="9" t="n">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="E620" s="9" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F620" s="9" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G620" s="10" t="inlineStr">
         <is>
-          <t>39833</t>
+          <t>124371</t>
         </is>
       </c>
       <c r="H620" s="9" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I620" s="11" t="inlineStr">
         <is>
@@ -36287,34 +37107,34 @@
       </c>
       <c r="B621" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C621" s="9" t="inlineStr">
         <is>
-          <t>SELASA</t>
+          <t>RABU</t>
         </is>
       </c>
       <c r="D621" s="9" t="n">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="E621" s="9" t="n">
         <v>72</v>
       </c>
       <c r="F621" s="9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G621" s="10" t="inlineStr">
         <is>
-          <t>124366</t>
+          <t>124586</t>
         </is>
       </c>
       <c r="H621" s="9" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="I621" s="11" t="inlineStr">
         <is>
-          <t>grade 8 sep.xlsx</t>
+          <t>grade 9 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -36333,21 +37153,21 @@
         </is>
       </c>
       <c r="D622" s="9" t="n">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="E622" s="9" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F622" s="9" t="n">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G622" s="10" t="inlineStr">
         <is>
-          <t>33879</t>
+          <t>124369</t>
         </is>
       </c>
       <c r="H622" s="9" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I622" s="11" t="inlineStr">
         <is>
@@ -36370,21 +37190,21 @@
         </is>
       </c>
       <c r="D623" s="9" t="n">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="E623" s="9" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="F623" s="9" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G623" s="10" t="inlineStr">
         <is>
-          <t>123934</t>
+          <t>124285</t>
         </is>
       </c>
       <c r="H623" s="9" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="I623" s="11" t="inlineStr">
         <is>
@@ -36407,21 +37227,21 @@
         </is>
       </c>
       <c r="D624" s="9" t="n">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="E624" s="9" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F624" s="9" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G624" s="10" t="inlineStr">
         <is>
-          <t>123935</t>
+          <t>39833</t>
         </is>
       </c>
       <c r="H624" s="9" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I624" s="11" t="inlineStr">
         <is>
@@ -36435,34 +37255,34 @@
       </c>
       <c r="B625" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C625" s="9" t="inlineStr">
         <is>
-          <t>SELASA</t>
+          <t>RABU</t>
         </is>
       </c>
       <c r="D625" s="9" t="n">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="E625" s="9" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F625" s="9" t="n">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="G625" s="10" t="inlineStr">
         <is>
-          <t>123933</t>
+          <t>124250</t>
         </is>
       </c>
       <c r="H625" s="9" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="I625" s="11" t="inlineStr">
         <is>
-          <t>grade 8 sep.xlsx</t>
+          <t>grade 9 sep.xlsx</t>
         </is>
       </c>
     </row>
@@ -36481,21 +37301,21 @@
         </is>
       </c>
       <c r="D626" s="9" t="n">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="E626" s="9" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F626" s="9" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G626" s="10" t="inlineStr">
         <is>
-          <t>123944</t>
+          <t>124366</t>
         </is>
       </c>
       <c r="H626" s="9" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I626" s="11" t="inlineStr">
         <is>
@@ -36518,21 +37338,21 @@
         </is>
       </c>
       <c r="D627" s="9" t="n">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="E627" s="9" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F627" s="9" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G627" s="10" t="inlineStr">
         <is>
-          <t>123932</t>
+          <t>33879</t>
         </is>
       </c>
       <c r="H627" s="9" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I627" s="11" t="inlineStr">
         <is>
@@ -36555,21 +37375,21 @@
         </is>
       </c>
       <c r="D628" s="9" t="n">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="E628" s="9" t="n">
         <v>57</v>
       </c>
       <c r="F628" s="9" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G628" s="10" t="inlineStr">
         <is>
-          <t>123929</t>
+          <t>123934</t>
         </is>
       </c>
       <c r="H628" s="9" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="I628" s="11" t="inlineStr">
         <is>
@@ -36592,21 +37412,21 @@
         </is>
       </c>
       <c r="D629" s="9" t="n">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="E629" s="9" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F629" s="9" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G629" s="10" t="inlineStr">
         <is>
-          <t>123931</t>
+          <t>123935</t>
         </is>
       </c>
       <c r="H629" s="9" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I629" s="11" t="inlineStr">
         <is>
@@ -36629,21 +37449,21 @@
         </is>
       </c>
       <c r="D630" s="9" t="n">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="E630" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F630" s="9" t="n">
         <v>57</v>
       </c>
-      <c r="F630" s="9" t="n">
-        <v>55</v>
-      </c>
       <c r="G630" s="10" t="inlineStr">
         <is>
-          <t>123930</t>
+          <t>123933</t>
         </is>
       </c>
       <c r="H630" s="9" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="I630" s="11" t="inlineStr">
         <is>
@@ -36666,7 +37486,7 @@
         </is>
       </c>
       <c r="D631" s="9" t="n">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="E631" s="9" t="n">
         <v>57</v>
@@ -36676,11 +37496,11 @@
       </c>
       <c r="G631" s="10" t="inlineStr">
         <is>
-          <t>123941</t>
+          <t>123944</t>
         </is>
       </c>
       <c r="H631" s="9" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="I631" s="11" t="inlineStr">
         <is>
@@ -36703,21 +37523,21 @@
         </is>
       </c>
       <c r="D632" s="9" t="n">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="E632" s="9" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="F632" s="9" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="G632" s="10" t="inlineStr">
         <is>
-          <t>124227</t>
+          <t>123932</t>
         </is>
       </c>
       <c r="H632" s="9" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="I632" s="11" t="inlineStr">
         <is>
@@ -36740,21 +37560,21 @@
         </is>
       </c>
       <c r="D633" s="9" t="n">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="E633" s="9" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F633" s="9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G633" s="10" t="inlineStr">
         <is>
-          <t>123940</t>
+          <t>123929</t>
         </is>
       </c>
       <c r="H633" s="9" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I633" s="11" t="inlineStr">
         <is>
@@ -36777,17 +37597,17 @@
         </is>
       </c>
       <c r="D634" s="9" t="n">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="E634" s="9" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F634" s="9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G634" s="10" t="inlineStr">
         <is>
-          <t>123943</t>
+          <t>123931</t>
         </is>
       </c>
       <c r="H634" s="9" t="n">
@@ -36814,21 +37634,21 @@
         </is>
       </c>
       <c r="D635" s="9" t="n">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E635" s="9" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F635" s="9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G635" s="10" t="inlineStr">
         <is>
-          <t>123942</t>
+          <t>123930</t>
         </is>
       </c>
       <c r="H635" s="9" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I635" s="11" t="inlineStr">
         <is>
@@ -36851,21 +37671,21 @@
         </is>
       </c>
       <c r="D636" s="9" t="n">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="E636" s="9" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F636" s="9" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G636" s="10" t="inlineStr">
         <is>
-          <t>123937</t>
+          <t>123941</t>
         </is>
       </c>
       <c r="H636" s="9" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="I636" s="11" t="inlineStr">
         <is>
@@ -36888,21 +37708,21 @@
         </is>
       </c>
       <c r="D637" s="9" t="n">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="E637" s="9" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="F637" s="9" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="G637" s="10" t="inlineStr">
         <is>
-          <t>33883</t>
+          <t>124227</t>
         </is>
       </c>
       <c r="H637" s="9" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="I637" s="11" t="inlineStr">
         <is>
@@ -36925,21 +37745,21 @@
         </is>
       </c>
       <c r="D638" s="9" t="n">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="E638" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F638" s="9" t="n">
         <v>56</v>
       </c>
-      <c r="F638" s="9" t="n">
-        <v>55</v>
-      </c>
       <c r="G638" s="10" t="inlineStr">
         <is>
-          <t>123936</t>
+          <t>123940</t>
         </is>
       </c>
       <c r="H638" s="9" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="I638" s="11" t="inlineStr">
         <is>
@@ -36962,21 +37782,21 @@
         </is>
       </c>
       <c r="D639" s="9" t="n">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="E639" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F639" s="9" t="n">
         <v>56</v>
       </c>
-      <c r="F639" s="9" t="n">
-        <v>55</v>
-      </c>
       <c r="G639" s="10" t="inlineStr">
         <is>
-          <t>123938</t>
+          <t>123943</t>
         </is>
       </c>
       <c r="H639" s="9" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I639" s="11" t="inlineStr">
         <is>
@@ -36999,21 +37819,21 @@
         </is>
       </c>
       <c r="D640" s="9" t="n">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="E640" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F640" s="9" t="n">
         <v>56</v>
       </c>
-      <c r="F640" s="9" t="n">
-        <v>55</v>
-      </c>
       <c r="G640" s="10" t="inlineStr">
         <is>
-          <t>123939</t>
+          <t>123942</t>
         </is>
       </c>
       <c r="H640" s="9" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I640" s="11" t="inlineStr">
         <is>
@@ -37036,21 +37856,21 @@
         </is>
       </c>
       <c r="D641" s="9" t="n">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="E641" s="9" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F641" s="9" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G641" s="10" t="inlineStr">
         <is>
-          <t>33881</t>
+          <t>123937</t>
         </is>
       </c>
       <c r="H641" s="9" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I641" s="11" t="inlineStr">
         <is>
@@ -37073,21 +37893,21 @@
         </is>
       </c>
       <c r="D642" s="9" t="n">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="E642" s="9" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F642" s="9" t="n">
         <v>50</v>
       </c>
       <c r="G642" s="10" t="inlineStr">
         <is>
-          <t>33884</t>
+          <t>33883</t>
         </is>
       </c>
       <c r="H642" s="9" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="I642" s="11" t="inlineStr">
         <is>
@@ -37110,17 +37930,17 @@
         </is>
       </c>
       <c r="D643" s="9" t="n">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="E643" s="9" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F643" s="9" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G643" s="10" t="inlineStr">
         <is>
-          <t>33880</t>
+          <t>123936</t>
         </is>
       </c>
       <c r="H643" s="9" t="n">
@@ -37147,45 +37967,1525 @@
         </is>
       </c>
       <c r="D644" s="9" t="n">
+        <v>890</v>
+      </c>
+      <c r="E644" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F644" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G644" s="10" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="H644" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I644" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="645" ht="20" customHeight="1">
+      <c r="A645" s="9" t="n">
+        <v>641</v>
+      </c>
+      <c r="B645" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C645" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D645" s="9" t="n">
+        <v>891</v>
+      </c>
+      <c r="E645" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F645" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G645" s="10" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="H645" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I645" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="646" ht="20" customHeight="1">
+      <c r="A646" s="9" t="n">
+        <v>642</v>
+      </c>
+      <c r="B646" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C646" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D646" s="9" t="n">
+        <v>892</v>
+      </c>
+      <c r="E646" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F646" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G646" s="10" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="H646" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I646" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="647" ht="20" customHeight="1">
+      <c r="A647" s="9" t="n">
+        <v>643</v>
+      </c>
+      <c r="B647" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C647" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D647" s="9" t="n">
+        <v>893</v>
+      </c>
+      <c r="E647" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F647" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G647" s="10" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="H647" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I647" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="648" ht="20" customHeight="1">
+      <c r="A648" s="9" t="n">
+        <v>644</v>
+      </c>
+      <c r="B648" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C648" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D648" s="9" t="n">
+        <v>894</v>
+      </c>
+      <c r="E648" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="F648" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G648" s="10" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="H648" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I648" s="11" t="inlineStr">
+        <is>
+          <t>grade 8 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="649" ht="20" customHeight="1">
+      <c r="A649" s="9" t="n">
+        <v>645</v>
+      </c>
+      <c r="B649" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C649" s="9" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D649" s="9" t="n">
         <v>895</v>
       </c>
-      <c r="E644" s="9" t="n">
+      <c r="E649" s="9" t="n">
         <v>53</v>
       </c>
-      <c r="F644" s="9" t="n">
+      <c r="F649" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="G644" s="10" t="inlineStr">
+      <c r="G649" s="10" t="inlineStr">
         <is>
           <t>33882</t>
         </is>
       </c>
-      <c r="H644" s="9" t="n">
+      <c r="H649" s="9" t="n">
         <v>49</v>
       </c>
-      <c r="I644" s="11" t="inlineStr">
+      <c r="I649" s="11" t="inlineStr">
         <is>
           <t>grade 8 sep.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="645">
-      <c r="A645" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (640 BAL)</t>
-        </is>
-      </c>
-      <c r="B645" s="4" t="n"/>
-      <c r="C645" s="4" t="n"/>
-      <c r="D645" s="4" t="n"/>
-      <c r="E645" s="4" t="n"/>
-      <c r="F645" s="4" t="n"/>
-      <c r="G645" s="4" t="n"/>
-      <c r="H645" s="4">
-        <f>SUM(H5:H644)</f>
+    <row r="650" ht="20" customHeight="1">
+      <c r="A650" s="9" t="n">
+        <v>646</v>
+      </c>
+      <c r="B650" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C650" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D650" s="9" t="n">
+        <v>899</v>
+      </c>
+      <c r="E650" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F650" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G650" s="10" t="inlineStr">
+        <is>
+          <t>124854</t>
+        </is>
+      </c>
+      <c r="H650" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I650" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="651" ht="20" customHeight="1">
+      <c r="A651" s="9" t="n">
+        <v>647</v>
+      </c>
+      <c r="B651" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C651" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D651" s="9" t="n">
+        <v>900</v>
+      </c>
+      <c r="E651" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F651" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G651" s="10" t="inlineStr">
+        <is>
+          <t>124855</t>
+        </is>
+      </c>
+      <c r="H651" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I651" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="652" ht="20" customHeight="1">
+      <c r="A652" s="9" t="n">
+        <v>648</v>
+      </c>
+      <c r="B652" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C652" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D652" s="9" t="n">
+        <v>901</v>
+      </c>
+      <c r="E652" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F652" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G652" s="10" t="inlineStr">
+        <is>
+          <t>124856</t>
+        </is>
+      </c>
+      <c r="H652" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I652" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="653" ht="20" customHeight="1">
+      <c r="A653" s="9" t="n">
+        <v>649</v>
+      </c>
+      <c r="B653" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C653" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D653" s="9" t="n">
+        <v>902</v>
+      </c>
+      <c r="E653" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F653" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G653" s="10" t="inlineStr">
+        <is>
+          <t>124857</t>
+        </is>
+      </c>
+      <c r="H653" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I653" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="654" ht="20" customHeight="1">
+      <c r="A654" s="9" t="n">
+        <v>650</v>
+      </c>
+      <c r="B654" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C654" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D654" s="9" t="n">
+        <v>903</v>
+      </c>
+      <c r="E654" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F654" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G654" s="10" t="inlineStr">
+        <is>
+          <t>124526</t>
+        </is>
+      </c>
+      <c r="H654" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I654" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="655" ht="20" customHeight="1">
+      <c r="A655" s="9" t="n">
+        <v>651</v>
+      </c>
+      <c r="B655" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C655" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D655" s="9" t="n">
+        <v>904</v>
+      </c>
+      <c r="E655" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F655" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G655" s="10" t="inlineStr">
+        <is>
+          <t>124588</t>
+        </is>
+      </c>
+      <c r="H655" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I655" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="656" ht="20" customHeight="1">
+      <c r="A656" s="9" t="n">
+        <v>652</v>
+      </c>
+      <c r="B656" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C656" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D656" s="9" t="n">
+        <v>905</v>
+      </c>
+      <c r="E656" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F656" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G656" s="10" t="inlineStr">
+        <is>
+          <t>124587</t>
+        </is>
+      </c>
+      <c r="H656" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I656" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="657" ht="20" customHeight="1">
+      <c r="A657" s="9" t="n">
+        <v>653</v>
+      </c>
+      <c r="B657" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C657" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D657" s="9" t="n">
+        <v>907</v>
+      </c>
+      <c r="E657" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F657" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="G657" s="10" t="inlineStr">
+        <is>
+          <t>33889</t>
+        </is>
+      </c>
+      <c r="H657" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I657" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="658" ht="20" customHeight="1">
+      <c r="A658" s="9" t="n">
+        <v>654</v>
+      </c>
+      <c r="B658" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C658" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D658" s="9" t="n">
+        <v>911</v>
+      </c>
+      <c r="E658" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F658" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G658" s="10" t="inlineStr">
+        <is>
+          <t>124808</t>
+        </is>
+      </c>
+      <c r="H658" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I658" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="659" ht="20" customHeight="1">
+      <c r="A659" s="9" t="n">
+        <v>655</v>
+      </c>
+      <c r="B659" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C659" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D659" s="9" t="n">
+        <v>912</v>
+      </c>
+      <c r="E659" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F659" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G659" s="10" t="inlineStr">
+        <is>
+          <t>124589</t>
+        </is>
+      </c>
+      <c r="H659" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I659" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="660" ht="20" customHeight="1">
+      <c r="A660" s="9" t="n">
+        <v>656</v>
+      </c>
+      <c r="B660" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C660" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D660" s="9" t="n">
+        <v>913</v>
+      </c>
+      <c r="E660" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F660" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G660" s="10" t="inlineStr">
+        <is>
+          <t>33890</t>
+        </is>
+      </c>
+      <c r="H660" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I660" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="661" ht="20" customHeight="1">
+      <c r="A661" s="9" t="n">
+        <v>657</v>
+      </c>
+      <c r="B661" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C661" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D661" s="9" t="n">
+        <v>914</v>
+      </c>
+      <c r="E661" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F661" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G661" s="10" t="inlineStr">
+        <is>
+          <t>124525</t>
+        </is>
+      </c>
+      <c r="H661" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I661" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="662" ht="20" customHeight="1">
+      <c r="A662" s="9" t="n">
+        <v>658</v>
+      </c>
+      <c r="B662" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C662" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D662" s="9" t="n">
+        <v>915</v>
+      </c>
+      <c r="E662" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F662" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G662" s="10" t="inlineStr">
+        <is>
+          <t>124523</t>
+        </is>
+      </c>
+      <c r="H662" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I662" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="663" ht="20" customHeight="1">
+      <c r="A663" s="9" t="n">
+        <v>659</v>
+      </c>
+      <c r="B663" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C663" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D663" s="9" t="n">
+        <v>916</v>
+      </c>
+      <c r="E663" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F663" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G663" s="10" t="inlineStr">
+        <is>
+          <t>124524</t>
+        </is>
+      </c>
+      <c r="H663" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I663" s="11" t="inlineStr">
+        <is>
+          <t>grade 9 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="664" ht="20" customHeight="1">
+      <c r="A664" s="9" t="n">
+        <v>660</v>
+      </c>
+      <c r="B664" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C664" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D664" s="9" t="n">
+        <v>917</v>
+      </c>
+      <c r="E664" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F664" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G664" s="10" t="inlineStr">
+        <is>
+          <t>125244</t>
+        </is>
+      </c>
+      <c r="H664" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I664" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="665" ht="20" customHeight="1">
+      <c r="A665" s="9" t="n">
+        <v>661</v>
+      </c>
+      <c r="B665" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C665" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D665" s="9" t="n">
+        <v>918</v>
+      </c>
+      <c r="E665" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F665" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G665" s="10" t="inlineStr">
+        <is>
+          <t>125245</t>
+        </is>
+      </c>
+      <c r="H665" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I665" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="666" ht="20" customHeight="1">
+      <c r="A666" s="9" t="n">
+        <v>662</v>
+      </c>
+      <c r="B666" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C666" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D666" s="9" t="n">
+        <v>919</v>
+      </c>
+      <c r="E666" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F666" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G666" s="10" t="inlineStr">
+        <is>
+          <t>125057</t>
+        </is>
+      </c>
+      <c r="H666" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I666" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="667" ht="20" customHeight="1">
+      <c r="A667" s="9" t="n">
+        <v>663</v>
+      </c>
+      <c r="B667" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C667" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D667" s="9" t="n">
+        <v>920</v>
+      </c>
+      <c r="E667" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F667" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G667" s="10" t="inlineStr">
+        <is>
+          <t>125055</t>
+        </is>
+      </c>
+      <c r="H667" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I667" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="668" ht="20" customHeight="1">
+      <c r="A668" s="9" t="n">
+        <v>664</v>
+      </c>
+      <c r="B668" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C668" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D668" s="9" t="n">
+        <v>921</v>
+      </c>
+      <c r="E668" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F668" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G668" s="10" t="inlineStr">
+        <is>
+          <t>125242</t>
+        </is>
+      </c>
+      <c r="H668" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I668" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="669" ht="20" customHeight="1">
+      <c r="A669" s="9" t="n">
+        <v>665</v>
+      </c>
+      <c r="B669" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C669" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D669" s="9" t="n">
+        <v>922</v>
+      </c>
+      <c r="E669" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F669" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G669" s="10" t="inlineStr">
+        <is>
+          <t>125243</t>
+        </is>
+      </c>
+      <c r="H669" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I669" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="670" ht="20" customHeight="1">
+      <c r="A670" s="9" t="n">
+        <v>666</v>
+      </c>
+      <c r="B670" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C670" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D670" s="9" t="n">
+        <v>923</v>
+      </c>
+      <c r="E670" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F670" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G670" s="10" t="inlineStr">
+        <is>
+          <t>125058</t>
+        </is>
+      </c>
+      <c r="H670" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I670" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="671" ht="20" customHeight="1">
+      <c r="A671" s="9" t="n">
+        <v>667</v>
+      </c>
+      <c r="B671" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C671" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D671" s="9" t="n">
+        <v>924</v>
+      </c>
+      <c r="E671" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F671" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G671" s="10" t="inlineStr">
+        <is>
+          <t>125056</t>
+        </is>
+      </c>
+      <c r="H671" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I671" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="672" ht="20" customHeight="1">
+      <c r="A672" s="9" t="n">
+        <v>668</v>
+      </c>
+      <c r="B672" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C672" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D672" s="9" t="n">
+        <v>925</v>
+      </c>
+      <c r="E672" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F672" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G672" s="10" t="inlineStr">
+        <is>
+          <t>125059</t>
+        </is>
+      </c>
+      <c r="H672" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I672" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="673" ht="20" customHeight="1">
+      <c r="A673" s="9" t="n">
+        <v>669</v>
+      </c>
+      <c r="B673" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C673" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D673" s="9" t="n">
+        <v>926</v>
+      </c>
+      <c r="E673" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F673" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G673" s="10" t="inlineStr">
+        <is>
+          <t>125246</t>
+        </is>
+      </c>
+      <c r="H673" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I673" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="674" ht="20" customHeight="1">
+      <c r="A674" s="9" t="n">
+        <v>670</v>
+      </c>
+      <c r="B674" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C674" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D674" s="9" t="n">
+        <v>927</v>
+      </c>
+      <c r="E674" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F674" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G674" s="10" t="inlineStr">
+        <is>
+          <t>125061</t>
+        </is>
+      </c>
+      <c r="H674" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I674" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="675" ht="20" customHeight="1">
+      <c r="A675" s="9" t="n">
+        <v>671</v>
+      </c>
+      <c r="B675" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C675" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D675" s="9" t="n">
+        <v>928</v>
+      </c>
+      <c r="E675" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F675" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G675" s="10" t="inlineStr">
+        <is>
+          <t>125247</t>
+        </is>
+      </c>
+      <c r="H675" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I675" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="676" ht="20" customHeight="1">
+      <c r="A676" s="9" t="n">
+        <v>672</v>
+      </c>
+      <c r="B676" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C676" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D676" s="9" t="n">
+        <v>929</v>
+      </c>
+      <c r="E676" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F676" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G676" s="10" t="inlineStr">
+        <is>
+          <t>125248</t>
+        </is>
+      </c>
+      <c r="H676" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I676" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="677" ht="20" customHeight="1">
+      <c r="A677" s="9" t="n">
+        <v>673</v>
+      </c>
+      <c r="B677" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C677" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D677" s="9" t="n">
+        <v>932</v>
+      </c>
+      <c r="E677" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F677" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G677" s="10" t="inlineStr">
+        <is>
+          <t>125060</t>
+        </is>
+      </c>
+      <c r="H677" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I677" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="678" ht="20" customHeight="1">
+      <c r="A678" s="9" t="n">
+        <v>674</v>
+      </c>
+      <c r="B678" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C678" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D678" s="9" t="n">
+        <v>933</v>
+      </c>
+      <c r="E678" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F678" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G678" s="10" t="inlineStr">
+        <is>
+          <t>125062</t>
+        </is>
+      </c>
+      <c r="H678" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="I678" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="679" ht="20" customHeight="1">
+      <c r="A679" s="9" t="n">
+        <v>675</v>
+      </c>
+      <c r="B679" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C679" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D679" s="9" t="n">
+        <v>934</v>
+      </c>
+      <c r="E679" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F679" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G679" s="10" t="inlineStr">
+        <is>
+          <t>124539</t>
+        </is>
+      </c>
+      <c r="H679" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I679" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="680" ht="20" customHeight="1">
+      <c r="A680" s="9" t="n">
+        <v>676</v>
+      </c>
+      <c r="B680" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C680" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D680" s="9" t="n">
+        <v>935</v>
+      </c>
+      <c r="E680" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F680" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G680" s="10" t="inlineStr">
+        <is>
+          <t>124538</t>
+        </is>
+      </c>
+      <c r="H680" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I680" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="681" ht="20" customHeight="1">
+      <c r="A681" s="9" t="n">
+        <v>677</v>
+      </c>
+      <c r="B681" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C681" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D681" s="9" t="n">
+        <v>936</v>
+      </c>
+      <c r="E681" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F681" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G681" s="10" t="inlineStr">
+        <is>
+          <t>124537</t>
+        </is>
+      </c>
+      <c r="H681" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I681" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="682" ht="20" customHeight="1">
+      <c r="A682" s="9" t="n">
+        <v>678</v>
+      </c>
+      <c r="B682" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C682" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D682" s="9" t="n">
+        <v>937</v>
+      </c>
+      <c r="E682" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="F682" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G682" s="10" t="inlineStr">
+        <is>
+          <t>124536</t>
+        </is>
+      </c>
+      <c r="H682" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I682" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="683" ht="20" customHeight="1">
+      <c r="A683" s="9" t="n">
+        <v>679</v>
+      </c>
+      <c r="B683" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C683" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D683" s="9" t="n">
+        <v>938</v>
+      </c>
+      <c r="E683" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="F683" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G683" s="10" t="inlineStr">
+        <is>
+          <t>125053</t>
+        </is>
+      </c>
+      <c r="H683" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I683" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="684" ht="20" customHeight="1">
+      <c r="A684" s="9" t="n">
+        <v>680</v>
+      </c>
+      <c r="B684" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C684" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D684" s="9" t="n">
+        <v>939</v>
+      </c>
+      <c r="E684" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="F684" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G684" s="10" t="inlineStr">
+        <is>
+          <t>125054</t>
+        </is>
+      </c>
+      <c r="H684" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I684" s="11" t="inlineStr">
+        <is>
+          <t>grade 10 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (680 BAL)</t>
+        </is>
+      </c>
+      <c r="B685" s="4" t="n"/>
+      <c r="C685" s="4" t="n"/>
+      <c r="D685" s="4" t="n"/>
+      <c r="E685" s="4" t="n"/>
+      <c r="F685" s="4" t="n"/>
+      <c r="G685" s="4" t="n"/>
+      <c r="H685" s="4">
+        <f>SUM(H5:H684)</f>
         <v/>
       </c>
-      <c r="I645" s="4" t="inlineStr">
+      <c r="I685" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -37194,7 +39494,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A645:G645"/>
+    <mergeCell ref="A685:G685"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -37207,7 +39507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -37792,35 +40092,93 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>RABU</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>811</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>42.68</v>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>859 - 916</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>858</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>40.86</v>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>917 - 939</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4">
-        <f>SUM(D5:D22)</f>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4">
+        <f>SUM(D5:D24)</f>
         <v/>
       </c>
-      <c r="E23" s="4">
-        <f>SUM(E5:E22)</f>
+      <c r="E25" s="4">
+        <f>SUM(E5:E24)</f>
         <v/>
       </c>
-      <c r="F23" s="4">
-        <f>AVERAGE(F5:F22)</f>
+      <c r="F25" s="4">
+        <f>AVERAGE(F5:F24)</f>
         <v/>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>3 - 895</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>3 - 939</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: tambah data bal 11 September 2026 (25 bal), sync Supabase Cloud, update rekap Excel dan cache v5.6
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F685"/>
+  <dimension ref="A1:F710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14194,20 +14194,520 @@
       </c>
       <c r="F684" s="5" t="n"/>
     </row>
-    <row r="685" ht="22" customHeight="1">
-      <c r="A685" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (680 BAL)</t>
-        </is>
-      </c>
-      <c r="B685" s="4" t="n"/>
-      <c r="C685" s="4" t="n"/>
-      <c r="D685" s="4" t="n"/>
-      <c r="E685" s="4">
-        <f>SUM(E5:E684)</f>
+    <row r="685" ht="20.25" customHeight="1">
+      <c r="A685" s="5" t="n">
+        <v>940</v>
+      </c>
+      <c r="B685" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C685" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D685" s="6" t="inlineStr">
+        <is>
+          <t>125295</t>
+        </is>
+      </c>
+      <c r="E685" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F685" s="5" t="n"/>
+    </row>
+    <row r="686" ht="20.25" customHeight="1">
+      <c r="A686" s="5" t="n">
+        <v>941</v>
+      </c>
+      <c r="B686" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C686" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D686" s="6" t="inlineStr">
+        <is>
+          <t>125291</t>
+        </is>
+      </c>
+      <c r="E686" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F686" s="5" t="n"/>
+    </row>
+    <row r="687" ht="20.25" customHeight="1">
+      <c r="A687" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="B687" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C687" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D687" s="6" t="inlineStr">
+        <is>
+          <t>125292</t>
+        </is>
+      </c>
+      <c r="E687" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F687" s="5" t="n"/>
+    </row>
+    <row r="688" ht="20.25" customHeight="1">
+      <c r="A688" s="5" t="n">
+        <v>943</v>
+      </c>
+      <c r="B688" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C688" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D688" s="6" t="inlineStr">
+        <is>
+          <t>125293</t>
+        </is>
+      </c>
+      <c r="E688" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F688" s="5" t="n"/>
+    </row>
+    <row r="689" ht="20.25" customHeight="1">
+      <c r="A689" s="5" t="n">
+        <v>944</v>
+      </c>
+      <c r="B689" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C689" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D689" s="6" t="inlineStr">
+        <is>
+          <t>125294</t>
+        </is>
+      </c>
+      <c r="E689" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F689" s="5" t="n"/>
+    </row>
+    <row r="690" ht="20.25" customHeight="1">
+      <c r="A690" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="B690" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C690" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D690" s="6" t="inlineStr">
+        <is>
+          <t>125581</t>
+        </is>
+      </c>
+      <c r="E690" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F690" s="5" t="n"/>
+    </row>
+    <row r="691" ht="20.25" customHeight="1">
+      <c r="A691" s="5" t="n">
+        <v>946</v>
+      </c>
+      <c r="B691" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C691" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D691" s="6" t="inlineStr">
+        <is>
+          <t>125582</t>
+        </is>
+      </c>
+      <c r="E691" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F691" s="5" t="n"/>
+    </row>
+    <row r="692" ht="20.25" customHeight="1">
+      <c r="A692" s="5" t="n">
+        <v>947</v>
+      </c>
+      <c r="B692" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C692" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D692" s="6" t="inlineStr">
+        <is>
+          <t>125479</t>
+        </is>
+      </c>
+      <c r="E692" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F692" s="5" t="n"/>
+    </row>
+    <row r="693" ht="20.25" customHeight="1">
+      <c r="A693" s="5" t="n">
+        <v>948</v>
+      </c>
+      <c r="B693" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C693" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D693" s="6" t="inlineStr">
+        <is>
+          <t>125480</t>
+        </is>
+      </c>
+      <c r="E693" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F693" s="5" t="n"/>
+    </row>
+    <row r="694" ht="20.25" customHeight="1">
+      <c r="A694" s="5" t="n">
+        <v>949</v>
+      </c>
+      <c r="B694" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C694" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D694" s="6" t="inlineStr">
+        <is>
+          <t>125481</t>
+        </is>
+      </c>
+      <c r="E694" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F694" s="5" t="n"/>
+    </row>
+    <row r="695" ht="20.25" customHeight="1">
+      <c r="A695" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="B695" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C695" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D695" s="6" t="inlineStr">
+        <is>
+          <t>125482</t>
+        </is>
+      </c>
+      <c r="E695" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F695" s="5" t="n"/>
+    </row>
+    <row r="696" ht="20.25" customHeight="1">
+      <c r="A696" s="5" t="n">
+        <v>951</v>
+      </c>
+      <c r="B696" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C696" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="D696" s="6" t="inlineStr">
+        <is>
+          <t>124544</t>
+        </is>
+      </c>
+      <c r="E696" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F696" s="5" t="n"/>
+    </row>
+    <row r="697" ht="20.25" customHeight="1">
+      <c r="A697" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="B697" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C697" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="D697" s="6" t="inlineStr">
+        <is>
+          <t>124545</t>
+        </is>
+      </c>
+      <c r="E697" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F697" s="5" t="n"/>
+    </row>
+    <row r="698" ht="20.25" customHeight="1">
+      <c r="A698" s="5" t="n">
+        <v>953</v>
+      </c>
+      <c r="B698" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C698" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D698" s="6" t="inlineStr">
+        <is>
+          <t>125334</t>
+        </is>
+      </c>
+      <c r="E698" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F698" s="5" t="n"/>
+    </row>
+    <row r="699" ht="20.25" customHeight="1">
+      <c r="A699" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="B699" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C699" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D699" s="6" t="inlineStr">
+        <is>
+          <t>125296</t>
+        </is>
+      </c>
+      <c r="E699" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F699" s="5" t="n"/>
+    </row>
+    <row r="700" ht="20.25" customHeight="1">
+      <c r="A700" s="5" t="n">
+        <v>955</v>
+      </c>
+      <c r="B700" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C700" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D700" s="6" t="inlineStr">
+        <is>
+          <t>125297</t>
+        </is>
+      </c>
+      <c r="E700" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F700" s="5" t="n"/>
+    </row>
+    <row r="701" ht="20.25" customHeight="1">
+      <c r="A701" s="5" t="n">
+        <v>956</v>
+      </c>
+      <c r="B701" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C701" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D701" s="6" t="inlineStr">
+        <is>
+          <t>124546</t>
+        </is>
+      </c>
+      <c r="E701" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F701" s="5" t="n"/>
+    </row>
+    <row r="702" ht="20.25" customHeight="1">
+      <c r="A702" s="5" t="n">
+        <v>957</v>
+      </c>
+      <c r="B702" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C702" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D702" s="6" t="inlineStr">
+        <is>
+          <t>35121</t>
+        </is>
+      </c>
+      <c r="E702" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F702" s="5" t="n"/>
+    </row>
+    <row r="703" ht="20.25" customHeight="1">
+      <c r="A703" s="5" t="n">
+        <v>958</v>
+      </c>
+      <c r="B703" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C703" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D703" s="6" t="inlineStr">
+        <is>
+          <t>35120</t>
+        </is>
+      </c>
+      <c r="E703" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F703" s="5" t="n"/>
+    </row>
+    <row r="704" ht="20.25" customHeight="1">
+      <c r="A704" s="5" t="n">
+        <v>959</v>
+      </c>
+      <c r="B704" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C704" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D704" s="6" t="inlineStr">
+        <is>
+          <t>124547</t>
+        </is>
+      </c>
+      <c r="E704" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F704" s="5" t="n"/>
+    </row>
+    <row r="705" ht="20.25" customHeight="1">
+      <c r="A705" s="5" t="n">
+        <v>960</v>
+      </c>
+      <c r="B705" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C705" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D705" s="6" t="inlineStr">
+        <is>
+          <t>35119</t>
+        </is>
+      </c>
+      <c r="E705" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F705" s="5" t="n"/>
+    </row>
+    <row r="706" ht="20.25" customHeight="1">
+      <c r="A706" s="5" t="n">
+        <v>961</v>
+      </c>
+      <c r="B706" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C706" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D706" s="6" t="inlineStr">
+        <is>
+          <t>125475</t>
+        </is>
+      </c>
+      <c r="E706" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="F706" s="5" t="n"/>
+    </row>
+    <row r="707" ht="20.25" customHeight="1">
+      <c r="A707" s="5" t="n">
+        <v>962</v>
+      </c>
+      <c r="B707" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C707" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D707" s="6" t="inlineStr">
+        <is>
+          <t>125478</t>
+        </is>
+      </c>
+      <c r="E707" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F707" s="5" t="n"/>
+    </row>
+    <row r="708" ht="20.25" customHeight="1">
+      <c r="A708" s="5" t="n">
+        <v>963</v>
+      </c>
+      <c r="B708" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C708" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D708" s="6" t="inlineStr">
+        <is>
+          <t>125476</t>
+        </is>
+      </c>
+      <c r="E708" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F708" s="5" t="n"/>
+    </row>
+    <row r="709" ht="20.25" customHeight="1">
+      <c r="A709" s="5" t="n">
+        <v>964</v>
+      </c>
+      <c r="B709" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C709" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="D709" s="6" t="inlineStr">
+        <is>
+          <t>125477</t>
+        </is>
+      </c>
+      <c r="E709" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F709" s="5" t="n"/>
+    </row>
+    <row r="710" ht="22" customHeight="1">
+      <c r="A710" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (705 BAL)</t>
+        </is>
+      </c>
+      <c r="B710" s="4" t="n"/>
+      <c r="C710" s="4" t="n"/>
+      <c r="D710" s="4" t="n"/>
+      <c r="E710" s="4">
+        <f>SUM(E5:E709)</f>
         <v/>
       </c>
-      <c r="F685" s="4" t="inlineStr">
+      <c r="F710" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -14219,7 +14719,7 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A685:D685"/>
+    <mergeCell ref="A710:D710"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -14234,7 +14734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I685"/>
+  <dimension ref="A1:I710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14258,7 +14758,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 680 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 705 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -39469,23 +39969,948 @@
         </is>
       </c>
     </row>
-    <row r="685">
-      <c r="A685" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (680 BAL)</t>
-        </is>
-      </c>
-      <c r="B685" s="4" t="n"/>
-      <c r="C685" s="4" t="n"/>
-      <c r="D685" s="4" t="n"/>
-      <c r="E685" s="4" t="n"/>
-      <c r="F685" s="4" t="n"/>
-      <c r="G685" s="4" t="n"/>
-      <c r="H685" s="4">
-        <f>SUM(H5:H684)</f>
+    <row r="685" ht="20" customHeight="1">
+      <c r="A685" s="9" t="n">
+        <v>681</v>
+      </c>
+      <c r="B685" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C685" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D685" s="9" t="n">
+        <v>940</v>
+      </c>
+      <c r="E685" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F685" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G685" s="10" t="inlineStr">
+        <is>
+          <t>125295</t>
+        </is>
+      </c>
+      <c r="H685" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I685" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="686" ht="20" customHeight="1">
+      <c r="A686" s="9" t="n">
+        <v>682</v>
+      </c>
+      <c r="B686" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C686" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D686" s="9" t="n">
+        <v>941</v>
+      </c>
+      <c r="E686" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F686" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G686" s="10" t="inlineStr">
+        <is>
+          <t>125291</t>
+        </is>
+      </c>
+      <c r="H686" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I686" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="687" ht="20" customHeight="1">
+      <c r="A687" s="9" t="n">
+        <v>683</v>
+      </c>
+      <c r="B687" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C687" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D687" s="9" t="n">
+        <v>942</v>
+      </c>
+      <c r="E687" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F687" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G687" s="10" t="inlineStr">
+        <is>
+          <t>125292</t>
+        </is>
+      </c>
+      <c r="H687" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I687" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="688" ht="20" customHeight="1">
+      <c r="A688" s="9" t="n">
+        <v>684</v>
+      </c>
+      <c r="B688" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C688" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D688" s="9" t="n">
+        <v>943</v>
+      </c>
+      <c r="E688" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F688" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G688" s="10" t="inlineStr">
+        <is>
+          <t>125293</t>
+        </is>
+      </c>
+      <c r="H688" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I688" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="689" ht="20" customHeight="1">
+      <c r="A689" s="9" t="n">
+        <v>685</v>
+      </c>
+      <c r="B689" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C689" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D689" s="9" t="n">
+        <v>944</v>
+      </c>
+      <c r="E689" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F689" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G689" s="10" t="inlineStr">
+        <is>
+          <t>125294</t>
+        </is>
+      </c>
+      <c r="H689" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I689" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="690" ht="20" customHeight="1">
+      <c r="A690" s="9" t="n">
+        <v>686</v>
+      </c>
+      <c r="B690" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C690" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D690" s="9" t="n">
+        <v>945</v>
+      </c>
+      <c r="E690" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F690" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G690" s="10" t="inlineStr">
+        <is>
+          <t>125581</t>
+        </is>
+      </c>
+      <c r="H690" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I690" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="691" ht="20" customHeight="1">
+      <c r="A691" s="9" t="n">
+        <v>687</v>
+      </c>
+      <c r="B691" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C691" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D691" s="9" t="n">
+        <v>946</v>
+      </c>
+      <c r="E691" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F691" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G691" s="10" t="inlineStr">
+        <is>
+          <t>125582</t>
+        </is>
+      </c>
+      <c r="H691" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I691" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="692" ht="20" customHeight="1">
+      <c r="A692" s="9" t="n">
+        <v>688</v>
+      </c>
+      <c r="B692" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C692" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D692" s="9" t="n">
+        <v>947</v>
+      </c>
+      <c r="E692" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F692" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G692" s="10" t="inlineStr">
+        <is>
+          <t>125479</t>
+        </is>
+      </c>
+      <c r="H692" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I692" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="693" ht="20" customHeight="1">
+      <c r="A693" s="9" t="n">
+        <v>689</v>
+      </c>
+      <c r="B693" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C693" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D693" s="9" t="n">
+        <v>948</v>
+      </c>
+      <c r="E693" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F693" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G693" s="10" t="inlineStr">
+        <is>
+          <t>125480</t>
+        </is>
+      </c>
+      <c r="H693" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I693" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="694" ht="20" customHeight="1">
+      <c r="A694" s="9" t="n">
+        <v>690</v>
+      </c>
+      <c r="B694" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C694" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D694" s="9" t="n">
+        <v>949</v>
+      </c>
+      <c r="E694" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F694" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G694" s="10" t="inlineStr">
+        <is>
+          <t>125481</t>
+        </is>
+      </c>
+      <c r="H694" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I694" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="695" ht="20" customHeight="1">
+      <c r="A695" s="9" t="n">
+        <v>691</v>
+      </c>
+      <c r="B695" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C695" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D695" s="9" t="n">
+        <v>950</v>
+      </c>
+      <c r="E695" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F695" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G695" s="10" t="inlineStr">
+        <is>
+          <t>125482</t>
+        </is>
+      </c>
+      <c r="H695" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I695" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="696" ht="20" customHeight="1">
+      <c r="A696" s="9" t="n">
+        <v>692</v>
+      </c>
+      <c r="B696" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C696" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D696" s="9" t="n">
+        <v>951</v>
+      </c>
+      <c r="E696" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="F696" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="G696" s="10" t="inlineStr">
+        <is>
+          <t>124544</t>
+        </is>
+      </c>
+      <c r="H696" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I696" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="697" ht="20" customHeight="1">
+      <c r="A697" s="9" t="n">
+        <v>693</v>
+      </c>
+      <c r="B697" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C697" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D697" s="9" t="n">
+        <v>952</v>
+      </c>
+      <c r="E697" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="F697" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="G697" s="10" t="inlineStr">
+        <is>
+          <t>124545</t>
+        </is>
+      </c>
+      <c r="H697" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I697" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="698" ht="20" customHeight="1">
+      <c r="A698" s="9" t="n">
+        <v>694</v>
+      </c>
+      <c r="B698" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C698" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D698" s="9" t="n">
+        <v>953</v>
+      </c>
+      <c r="E698" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F698" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G698" s="10" t="inlineStr">
+        <is>
+          <t>125334</t>
+        </is>
+      </c>
+      <c r="H698" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I698" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="699" ht="20" customHeight="1">
+      <c r="A699" s="9" t="n">
+        <v>695</v>
+      </c>
+      <c r="B699" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C699" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D699" s="9" t="n">
+        <v>954</v>
+      </c>
+      <c r="E699" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F699" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G699" s="10" t="inlineStr">
+        <is>
+          <t>125296</t>
+        </is>
+      </c>
+      <c r="H699" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I699" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="700" ht="20" customHeight="1">
+      <c r="A700" s="9" t="n">
+        <v>696</v>
+      </c>
+      <c r="B700" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C700" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D700" s="9" t="n">
+        <v>955</v>
+      </c>
+      <c r="E700" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F700" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G700" s="10" t="inlineStr">
+        <is>
+          <t>125297</t>
+        </is>
+      </c>
+      <c r="H700" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I700" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="701" ht="20" customHeight="1">
+      <c r="A701" s="9" t="n">
+        <v>697</v>
+      </c>
+      <c r="B701" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C701" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D701" s="9" t="n">
+        <v>956</v>
+      </c>
+      <c r="E701" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F701" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G701" s="10" t="inlineStr">
+        <is>
+          <t>124546</t>
+        </is>
+      </c>
+      <c r="H701" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I701" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="702" ht="20" customHeight="1">
+      <c r="A702" s="9" t="n">
+        <v>698</v>
+      </c>
+      <c r="B702" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C702" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D702" s="9" t="n">
+        <v>957</v>
+      </c>
+      <c r="E702" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F702" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="G702" s="10" t="inlineStr">
+        <is>
+          <t>35121</t>
+        </is>
+      </c>
+      <c r="H702" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I702" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="703" ht="20" customHeight="1">
+      <c r="A703" s="9" t="n">
+        <v>699</v>
+      </c>
+      <c r="B703" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C703" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D703" s="9" t="n">
+        <v>958</v>
+      </c>
+      <c r="E703" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F703" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G703" s="10" t="inlineStr">
+        <is>
+          <t>35120</t>
+        </is>
+      </c>
+      <c r="H703" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I703" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="704" ht="20" customHeight="1">
+      <c r="A704" s="9" t="n">
+        <v>700</v>
+      </c>
+      <c r="B704" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C704" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D704" s="9" t="n">
+        <v>959</v>
+      </c>
+      <c r="E704" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F704" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G704" s="10" t="inlineStr">
+        <is>
+          <t>124547</t>
+        </is>
+      </c>
+      <c r="H704" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I704" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="705" ht="20" customHeight="1">
+      <c r="A705" s="9" t="n">
+        <v>701</v>
+      </c>
+      <c r="B705" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C705" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D705" s="9" t="n">
+        <v>960</v>
+      </c>
+      <c r="E705" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F705" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G705" s="10" t="inlineStr">
+        <is>
+          <t>35119</t>
+        </is>
+      </c>
+      <c r="H705" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I705" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="706" ht="20" customHeight="1">
+      <c r="A706" s="9" t="n">
+        <v>702</v>
+      </c>
+      <c r="B706" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C706" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D706" s="9" t="n">
+        <v>961</v>
+      </c>
+      <c r="E706" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F706" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G706" s="10" t="inlineStr">
+        <is>
+          <t>125475</t>
+        </is>
+      </c>
+      <c r="H706" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="I706" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="707" ht="20" customHeight="1">
+      <c r="A707" s="9" t="n">
+        <v>703</v>
+      </c>
+      <c r="B707" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C707" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D707" s="9" t="n">
+        <v>962</v>
+      </c>
+      <c r="E707" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F707" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G707" s="10" t="inlineStr">
+        <is>
+          <t>125478</t>
+        </is>
+      </c>
+      <c r="H707" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I707" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="708" ht="20" customHeight="1">
+      <c r="A708" s="9" t="n">
+        <v>704</v>
+      </c>
+      <c r="B708" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C708" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D708" s="9" t="n">
+        <v>963</v>
+      </c>
+      <c r="E708" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F708" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G708" s="10" t="inlineStr">
+        <is>
+          <t>125476</t>
+        </is>
+      </c>
+      <c r="H708" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="I708" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="709" ht="20" customHeight="1">
+      <c r="A709" s="9" t="n">
+        <v>705</v>
+      </c>
+      <c r="B709" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C709" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D709" s="9" t="n">
+        <v>964</v>
+      </c>
+      <c r="E709" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F709" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G709" s="10" t="inlineStr">
+        <is>
+          <t>125477</t>
+        </is>
+      </c>
+      <c r="H709" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I709" s="11" t="inlineStr">
+        <is>
+          <t>grade 11 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (705 BAL)</t>
+        </is>
+      </c>
+      <c r="B710" s="4" t="n"/>
+      <c r="C710" s="4" t="n"/>
+      <c r="D710" s="4" t="n"/>
+      <c r="E710" s="4" t="n"/>
+      <c r="F710" s="4" t="n"/>
+      <c r="G710" s="4" t="n"/>
+      <c r="H710" s="4">
+        <f>SUM(H5:H709)</f>
         <v/>
       </c>
-      <c r="I685" s="4" t="inlineStr">
+      <c r="I710" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -39494,7 +40919,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A685:G685"/>
+    <mergeCell ref="A710:G710"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39507,7 +40932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -40150,35 +41575,64 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>JUMAT</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>1032</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>41.28</v>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>940 - 964</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4">
-        <f>SUM(D5:D24)</f>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4">
+        <f>SUM(D5:D25)</f>
         <v/>
       </c>
-      <c r="E25" s="4">
-        <f>SUM(E5:E24)</f>
+      <c r="E26" s="4">
+        <f>SUM(E5:E25)</f>
         <v/>
       </c>
-      <c r="F25" s="4">
-        <f>AVERAGE(F5:F24)</f>
+      <c r="F26" s="4">
+        <f>AVERAGE(F5:F25)</f>
         <v/>
       </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>3 - 939</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>3 - 964</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: tambah data bal 12 September 2026 (20 bal), sync Supabase Cloud, update rekap Excel dan cache v5.7
</commit_message>
<xml_diff>
--- a/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
+++ b/Laporan Grade Induk/buku_grade_induk_rekap_barkot_tgl_21_sd_31.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F710"/>
+  <dimension ref="A1:F729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14694,20 +14694,400 @@
       </c>
       <c r="F709" s="5" t="n"/>
     </row>
-    <row r="710" ht="22" customHeight="1">
-      <c r="A710" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (705 BAL)</t>
-        </is>
-      </c>
-      <c r="B710" s="4" t="n"/>
-      <c r="C710" s="4" t="n"/>
-      <c r="D710" s="4" t="n"/>
-      <c r="E710" s="4">
-        <f>SUM(E5:E709)</f>
+    <row r="710" ht="20.25" customHeight="1">
+      <c r="A710" s="5" t="n">
+        <v>968</v>
+      </c>
+      <c r="B710" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C710" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D710" s="6" t="inlineStr">
+        <is>
+          <t>280139</t>
+        </is>
+      </c>
+      <c r="E710" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="F710" s="5" t="n"/>
+    </row>
+    <row r="711" ht="20.25" customHeight="1">
+      <c r="A711" s="5" t="n">
+        <v>969</v>
+      </c>
+      <c r="B711" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C711" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D711" s="6" t="inlineStr">
+        <is>
+          <t>280140</t>
+        </is>
+      </c>
+      <c r="E711" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F711" s="5" t="n"/>
+    </row>
+    <row r="712" ht="20.25" customHeight="1">
+      <c r="A712" s="5" t="n">
+        <v>970</v>
+      </c>
+      <c r="B712" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C712" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D712" s="6" t="inlineStr">
+        <is>
+          <t>280141</t>
+        </is>
+      </c>
+      <c r="E712" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F712" s="5" t="n"/>
+    </row>
+    <row r="713" ht="20.25" customHeight="1">
+      <c r="A713" s="5" t="n">
+        <v>971</v>
+      </c>
+      <c r="B713" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C713" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D713" s="6" t="inlineStr">
+        <is>
+          <t>125987</t>
+        </is>
+      </c>
+      <c r="E713" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F713" s="5" t="n"/>
+    </row>
+    <row r="714" ht="20.25" customHeight="1">
+      <c r="A714" s="5" t="n">
+        <v>972</v>
+      </c>
+      <c r="B714" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C714" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D714" s="6" t="inlineStr">
+        <is>
+          <t>39841</t>
+        </is>
+      </c>
+      <c r="E714" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="F714" s="5" t="n"/>
+    </row>
+    <row r="715" ht="20.25" customHeight="1">
+      <c r="A715" s="5" t="n">
+        <v>973</v>
+      </c>
+      <c r="B715" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C715" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D715" s="6" t="inlineStr">
+        <is>
+          <t>39842</t>
+        </is>
+      </c>
+      <c r="E715" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F715" s="5" t="n"/>
+    </row>
+    <row r="716" ht="20.25" customHeight="1">
+      <c r="A716" s="5" t="n">
+        <v>975</v>
+      </c>
+      <c r="B716" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C716" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D716" s="6" t="inlineStr">
+        <is>
+          <t>280145</t>
+        </is>
+      </c>
+      <c r="E716" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F716" s="5" t="n"/>
+    </row>
+    <row r="717" ht="20.25" customHeight="1">
+      <c r="A717" s="5" t="n">
+        <v>976</v>
+      </c>
+      <c r="B717" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C717" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D717" s="6" t="inlineStr">
+        <is>
+          <t>280146</t>
+        </is>
+      </c>
+      <c r="E717" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F717" s="5" t="n"/>
+    </row>
+    <row r="718" ht="20.25" customHeight="1">
+      <c r="A718" s="5" t="n">
+        <v>977</v>
+      </c>
+      <c r="B718" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C718" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D718" s="6" t="inlineStr">
+        <is>
+          <t>280144</t>
+        </is>
+      </c>
+      <c r="E718" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F718" s="5" t="n"/>
+    </row>
+    <row r="719" ht="20.25" customHeight="1">
+      <c r="A719" s="5" t="n">
+        <v>978</v>
+      </c>
+      <c r="B719" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C719" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D719" s="6" t="inlineStr">
+        <is>
+          <t>125822</t>
+        </is>
+      </c>
+      <c r="E719" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F719" s="5" t="n"/>
+    </row>
+    <row r="720" ht="20.25" customHeight="1">
+      <c r="A720" s="5" t="n">
+        <v>979</v>
+      </c>
+      <c r="B720" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="C720" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D720" s="6" t="inlineStr">
+        <is>
+          <t>125821</t>
+        </is>
+      </c>
+      <c r="E720" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F720" s="5" t="n"/>
+    </row>
+    <row r="721" ht="20.25" customHeight="1">
+      <c r="A721" s="5" t="n">
+        <v>980</v>
+      </c>
+      <c r="B721" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C721" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D721" s="6" t="inlineStr">
+        <is>
+          <t>280302</t>
+        </is>
+      </c>
+      <c r="E721" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F721" s="5" t="n"/>
+    </row>
+    <row r="722" ht="20.25" customHeight="1">
+      <c r="A722" s="5" t="n">
+        <v>981</v>
+      </c>
+      <c r="B722" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C722" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D722" s="6" t="inlineStr">
+        <is>
+          <t>125991</t>
+        </is>
+      </c>
+      <c r="E722" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F722" s="5" t="n"/>
+    </row>
+    <row r="723" ht="20.25" customHeight="1">
+      <c r="A723" s="5" t="n">
+        <v>982</v>
+      </c>
+      <c r="B723" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C723" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D723" s="6" t="inlineStr">
+        <is>
+          <t>125990</t>
+        </is>
+      </c>
+      <c r="E723" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F723" s="5" t="n"/>
+    </row>
+    <row r="724" ht="20.25" customHeight="1">
+      <c r="A724" s="5" t="n">
+        <v>983</v>
+      </c>
+      <c r="B724" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C724" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D724" s="6" t="inlineStr">
+        <is>
+          <t>125992</t>
+        </is>
+      </c>
+      <c r="E724" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F724" s="5" t="n"/>
+    </row>
+    <row r="725" ht="20.25" customHeight="1">
+      <c r="A725" s="5" t="n">
+        <v>984</v>
+      </c>
+      <c r="B725" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C725" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D725" s="6" t="inlineStr">
+        <is>
+          <t>125988</t>
+        </is>
+      </c>
+      <c r="E725" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F725" s="5" t="n"/>
+    </row>
+    <row r="726" ht="20.25" customHeight="1">
+      <c r="A726" s="5" t="n">
+        <v>985</v>
+      </c>
+      <c r="B726" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C726" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D726" s="6" t="inlineStr">
+        <is>
+          <t>280143</t>
+        </is>
+      </c>
+      <c r="E726" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F726" s="5" t="n"/>
+    </row>
+    <row r="727" ht="20.25" customHeight="1">
+      <c r="A727" s="5" t="n">
+        <v>986</v>
+      </c>
+      <c r="B727" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C727" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D727" s="6" t="inlineStr">
+        <is>
+          <t>125989</t>
+        </is>
+      </c>
+      <c r="E727" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="F727" s="5" t="n"/>
+    </row>
+    <row r="728" ht="20.25" customHeight="1">
+      <c r="A728" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="B728" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="C728" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D728" s="6" t="inlineStr">
+        <is>
+          <t>280142</t>
+        </is>
+      </c>
+      <c r="E728" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F728" s="5" t="n"/>
+    </row>
+    <row r="729" ht="22" customHeight="1">
+      <c r="A729" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (724 BAL)</t>
+        </is>
+      </c>
+      <c r="B729" s="4" t="n"/>
+      <c r="C729" s="4" t="n"/>
+      <c r="D729" s="4" t="n"/>
+      <c r="E729" s="4">
+        <f>SUM(E5:E728)</f>
         <v/>
       </c>
-      <c r="F710" s="4" t="inlineStr">
+      <c r="F729" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -14716,10 +15096,10 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A729:D729"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A710:D710"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B3:C4"/>
@@ -14734,7 +15114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I710"/>
+  <dimension ref="A1:I729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14758,7 +15138,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 705 Bal Berbarkot</t>
+          <t>Diurutkan berdasarkan No Gudang terkecil sampai terbesar | Total: 724 Bal Berbarkot</t>
         </is>
       </c>
     </row>
@@ -40894,23 +41274,726 @@
         </is>
       </c>
     </row>
-    <row r="710">
-      <c r="A710" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL (705 BAL)</t>
-        </is>
-      </c>
-      <c r="B710" s="4" t="n"/>
-      <c r="C710" s="4" t="n"/>
-      <c r="D710" s="4" t="n"/>
-      <c r="E710" s="4" t="n"/>
-      <c r="F710" s="4" t="n"/>
-      <c r="G710" s="4" t="n"/>
-      <c r="H710" s="4">
-        <f>SUM(H5:H709)</f>
+    <row r="710" ht="20" customHeight="1">
+      <c r="A710" s="9" t="n">
+        <v>706</v>
+      </c>
+      <c r="B710" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C710" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D710" s="9" t="n">
+        <v>968</v>
+      </c>
+      <c r="E710" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="F710" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G710" s="10" t="inlineStr">
+        <is>
+          <t>280139</t>
+        </is>
+      </c>
+      <c r="H710" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="I710" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="711" ht="20" customHeight="1">
+      <c r="A711" s="9" t="n">
+        <v>707</v>
+      </c>
+      <c r="B711" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C711" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D711" s="9" t="n">
+        <v>969</v>
+      </c>
+      <c r="E711" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F711" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G711" s="10" t="inlineStr">
+        <is>
+          <t>280140</t>
+        </is>
+      </c>
+      <c r="H711" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I711" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="712" ht="20" customHeight="1">
+      <c r="A712" s="9" t="n">
+        <v>708</v>
+      </c>
+      <c r="B712" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C712" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D712" s="9" t="n">
+        <v>970</v>
+      </c>
+      <c r="E712" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F712" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="G712" s="10" t="inlineStr">
+        <is>
+          <t>280141</t>
+        </is>
+      </c>
+      <c r="H712" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I712" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="713" ht="20" customHeight="1">
+      <c r="A713" s="9" t="n">
+        <v>709</v>
+      </c>
+      <c r="B713" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C713" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D713" s="9" t="n">
+        <v>971</v>
+      </c>
+      <c r="E713" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F713" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G713" s="10" t="inlineStr">
+        <is>
+          <t>125987</t>
+        </is>
+      </c>
+      <c r="H713" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I713" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="714" ht="20" customHeight="1">
+      <c r="A714" s="9" t="n">
+        <v>710</v>
+      </c>
+      <c r="B714" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C714" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D714" s="9" t="n">
+        <v>972</v>
+      </c>
+      <c r="E714" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F714" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G714" s="10" t="inlineStr">
+        <is>
+          <t>39841</t>
+        </is>
+      </c>
+      <c r="H714" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="I714" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="715" ht="20" customHeight="1">
+      <c r="A715" s="9" t="n">
+        <v>711</v>
+      </c>
+      <c r="B715" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C715" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D715" s="9" t="n">
+        <v>973</v>
+      </c>
+      <c r="E715" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="F715" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G715" s="10" t="inlineStr">
+        <is>
+          <t>39842</t>
+        </is>
+      </c>
+      <c r="H715" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="I715" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="716" ht="20" customHeight="1">
+      <c r="A716" s="9" t="n">
+        <v>712</v>
+      </c>
+      <c r="B716" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C716" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D716" s="9" t="n">
+        <v>975</v>
+      </c>
+      <c r="E716" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F716" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G716" s="10" t="inlineStr">
+        <is>
+          <t>280145</t>
+        </is>
+      </c>
+      <c r="H716" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I716" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="717" ht="20" customHeight="1">
+      <c r="A717" s="9" t="n">
+        <v>713</v>
+      </c>
+      <c r="B717" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C717" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D717" s="9" t="n">
+        <v>976</v>
+      </c>
+      <c r="E717" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F717" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G717" s="10" t="inlineStr">
+        <is>
+          <t>280146</t>
+        </is>
+      </c>
+      <c r="H717" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I717" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="718" ht="20" customHeight="1">
+      <c r="A718" s="9" t="n">
+        <v>714</v>
+      </c>
+      <c r="B718" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C718" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D718" s="9" t="n">
+        <v>977</v>
+      </c>
+      <c r="E718" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F718" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G718" s="10" t="inlineStr">
+        <is>
+          <t>280144</t>
+        </is>
+      </c>
+      <c r="H718" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I718" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="719" ht="20" customHeight="1">
+      <c r="A719" s="9" t="n">
+        <v>715</v>
+      </c>
+      <c r="B719" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C719" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D719" s="9" t="n">
+        <v>978</v>
+      </c>
+      <c r="E719" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F719" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G719" s="10" t="inlineStr">
+        <is>
+          <t>125822</t>
+        </is>
+      </c>
+      <c r="H719" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I719" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="720" ht="20" customHeight="1">
+      <c r="A720" s="9" t="n">
+        <v>716</v>
+      </c>
+      <c r="B720" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C720" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D720" s="9" t="n">
+        <v>979</v>
+      </c>
+      <c r="E720" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="F720" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G720" s="10" t="inlineStr">
+        <is>
+          <t>125821</t>
+        </is>
+      </c>
+      <c r="H720" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I720" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="721" ht="20" customHeight="1">
+      <c r="A721" s="9" t="n">
+        <v>717</v>
+      </c>
+      <c r="B721" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C721" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D721" s="9" t="n">
+        <v>980</v>
+      </c>
+      <c r="E721" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F721" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G721" s="10" t="inlineStr">
+        <is>
+          <t>280302</t>
+        </is>
+      </c>
+      <c r="H721" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="I721" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="722" ht="20" customHeight="1">
+      <c r="A722" s="9" t="n">
+        <v>718</v>
+      </c>
+      <c r="B722" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C722" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D722" s="9" t="n">
+        <v>981</v>
+      </c>
+      <c r="E722" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F722" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G722" s="10" t="inlineStr">
+        <is>
+          <t>125991</t>
+        </is>
+      </c>
+      <c r="H722" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I722" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="723" ht="20" customHeight="1">
+      <c r="A723" s="9" t="n">
+        <v>719</v>
+      </c>
+      <c r="B723" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C723" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D723" s="9" t="n">
+        <v>982</v>
+      </c>
+      <c r="E723" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F723" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G723" s="10" t="inlineStr">
+        <is>
+          <t>125990</t>
+        </is>
+      </c>
+      <c r="H723" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I723" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="724" ht="20" customHeight="1">
+      <c r="A724" s="9" t="n">
+        <v>720</v>
+      </c>
+      <c r="B724" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C724" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D724" s="9" t="n">
+        <v>983</v>
+      </c>
+      <c r="E724" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="F724" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G724" s="10" t="inlineStr">
+        <is>
+          <t>125992</t>
+        </is>
+      </c>
+      <c r="H724" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I724" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="725" ht="20" customHeight="1">
+      <c r="A725" s="9" t="n">
+        <v>721</v>
+      </c>
+      <c r="B725" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C725" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D725" s="9" t="n">
+        <v>984</v>
+      </c>
+      <c r="E725" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F725" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G725" s="10" t="inlineStr">
+        <is>
+          <t>125988</t>
+        </is>
+      </c>
+      <c r="H725" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I725" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="726" ht="20" customHeight="1">
+      <c r="A726" s="9" t="n">
+        <v>722</v>
+      </c>
+      <c r="B726" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C726" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D726" s="9" t="n">
+        <v>985</v>
+      </c>
+      <c r="E726" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="F726" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G726" s="10" t="inlineStr">
+        <is>
+          <t>280143</t>
+        </is>
+      </c>
+      <c r="H726" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I726" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="727" ht="20" customHeight="1">
+      <c r="A727" s="9" t="n">
+        <v>723</v>
+      </c>
+      <c r="B727" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C727" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D727" s="9" t="n">
+        <v>986</v>
+      </c>
+      <c r="E727" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F727" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="G727" s="10" t="inlineStr">
+        <is>
+          <t>125989</t>
+        </is>
+      </c>
+      <c r="H727" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="I727" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="728" ht="20" customHeight="1">
+      <c r="A728" s="9" t="n">
+        <v>724</v>
+      </c>
+      <c r="B728" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C728" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D728" s="9" t="n">
+        <v>987</v>
+      </c>
+      <c r="E728" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="F728" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G728" s="10" t="inlineStr">
+        <is>
+          <t>280142</t>
+        </is>
+      </c>
+      <c r="H728" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I728" s="11" t="inlineStr">
+        <is>
+          <t>grade 12 sep.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL (724 BAL)</t>
+        </is>
+      </c>
+      <c r="B729" s="4" t="n"/>
+      <c r="C729" s="4" t="n"/>
+      <c r="D729" s="4" t="n"/>
+      <c r="E729" s="4" t="n"/>
+      <c r="F729" s="4" t="n"/>
+      <c r="G729" s="4" t="n"/>
+      <c r="H729" s="4">
+        <f>SUM(H5:H728)</f>
         <v/>
       </c>
-      <c r="I710" s="4" t="inlineStr">
+      <c r="I729" s="4" t="inlineStr">
         <is>
           <t>KG</t>
         </is>
@@ -40919,7 +42002,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A710:G710"/>
+    <mergeCell ref="A729:G729"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -40932,7 +42015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -41604,35 +42687,64 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>SABTU</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>741</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>968 - 987</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4">
-        <f>SUM(D5:D25)</f>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4">
+        <f>SUM(D5:D26)</f>
         <v/>
       </c>
-      <c r="E26" s="4">
-        <f>SUM(E5:E25)</f>
+      <c r="E27" s="4">
+        <f>SUM(E5:E26)</f>
         <v/>
       </c>
-      <c r="F26" s="4">
-        <f>AVERAGE(F5:F25)</f>
+      <c r="F27" s="4">
+        <f>AVERAGE(F5:F26)</f>
         <v/>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>3 - 964</t>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>3 - 987</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>